<commit_message>
Training sheet v3: CVD-validated KRA color families on both outputs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,18 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -55,11 +65,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
+        <fgColor rgb="00F2F7FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF6F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1FAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFEBF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF3EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF1D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCEBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -69,37 +129,278 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00C8C8C8"/>
       </left>
       <right style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00C8C8C8"/>
       </right>
       <top style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00C8C8C8"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C8C8C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="002A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="002A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C8C8C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C8C8C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C8C8C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C8C8C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00E87BA4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00E87BA4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C8C8C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -566,37 +867,37 @@
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="5" t="n"/>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Module-Quiz Score Bands</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>classroom-quiz attempts &amp; performance · practice completion % · module-quiz participation 100% (SPI eligibility)</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>≥8.0: 30% · 7.0–8.0: 40% · 5.0–7.0: 30% · &lt;5.0: ~0% (quiz 10-pt scale, one band stricter than org)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>quiz conducted → attempted → scores band 30/40/30 → the authored 15% lands → SPI Bands</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Learning Domains</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Content (SMEs) + Pedagogy + DA/DE</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
@@ -604,37 +905,37 @@
     </row>
     <row r="4" ht="150" customHeight="1">
       <c r="A4" s="5" t="n"/>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Content–Assessment Alignment</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>assessment blueprints visible · ≥3-month change notice honored · content coverage of the blueprint</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>|delta| ≤10pp, ≤5pp after 3 clean cycles</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>blueprints visible → content teaches what's tested → quiz scores ≈ assessment scores → the 75% lands → SPI Bands</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Learning Domains</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Content (SMEs) + Pedagogy + DA/DE</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
@@ -642,37 +943,37 @@
     </row>
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="5" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Engagement-Matrix Cell Migration  [SAMPLE]</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>capability adoption (tutor, revision, leaderboard, adaptive) · LE effort signals · value signals</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>HE×HV 4% → 10% or M×M 10% → 20%, per cycle (semester NIAT · quarter rolling) — SAMPLE until LE baselines</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>capabilities adopted → effort &amp; value rise → cells migrate up → scores follow → SPI Bands (leading)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Learning Platform</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Product (LP PMs) + Engineering (LP) + DA/DE</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
@@ -680,707 +981,707 @@
     </row>
     <row r="6" ht="150" customHeight="1">
       <c r="A6" s="5" t="n"/>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Summative &amp; Formative Achievement  [ORG]</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>steps above held · assessments conducted on schedule (Program Ops) · instruments authored (Assessments dept)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>same 30/40/30 on assessment scores, per batch</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>steps 1–3 held → assessments run → 30/40/30 on the 75% → SPI Bands</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>org scoreboard — tracked, not owned</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>— context</t>
         </is>
       </c>
     </row>
     <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>KRA 2 — Academics CSAT
 4.5 / 5
 (content quality, fast visible fixes, issues that never repeat)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>issue intake &amp; triage · fix TAT 48 h · student notified</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>≥80% within the fixed 2-day TAT</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>issue reported → fixed in 48 h → trust in content → Academics CSAT</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Agentic Content Platform</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Content (SMEs) + Engineering (ACP)</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Content Issue Recurrence</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>root-cause close — 4-checkbox: instance fixed · artifact changed · tripwire added · broadcast sent</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>≤2% of resolved issues / quarter</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>fixed once → closed at root cause → never twice → trust → Academics CSAT</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Agentic Content Platform</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Content (SMEs) + Engineering (ACP)</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="9" ht="128.3225806451613" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Learning Environment Satisfaction</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>driven by the four rows below</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>≥4.5 / 5, monthly</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>platform reliable &amp; fast → rating ≥4.5 → Academics CSAT</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Developer Platform</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Engineering (DP)</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
       </c>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Availability &amp; Saturation Detection</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>critical services (IDE, compiler, workflows) · alert thresholds · detection time</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>100% thresholds alerted · detection ≤10 min</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>saturation detected ≤10 min → fixed before students feel it → LES → Academics CSAT</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Developer Platform</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Engineering (DP)</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Tail-Latency User Impact</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>IDE launch / submit / publish P99 &lt;60 s · compiler per-language limits</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>students beyond P99 limits → 0%</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>P99 within limits → coding feels instant → LES → Academics CSAT</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Developer Platform</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Engineering (DP)</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="12" ht="117.8387096774194" customHeight="1">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Platform Issue Resolution Efficiency</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>2-day TAT (internal same-day)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>≥80% within the fixed 2-day TAT</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>platform issue → fixed fast → LES → Academics CSAT</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Developer Platform</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Engineering (DP)</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="13" ht="101.0645161290323" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Platform Issue Recurrence</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>root-cause close</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>≤2% of resolved issues / quarter</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>fixed → never twice → LES → Academics CSAT</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Developer Platform</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="13" t="inlineStr">
         <is>
           <t>Engineering (DP)</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Journey Step Health (NIAT first)</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>the 11 journey steps — attendance · class runs · classroom quiz · practice · revision · module quiz · skill assessment … (one-pager §11)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>% of steps green, per product (baseline first quarter)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>capabilities configured → 11 steps green → assembled experience works → Academics CSAT (+ SPI)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Product (PLE PM) + DA/DE + CSI team</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
       </c>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Product Issue Resolution Efficiency  [CROSS-DEPT]</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>routing to owning department · fix live · students notified (silent fixes don't count)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>first-quarter baseline sets the TAT target</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>any student issue → routed → fixed + notified → Academics CSAT</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>Product (PLE PM) + CSI team</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="16" ht="140.9032258064516" customHeight="1">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Product Issue Recurrence  [CROSS-DEPT]</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>student-journey-level recurrence watch</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>≤2% of resolved issues / quarter</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>resolved once → never twice at journey level → Academics CSAT</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Product (PLE PM) + CSI team</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>KRA 3 — University Relations CSAT
 4.5 · 4.0 · 4.0
 (BOS-compliant curriculum, delivered as approved, responsive partnership)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>BOS Credit Acceptance</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>per-credit acceptance per university · curriculum finalisation (Bharath, PK Das, Visakha pending)</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>B3 85% · B4 90%</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>credits proposed → accepted first pass → university leadership confidence → Univ Relations CSAT</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>CSI team + Content (SMEs)</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>Business Impact</t>
         </is>
       </c>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Program Delivery Gap  [CASCADE]</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>same triggers as the KRA 1 row — one KPI feeding two KRAs</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>0% deviation</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>delivered = approved plan → university trust → Univ Relations CSAT</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>CSI team + Product (PLE PM)</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="A19" s="17" t="n"/>
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>University Communication TAT</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>ack ≤1 business day · request-class TATs (standard 3 days, heavy artefacts pre-agreed) · university-request log (month 1)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>≥90% answered within TAT</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>requests answered in TAT → partnership friction drops → Univ Relations CSAT</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>CSI team</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="A20" s="17" t="n"/>
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>University Curriculum Compliance · Framework Compliance</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>delivery matches the approved BOS syllabus · NHQRF / Woolf / AICTE / UGC audits</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>compliant, every submission cycle</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>BOS &amp; frameworks kept → zero partnership risk → Univ Relations CSAT</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>Product Learning Experience</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>CSI team + Content (SMEs)</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="21" ht="150" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>KRA 4 — GRIT Novice Badges
 5,000
 (classroom learning trains to contest level)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>Industry Update Adherence (Learning–GRIT delta)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>GRIT-tested skills inventory vs live course content</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>delta → 0</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>course content covers GRIT-tested skills → students contest-ready → Novice badges</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>Learning Domains</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>Content (SMEs)</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>Quality &amp; Reliability</t>
         </is>
       </c>
     </row>
     <row r="22" ht="128.3225806451613" customHeight="1">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>GRIT-feature KPIs  [ORG]</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>ask raised to the GRIT owner (Sundar) to define</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t>pending definition</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>GRIT features drive practice → badges (mapping pending)</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="25" t="inlineStr">
         <is>
           <t>GRIT owner</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="25" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="25" t="inlineStr">
         <is>
           <t>— context</t>
         </is>
       </c>
     </row>
     <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>KRA 5 — Employability
 B3 80% · B4 80%
 (skill mastered this semester → offers next year)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>Mapping yet to be thought through</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>skill mastery is the long lever — adaptive practice, stronger question banks</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>real skill rises → placements later (mapping deliberately not forced yet)</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="28" t="inlineStr">
         <is>
           <t>— placeholder</t>
         </is>
@@ -1430,97 +1731,97 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>Product (PMs)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>Program Delivery Gap (both KRAs) · Engagement-Matrix Cell Migration · Journey Step Health · Product Issue Resolution + Recurrence</t>
         </is>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="31">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*Product (*")</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="33" t="inlineStr">
         <is>
           <t>LES + its four drivers (DP) · Content Issue pair tooling/routing (ACP) · Cell Migration build (LP)</t>
         </is>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="34">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*Engineering*")</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Content (SMEs)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Module-Quiz Score Bands · Content–Assessment Alignment · Content Issue pair (fixes) · BOS curriculum artifacts · Compliance · GRIT delta</t>
         </is>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="31">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*Content (SMEs)*")</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Pedagogy</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Module-Quiz Score Bands · Content–Assessment Alignment</t>
         </is>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="34">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*Pedagogy*")</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>DA/DE</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>score analysis (bands, alignment) · LE dashboard (cell migration) · Journey Step Health instrumentation</t>
         </is>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="31">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*DA/DE*")</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>CSI team</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>Program Delivery Gap (both KRAs) · Journey Step Health · Product Issue pair · BOS · University Communication TAT · Compliance</t>
         </is>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="34">
         <f>COUNTIF('KRA-KPI Map'!$G$2:$G$23,"*CSI team*")</f>
         <v/>
       </c>
@@ -1536,7 +1837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1544,98 +1845,170 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>How to read</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>A KRA (Key Result Area) is an org outcome NIAT is judged on — it carries the target (column A). Each KRA is served by department KPIs (column B) with their own targets (column D).</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Color coding</t>
+        </is>
+      </c>
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>Each KRA block carries its own color family — the deep band on the KRA cell, a whisper tint on its member rows. Color is a reading aid only: identity is always in the text (palette validated for color-vision deficiency).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Lane (KPI owner)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="33" t="inlineStr">
         <is>
           <t>A lane is an accountability grouping of KPIs, NOT a team — the lane lead answers for the number at review. Lanes: Learning Domains · Learning Platform · Developer Platform · Agentic Content Platform · Product Learning Experience.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>Functions that move it</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>The real teams whose day job moves the KPI — Product, Engineering, Content (SMEs), Pedagogy, DA/DE, CSI team. Training runs per function; the Session Index sheet is the room-by-room cut. THIS COLUMN IS A DRAFT — edit freely, the index counts recompute.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Triggers / sub-metrics</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>What composes or precedes the KPI — journey-wise sub-metrics for Program Delivery Gap, drivers for LES, eligibility rules for quiz metrics.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Funnel</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>The causal chain from the KPI to the org KRA it moves.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Markers</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>[ORG] org-owned scoreboard, tracked not owned · [CROSS-DEPT] resolved across departments, we route · [SAMPLE] illustrative numbers until baselines land · [CASCADE] same KPI feeds two KRAs.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Editable</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>Everything is editable. Cells most expected to change: Functions column (G, draft), SAMPLE targets (cell migration — awaiting LE-dashboard baselines), Journey Step Health baseline, conduction-adherence ground truth.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="33" t="inlineStr">
         <is>
           <t>Compiled from the HOD KPI one-pager (§6 scoreboard + mechanism trees) and the internal operating view, Curriculum &amp; Content dept, as of 2026-08-19. Targets are the accountable numbers on that date; function mapping drafted by Claude for HOD red-pen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>KRA 1 — SPI Bands</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>color key — this KRA's band and row tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>KRA 2 — Academics CSAT</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>color key — this KRA's band and row tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>KRA 3 — University Relations CSAT</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>color key — this KRA's band and row tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>KRA 4 — GRIT Novice Badges</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>color key — this KRA's band and row tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>KRA 5 — Employability</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>color key — this KRA's band and row tint</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Training sheet: Triggers/sub-metrics column renamed Dependent metrics
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -119,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -295,11 +295,143 @@
         <color rgb="00C8C8C8"/>
       </bottom>
     </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EB6834"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EDA100"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00EDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001BAF7A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="002A78D6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="002A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="002A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -401,6 +533,13 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -792,7 +931,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Triggers / sub-metrics</t>
+          <t>Dependent metrics</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -866,7 +1005,7 @@
       </c>
     </row>
     <row r="3" ht="150" customHeight="1">
-      <c r="A3" s="5" t="n"/>
+      <c r="A3" s="41" t="n"/>
       <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Module-Quiz Score Bands</t>
@@ -904,7 +1043,7 @@
       </c>
     </row>
     <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="5" t="n"/>
+      <c r="A4" s="41" t="n"/>
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Content–Assessment Alignment</t>
@@ -942,7 +1081,7 @@
       </c>
     </row>
     <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="5" t="n"/>
+      <c r="A5" s="41" t="n"/>
       <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Engagement-Matrix Cell Migration  [SAMPLE]</t>
@@ -980,7 +1119,7 @@
       </c>
     </row>
     <row r="6" ht="150" customHeight="1">
-      <c r="A6" s="5" t="n"/>
+      <c r="A6" s="42" t="n"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Summative &amp; Formative Achievement  [ORG]</t>
@@ -1062,7 +1201,7 @@
       </c>
     </row>
     <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="11" t="n"/>
+      <c r="A8" s="43" t="n"/>
       <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Content Issue Recurrence</t>
@@ -1100,7 +1239,7 @@
       </c>
     </row>
     <row r="9" ht="128.3225806451613" customHeight="1">
-      <c r="A9" s="11" t="n"/>
+      <c r="A9" s="43" t="n"/>
       <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Learning Environment Satisfaction</t>
@@ -1138,7 +1277,7 @@
       </c>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="11" t="n"/>
+      <c r="A10" s="43" t="n"/>
       <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Availability &amp; Saturation Detection</t>
@@ -1176,7 +1315,7 @@
       </c>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="11" t="n"/>
+      <c r="A11" s="43" t="n"/>
       <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Tail-Latency User Impact</t>
@@ -1214,7 +1353,7 @@
       </c>
     </row>
     <row r="12" ht="117.8387096774194" customHeight="1">
-      <c r="A12" s="11" t="n"/>
+      <c r="A12" s="43" t="n"/>
       <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Platform Issue Resolution Efficiency</t>
@@ -1252,7 +1391,7 @@
       </c>
     </row>
     <row r="13" ht="101.0645161290323" customHeight="1">
-      <c r="A13" s="11" t="n"/>
+      <c r="A13" s="43" t="n"/>
       <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Platform Issue Recurrence</t>
@@ -1290,7 +1429,7 @@
       </c>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="11" t="n"/>
+      <c r="A14" s="43" t="n"/>
       <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Journey Step Health (NIAT first)</t>
@@ -1328,7 +1467,7 @@
       </c>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="11" t="n"/>
+      <c r="A15" s="43" t="n"/>
       <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Product Issue Resolution Efficiency  [CROSS-DEPT]</t>
@@ -1366,7 +1505,7 @@
       </c>
     </row>
     <row r="16" ht="140.9032258064516" customHeight="1">
-      <c r="A16" s="11" t="n"/>
+      <c r="A16" s="44" t="n"/>
       <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Product Issue Recurrence  [CROSS-DEPT]</t>
@@ -1448,7 +1587,7 @@
       </c>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="17" t="n"/>
+      <c r="A18" s="45" t="n"/>
       <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Program Delivery Gap  [CASCADE]</t>
@@ -1486,7 +1625,7 @@
       </c>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="17" t="n"/>
+      <c r="A19" s="45" t="n"/>
       <c r="B19" s="18" t="inlineStr">
         <is>
           <t>University Communication TAT</t>
@@ -1524,7 +1663,7 @@
       </c>
     </row>
     <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="17" t="n"/>
+      <c r="A20" s="46" t="n"/>
       <c r="B20" s="18" t="inlineStr">
         <is>
           <t>University Curriculum Compliance · Framework Compliance</t>
@@ -1606,7 +1745,7 @@
       </c>
     </row>
     <row r="22" ht="128.3225806451613" customHeight="1">
-      <c r="A22" s="23" t="n"/>
+      <c r="A22" s="47" t="n"/>
       <c r="B22" s="24" t="inlineStr">
         <is>
           <t>GRIT-feature KPIs  [ORG]</t>
@@ -1895,12 +2034,12 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="32" t="inlineStr">
         <is>
-          <t>Triggers / sub-metrics</t>
+          <t>Dependent metrics</t>
         </is>
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>What composes or precedes the KPI — journey-wise sub-metrics for Program Delivery Gap, drivers for LES, eligibility rules for quiz metrics.</t>
+          <t>The trigger metrics that compose or precede the KPI — journey-wise dependent metrics for Program Delivery Gap, drivers for LES, eligibility rule</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
KPI Tracker FY26-27: workbook tab 4 + artifact §3, B3/B4 cohort rows
Org Head-Abstract format with one annual Budgeted/Actual/Variance set;
27 numbered rows (bands as 4 rows per batch, per-batch rows split B3/B4);
variance = Budgeted − Actual as live formula; builder + data source committed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRA-KPI Map" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Index" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker FY26-27" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +53,31 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF1A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF777777"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -118,8 +142,63 @@
         <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F7FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF6F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1FAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF9F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDFEBF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDF3EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCF1D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCEBF1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="59">
     <border>
       <left/>
       <right/>
@@ -427,11 +506,418 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF2A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF2A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF1BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF1BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFE87BA4"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEDA100"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEDA100"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF2A78D6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF2A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF2A78D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF1BAF7A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF1BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF1BAF7A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEB6834"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFEB6834"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -540,6 +1026,160 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1976,7 +2616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2091,6 +2731,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
@@ -2148,10 +2789,1670 @@
       <c r="B15" s="36" t="inlineStr">
         <is>
           <t>color key — this KRA's band and row tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>KPI Tracker FY26-27 (tab 4)</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Annual tracker in the org Head-Abstract format — one Budgeted / Actual / Variance / Remarks set for FY 2026-27, Actual updated at each KPI's frequency. Variance = Budgeted − Actual (org convention): negative = beat on higher-is-better rows; rows flagged 'lower is better' read inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="48" t="inlineStr">
+        <is>
+          <t>Tracker conventions</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>KPI name follows Category:Product:Cohort::Name; per-batch rows split into B3 / B4. Budgets are numeric — the ≤ / ≥ direction lives in Description and Remarks. Blank Budgeted = first-quarter baseline sets it. The tracker's Budgeted is the number of record; the map's KPI target mirrors it, never the reverse.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="50" t="inlineStr">
+        <is>
+          <t>S. No.</t>
+        </is>
+      </c>
+      <c r="B1" s="50" t="inlineStr">
+        <is>
+          <t>KRA</t>
+        </is>
+      </c>
+      <c r="C1" s="50" t="inlineStr">
+        <is>
+          <t>Metric category</t>
+        </is>
+      </c>
+      <c r="D1" s="50" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" s="50" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="F1" s="50" t="inlineStr">
+        <is>
+          <t>Metric name</t>
+        </is>
+      </c>
+      <c r="G1" s="50" t="inlineStr">
+        <is>
+          <t>KPI name (naming convention)</t>
+        </is>
+      </c>
+      <c r="H1" s="50" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="I1" s="50" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="J1" s="50" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="K1" s="50" t="inlineStr">
+        <is>
+          <t>Lane (KPI owner)</t>
+        </is>
+      </c>
+      <c r="L1" s="51" t="inlineStr">
+        <is>
+          <t>FY 2026-27 — annual</t>
+        </is>
+      </c>
+      <c r="M1" s="52" t="n"/>
+      <c r="N1" s="52" t="n"/>
+      <c r="O1" s="52" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="50" t="n"/>
+      <c r="B2" s="50" t="n"/>
+      <c r="C2" s="50" t="n"/>
+      <c r="D2" s="50" t="n"/>
+      <c r="E2" s="50" t="n"/>
+      <c r="F2" s="50" t="n"/>
+      <c r="G2" s="50" t="n"/>
+      <c r="H2" s="50" t="n"/>
+      <c r="I2" s="50" t="n"/>
+      <c r="J2" s="50" t="n"/>
+      <c r="K2" s="50" t="n"/>
+      <c r="L2" s="50" t="inlineStr">
+        <is>
+          <t>Budgeted</t>
+        </is>
+      </c>
+      <c r="M2" s="50" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="N2" s="50" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="O2" s="50" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="54" t="inlineStr">
+        <is>
+          <t>KRA 1 — SPI Bands
+30% at ≥8.0 · 40% at 7.0–8.0 · 30% at 6.0–7.0, per batch</t>
+        </is>
+      </c>
+      <c r="C3" s="55" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D3" s="53" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E3" s="53" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F3" s="56" t="inlineStr">
+        <is>
+          <t>Program Delivery Gap  [CASCADE]</t>
+        </is>
+      </c>
+      <c r="G3" s="55" t="inlineStr">
+        <is>
+          <t>Delivery:NIAT::Program Delivery Gap</t>
+        </is>
+      </c>
+      <c r="H3" s="55" t="inlineStr">
+        <is>
+          <t>% deviation of the executed schedule vs the designed schedule, across the journey steps (lectures, quizzes, practice releases, assets)</t>
+        </is>
+      </c>
+      <c r="I3" s="53" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J3" s="55" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K3" s="55" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L3" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="58" t="n"/>
+      <c r="N3" s="59">
+        <f>IF(AND(ISNUMBER(L3),ISNUMBER(M3)),L3-M3,"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="55" t="inlineStr">
+        <is>
+          <t>CASCADE — feeds KRA 1 + KRA 3, tracked once (no double count). Lower is better — variance reads inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="61" t="n"/>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F4" s="63" t="inlineStr">
+        <is>
+          <t>Module-Quiz Score Bands</t>
+        </is>
+      </c>
+      <c r="G4" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::% in Module-Quiz Band ≥8.0</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>Share of the batch in each module-quiz band (10-pt scale) — one band stricter than the org bands</t>
+        </is>
+      </c>
+      <c r="I4" s="60" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J4" s="62" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K4" s="62" t="inlineStr">
+        <is>
+          <t>Learning Domains</t>
+        </is>
+      </c>
+      <c r="L4" s="64" t="n">
+        <v>30</v>
+      </c>
+      <c r="M4" s="65" t="n"/>
+      <c r="N4" s="66">
+        <f>IF(AND(ISNUMBER(L4),ISNUMBER(M4)),L4-M4,"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="62" t="inlineStr">
+        <is>
+          <t>Four band rows per batch sum to 100; the &lt;5.0 rows target 0 (lower is better). B4 rows go live with the batch's first module quiz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="61" t="n"/>
+      <c r="C5" s="65" t="n"/>
+      <c r="D5" s="65" t="n"/>
+      <c r="E5" s="65" t="n"/>
+      <c r="F5" s="65" t="n"/>
+      <c r="G5" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::% in Module-Quiz Band 7.0–8.0</t>
+        </is>
+      </c>
+      <c r="H5" s="65" t="n"/>
+      <c r="I5" s="65" t="n"/>
+      <c r="J5" s="65" t="n"/>
+      <c r="K5" s="65" t="n"/>
+      <c r="L5" s="64" t="n">
+        <v>40</v>
+      </c>
+      <c r="M5" s="65" t="n"/>
+      <c r="N5" s="66">
+        <f>IF(AND(ISNUMBER(L5),ISNUMBER(M5)),L5-M5,"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="65" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="61" t="n"/>
+      <c r="C6" s="65" t="n"/>
+      <c r="D6" s="65" t="n"/>
+      <c r="E6" s="65" t="n"/>
+      <c r="F6" s="65" t="n"/>
+      <c r="G6" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::% in Module-Quiz Band 5.0–7.0</t>
+        </is>
+      </c>
+      <c r="H6" s="65" t="n"/>
+      <c r="I6" s="65" t="n"/>
+      <c r="J6" s="65" t="n"/>
+      <c r="K6" s="65" t="n"/>
+      <c r="L6" s="64" t="n">
+        <v>30</v>
+      </c>
+      <c r="M6" s="65" t="n"/>
+      <c r="N6" s="66">
+        <f>IF(AND(ISNUMBER(L6),ISNUMBER(M6)),L6-M6,"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="65" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="61" t="n"/>
+      <c r="C7" s="65" t="n"/>
+      <c r="D7" s="65" t="n"/>
+      <c r="E7" s="65" t="n"/>
+      <c r="F7" s="65" t="n"/>
+      <c r="G7" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::% in Module-Quiz Band &lt;5.0</t>
+        </is>
+      </c>
+      <c r="H7" s="65" t="n"/>
+      <c r="I7" s="65" t="n"/>
+      <c r="J7" s="65" t="n"/>
+      <c r="K7" s="65" t="n"/>
+      <c r="L7" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="65" t="n"/>
+      <c r="N7" s="66">
+        <f>IF(AND(ISNUMBER(L7),ISNUMBER(M7)),L7-M7,"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="65" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="61" t="n"/>
+      <c r="C8" s="65" t="n"/>
+      <c r="D8" s="65" t="n"/>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="F8" s="65" t="n"/>
+      <c r="G8" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::% in Module-Quiz Band ≥8.0</t>
+        </is>
+      </c>
+      <c r="H8" s="65" t="n"/>
+      <c r="I8" s="65" t="n"/>
+      <c r="J8" s="65" t="n"/>
+      <c r="K8" s="65" t="n"/>
+      <c r="L8" s="64" t="n">
+        <v>30</v>
+      </c>
+      <c r="M8" s="65" t="n"/>
+      <c r="N8" s="66">
+        <f>IF(AND(ISNUMBER(L8),ISNUMBER(M8)),L8-M8,"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="65" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="61" t="n"/>
+      <c r="C9" s="65" t="n"/>
+      <c r="D9" s="65" t="n"/>
+      <c r="E9" s="65" t="n"/>
+      <c r="F9" s="65" t="n"/>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::% in Module-Quiz Band 7.0–8.0</t>
+        </is>
+      </c>
+      <c r="H9" s="65" t="n"/>
+      <c r="I9" s="65" t="n"/>
+      <c r="J9" s="65" t="n"/>
+      <c r="K9" s="65" t="n"/>
+      <c r="L9" s="64" t="n">
+        <v>40</v>
+      </c>
+      <c r="M9" s="65" t="n"/>
+      <c r="N9" s="66">
+        <f>IF(AND(ISNUMBER(L9),ISNUMBER(M9)),L9-M9,"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="65" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="61" t="n"/>
+      <c r="C10" s="65" t="n"/>
+      <c r="D10" s="65" t="n"/>
+      <c r="E10" s="65" t="n"/>
+      <c r="F10" s="65" t="n"/>
+      <c r="G10" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::% in Module-Quiz Band 5.0–7.0</t>
+        </is>
+      </c>
+      <c r="H10" s="65" t="n"/>
+      <c r="I10" s="65" t="n"/>
+      <c r="J10" s="65" t="n"/>
+      <c r="K10" s="65" t="n"/>
+      <c r="L10" s="64" t="n">
+        <v>30</v>
+      </c>
+      <c r="M10" s="65" t="n"/>
+      <c r="N10" s="66">
+        <f>IF(AND(ISNUMBER(L10),ISNUMBER(M10)),L10-M10,"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="65" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="61" t="n"/>
+      <c r="C11" s="65" t="n"/>
+      <c r="D11" s="65" t="n"/>
+      <c r="E11" s="65" t="n"/>
+      <c r="F11" s="65" t="n"/>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::% in Module-Quiz Band &lt;5.0</t>
+        </is>
+      </c>
+      <c r="H11" s="65" t="n"/>
+      <c r="I11" s="65" t="n"/>
+      <c r="J11" s="65" t="n"/>
+      <c r="K11" s="65" t="n"/>
+      <c r="L11" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="65" t="n"/>
+      <c r="N11" s="66">
+        <f>IF(AND(ISNUMBER(L11),ISNUMBER(M11)),L11-M11,"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="65" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="60" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="61" t="n"/>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F12" s="63" t="inlineStr">
+        <is>
+          <t>Content–Assessment Alignment</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::Content–Assessment Alignment</t>
+        </is>
+      </c>
+      <c r="H12" s="62" t="inlineStr">
+        <is>
+          <t>|avg module-quiz score − avg skill-assessment score| — the taught-vs-tested gap</t>
+        </is>
+      </c>
+      <c r="I12" s="60" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
+      </c>
+      <c r="J12" s="62" t="inlineStr">
+        <is>
+          <t>Per cycle</t>
+        </is>
+      </c>
+      <c r="K12" s="62" t="inlineStr">
+        <is>
+          <t>Learning Domains</t>
+        </is>
+      </c>
+      <c r="L12" s="64" t="n">
+        <v>10</v>
+      </c>
+      <c r="M12" s="65" t="n"/>
+      <c r="N12" s="66">
+        <f>IF(AND(ISNUMBER(L12),ISNUMBER(M12)),L12-M12,"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="62" t="inlineStr">
+        <is>
+          <t>Lower is better — variance reads inverted. Tightens to ≤5 pp after 3 clean cycles (cycle = semester).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="60" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="61" t="n"/>
+      <c r="C13" s="65" t="n"/>
+      <c r="D13" s="65" t="n"/>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="F13" s="65" t="n"/>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::Content–Assessment Alignment</t>
+        </is>
+      </c>
+      <c r="H13" s="65" t="n"/>
+      <c r="I13" s="65" t="n"/>
+      <c r="J13" s="65" t="n"/>
+      <c r="K13" s="65" t="n"/>
+      <c r="L13" s="64" t="n">
+        <v>10</v>
+      </c>
+      <c r="M13" s="65" t="n"/>
+      <c r="N13" s="66">
+        <f>IF(AND(ISNUMBER(L13),ISNUMBER(M13)),L13-M13,"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="65" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="61" t="n"/>
+      <c r="C14" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F14" s="63" t="inlineStr">
+        <is>
+          <t>Engagement-Matrix Cell Migration  [SAMPLE]</t>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr">
+        <is>
+          <t>Business Impact:All::% Learners in HE×HV Cell</t>
+        </is>
+      </c>
+      <c r="H14" s="62" t="inlineStr">
+        <is>
+          <t>% of learners in the HE×HV (high-effort × high-value) cell; the full 3×3 matrix stays diagnostic</t>
+        </is>
+      </c>
+      <c r="I14" s="60" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J14" s="62" t="inlineStr">
+        <is>
+          <t>Per cycle · read monthly</t>
+        </is>
+      </c>
+      <c r="K14" s="62" t="inlineStr">
+        <is>
+          <t>Learning Platform</t>
+        </is>
+      </c>
+      <c r="L14" s="64" t="n">
+        <v>10</v>
+      </c>
+      <c r="M14" s="65" t="n"/>
+      <c r="N14" s="66">
+        <f>IF(AND(ISNUMBER(L14),ISNUMBER(M14)),L14-M14,"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="62" t="inlineStr">
+        <is>
+          <t>SAMPLE — from ~4% baseline; budget confirms when the LE dashboard lands. Alt pick: M×M 10 → 20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="67" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="68" t="inlineStr">
+        <is>
+          <t>KRA 2 — Academics CSAT
+4.5 / 5</t>
+        </is>
+      </c>
+      <c r="C15" s="69" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D15" s="67" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E15" s="67" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F15" s="70" t="inlineStr">
+        <is>
+          <t>Content Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="G15" s="69" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Content Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="H15" s="69" t="inlineStr">
+        <is>
+          <t>% of content issues resolved within the 2-day TAT — resolved = fix live + students notified</t>
+        </is>
+      </c>
+      <c r="I15" s="67" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J15" s="69" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K15" s="69" t="inlineStr">
+        <is>
+          <t>Agentic Content Platform</t>
+        </is>
+      </c>
+      <c r="L15" s="71" t="n">
+        <v>80</v>
+      </c>
+      <c r="M15" s="72" t="n"/>
+      <c r="N15" s="73">
+        <f>IF(AND(ISNUMBER(L15),ISNUMBER(M15)),L15-M15,"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="69" t="inlineStr">
+        <is>
+          <t>The % climbs over the year; the 2-day TAT itself doesn't move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="74" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="75" t="n"/>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D16" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E16" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F16" s="77" t="inlineStr">
+        <is>
+          <t>Content Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="G16" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Content Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="H16" s="76" t="inlineStr">
+        <is>
+          <t>% of resolved content issues that recur — root-cause close: instance fixed · artifact changed · tripwire added · broadcast sent</t>
+        </is>
+      </c>
+      <c r="I16" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J16" s="76" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="K16" s="76" t="inlineStr">
+        <is>
+          <t>Agentic Content Platform</t>
+        </is>
+      </c>
+      <c r="L16" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" s="79" t="n"/>
+      <c r="N16" s="80">
+        <f>IF(AND(ISNUMBER(L16),ISNUMBER(M16)),L16-M16,"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="76" t="inlineStr">
+        <is>
+          <t>Lower is better — variance reads inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="74" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="75" t="n"/>
+      <c r="C17" s="76" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D17" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E17" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F17" s="77" t="inlineStr">
+        <is>
+          <t>Learning Environment Satisfaction</t>
+        </is>
+      </c>
+      <c r="G17" s="76" t="inlineStr">
+        <is>
+          <t>Business Impact:All::Learning Environment Satisfaction</t>
+        </is>
+      </c>
+      <c r="H17" s="76" t="inlineStr">
+        <is>
+          <t>Student rating of the learning environment — driven by the four platform rows below</t>
+        </is>
+      </c>
+      <c r="I17" s="74" t="inlineStr">
+        <is>
+          <t>score /5</t>
+        </is>
+      </c>
+      <c r="J17" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K17" s="76" t="inlineStr">
+        <is>
+          <t>Developer Platform</t>
+        </is>
+      </c>
+      <c r="L17" s="78" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M17" s="79" t="n"/>
+      <c r="N17" s="80">
+        <f>IF(AND(ISNUMBER(L17),ISNUMBER(M17)),L17-M17,"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="76" t="inlineStr"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="74" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="75" t="n"/>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D18" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E18" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F18" s="77" t="inlineStr">
+        <is>
+          <t>Availability &amp; Saturation Detection</t>
+        </is>
+      </c>
+      <c r="G18" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Availability &amp; Saturation Detection</t>
+        </is>
+      </c>
+      <c r="H18" s="76" t="inlineStr">
+        <is>
+          <t>% of critical-service saturations alerted, detection ≤10 min (IDE, compiler, workflows)</t>
+        </is>
+      </c>
+      <c r="I18" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J18" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K18" s="76" t="inlineStr">
+        <is>
+          <t>Developer Platform</t>
+        </is>
+      </c>
+      <c r="L18" s="78" t="n">
+        <v>100</v>
+      </c>
+      <c r="M18" s="79" t="n"/>
+      <c r="N18" s="80">
+        <f>IF(AND(ISNUMBER(L18),ISNUMBER(M18)),L18-M18,"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="76" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="74" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="75" t="n"/>
+      <c r="C19" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D19" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E19" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F19" s="77" t="inlineStr">
+        <is>
+          <t>Tail-Latency User Impact</t>
+        </is>
+      </c>
+      <c r="G19" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Tail-Latency User Impact</t>
+        </is>
+      </c>
+      <c r="H19" s="76" t="inlineStr">
+        <is>
+          <t>% of students beyond P99 latency limits — IDE launch / submit / publish &lt;60 s</t>
+        </is>
+      </c>
+      <c r="I19" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J19" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K19" s="76" t="inlineStr">
+        <is>
+          <t>Developer Platform</t>
+        </is>
+      </c>
+      <c r="L19" s="78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="79" t="n"/>
+      <c r="N19" s="80">
+        <f>IF(AND(ISNUMBER(L19),ISNUMBER(M19)),L19-M19,"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="76" t="inlineStr">
+        <is>
+          <t>Lower is better — variance reads inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="74" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="75" t="n"/>
+      <c r="C20" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D20" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E20" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F20" s="77" t="inlineStr">
+        <is>
+          <t>Platform Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="G20" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Platform Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="H20" s="76" t="inlineStr">
+        <is>
+          <t>% of platform issues resolved within the 2-day TAT (internal same-day)</t>
+        </is>
+      </c>
+      <c r="I20" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J20" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K20" s="76" t="inlineStr">
+        <is>
+          <t>Developer Platform</t>
+        </is>
+      </c>
+      <c r="L20" s="78" t="n">
+        <v>80</v>
+      </c>
+      <c r="M20" s="79" t="n"/>
+      <c r="N20" s="80">
+        <f>IF(AND(ISNUMBER(L20),ISNUMBER(M20)),L20-M20,"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="76" t="inlineStr"/>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="74" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="75" t="n"/>
+      <c r="C21" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D21" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E21" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F21" s="77" t="inlineStr">
+        <is>
+          <t>Platform Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="G21" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:All::Platform Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="H21" s="76" t="inlineStr">
+        <is>
+          <t>% of resolved platform issues that recur (quarter)</t>
+        </is>
+      </c>
+      <c r="I21" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J21" s="76" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="K21" s="76" t="inlineStr">
+        <is>
+          <t>Developer Platform</t>
+        </is>
+      </c>
+      <c r="L21" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="79" t="n"/>
+      <c r="N21" s="80">
+        <f>IF(AND(ISNUMBER(L21),ISNUMBER(M21)),L21-M21,"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="76" t="inlineStr">
+        <is>
+          <t>Lower is better — variance reads inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="74" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="75" t="n"/>
+      <c r="C22" s="76" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D22" s="74" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E22" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F22" s="77" t="inlineStr">
+        <is>
+          <t>Journey Step Health</t>
+        </is>
+      </c>
+      <c r="G22" s="76" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT::Journey Step Health</t>
+        </is>
+      </c>
+      <c r="H22" s="76" t="inlineStr">
+        <is>
+          <t>% of the 11 journey steps green — NIAT first, then per product</t>
+        </is>
+      </c>
+      <c r="I22" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J22" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K22" s="76" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L22" s="79" t="n"/>
+      <c r="M22" s="79" t="n"/>
+      <c r="N22" s="80">
+        <f>IF(AND(ISNUMBER(L22),ISNUMBER(M22)),L22-M22,"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="76" t="inlineStr">
+        <is>
+          <t>Q1 baseline sets the budget — blank until then (org-tracker precedent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="74" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="75" t="n"/>
+      <c r="C23" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D23" s="74" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E23" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F23" s="77" t="inlineStr">
+        <is>
+          <t>Product Issue Resolution Efficiency  [CROSS-DEPT]</t>
+        </is>
+      </c>
+      <c r="G23" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:NIAT::Product Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="H23" s="76" t="inlineStr">
+        <is>
+          <t>% of student-reported product issues resolved within TAT — resolved across departments, we route; fix live + students notified</t>
+        </is>
+      </c>
+      <c r="I23" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J23" s="76" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K23" s="76" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L23" s="79" t="n"/>
+      <c r="M23" s="79" t="n"/>
+      <c r="N23" s="80">
+        <f>IF(AND(ISNUMBER(L23),ISNUMBER(M23)),L23-M23,"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="76" t="inlineStr">
+        <is>
+          <t>Q1 baseline sets the TAT target — blank until then.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="74" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="75" t="n"/>
+      <c r="C24" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D24" s="74" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E24" s="74" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F24" s="77" t="inlineStr">
+        <is>
+          <t>Product Issue Recurrence  [CROSS-DEPT]</t>
+        </is>
+      </c>
+      <c r="G24" s="76" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:NIAT::Product Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="H24" s="76" t="inlineStr">
+        <is>
+          <t>% of resolved product issues that recur at student-journey level (quarter)</t>
+        </is>
+      </c>
+      <c r="I24" s="74" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J24" s="76" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="K24" s="76" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L24" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="79" t="n"/>
+      <c r="N24" s="80">
+        <f>IF(AND(ISNUMBER(L24),ISNUMBER(M24)),L24-M24,"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="76" t="inlineStr">
+        <is>
+          <t>Lower is better — variance reads inverted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="81" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="82" t="inlineStr">
+        <is>
+          <t>KRA 3 — University Relations CSAT
+4.5 · 4.0 · 4.0</t>
+        </is>
+      </c>
+      <c r="C25" s="83" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D25" s="81" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E25" s="81" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F25" s="84" t="inlineStr">
+        <is>
+          <t>BOS Credit Acceptance</t>
+        </is>
+      </c>
+      <c r="G25" s="83" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B3::BOS Credit Acceptance</t>
+        </is>
+      </c>
+      <c r="H25" s="83" t="inlineStr">
+        <is>
+          <t>% of proposed credits accepted first-pass by the university BOS</t>
+        </is>
+      </c>
+      <c r="I25" s="81" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J25" s="83" t="inlineStr">
+        <is>
+          <t>Per cycle</t>
+        </is>
+      </c>
+      <c r="K25" s="83" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L25" s="85" t="n">
+        <v>85</v>
+      </c>
+      <c r="M25" s="86" t="n"/>
+      <c r="N25" s="87">
+        <f>IF(AND(ISNUMBER(L25),ISNUMBER(M25)),L25-M25,"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="83" t="inlineStr">
+        <is>
+          <t>Cohort rows split where targets differ: B3 85 · B4 90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="88" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="89" t="n"/>
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="90" t="n"/>
+      <c r="E26" s="88" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="F26" s="90" t="n"/>
+      <c r="G26" s="91" t="inlineStr">
+        <is>
+          <t>Business Impact:NIAT:B4::BOS Credit Acceptance</t>
+        </is>
+      </c>
+      <c r="H26" s="90" t="n"/>
+      <c r="I26" s="90" t="n"/>
+      <c r="J26" s="90" t="n"/>
+      <c r="K26" s="90" t="n"/>
+      <c r="L26" s="92" t="n">
+        <v>90</v>
+      </c>
+      <c r="M26" s="90" t="n"/>
+      <c r="N26" s="93">
+        <f>IF(AND(ISNUMBER(L26),ISNUMBER(M26)),L26-M26,"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="90" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="88" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="89" t="n"/>
+      <c r="C27" s="91" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D27" s="88" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E27" s="88" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="94" t="inlineStr">
+        <is>
+          <t>University Communication TAT</t>
+        </is>
+      </c>
+      <c r="G27" s="91" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:NIAT::University Communication TAT</t>
+        </is>
+      </c>
+      <c r="H27" s="91" t="inlineStr">
+        <is>
+          <t>% of university requests answered within TAT — ack ≤1 business day, standard 3-day TAT</t>
+        </is>
+      </c>
+      <c r="I27" s="88" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J27" s="91" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K27" s="91" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L27" s="92" t="n">
+        <v>90</v>
+      </c>
+      <c r="M27" s="90" t="n"/>
+      <c r="N27" s="93">
+        <f>IF(AND(ISNUMBER(L27),ISNUMBER(M27)),L27-M27,"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="91" t="inlineStr">
+        <is>
+          <t>University-request log builds in month 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="88" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="89" t="n"/>
+      <c r="C28" s="91" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D28" s="88" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E28" s="88" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F28" s="94" t="inlineStr">
+        <is>
+          <t>University Curriculum &amp; Framework Compliance</t>
+        </is>
+      </c>
+      <c r="G28" s="91" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:NIAT::University Curriculum &amp; Framework Compliance</t>
+        </is>
+      </c>
+      <c r="H28" s="91" t="inlineStr">
+        <is>
+          <t>% of submission cycles fully compliant — approved BOS syllabus + NHQRF / Woolf / AICTE / UGC</t>
+        </is>
+      </c>
+      <c r="I28" s="88" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J28" s="91" t="inlineStr">
+        <is>
+          <t>Per cycle</t>
+        </is>
+      </c>
+      <c r="K28" s="91" t="inlineStr">
+        <is>
+          <t>Product Learning Experience</t>
+        </is>
+      </c>
+      <c r="L28" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="M28" s="90" t="n"/>
+      <c r="N28" s="93">
+        <f>IF(AND(ISNUMBER(L28),ISNUMBER(M28)),L28-M28,"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="91" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="95" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="96" t="inlineStr">
+        <is>
+          <t>KRA 4 — GRIT Novice Badges
+5,000</t>
+        </is>
+      </c>
+      <c r="C29" s="97" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D29" s="95" t="inlineStr">
+        <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="E29" s="95" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F29" s="98" t="inlineStr">
+        <is>
+          <t>Industry Update Adherence</t>
+        </is>
+      </c>
+      <c r="G29" s="97" t="inlineStr">
+        <is>
+          <t>Quality &amp; Reliability:NIAT::Industry Update Adherence</t>
+        </is>
+      </c>
+      <c r="H29" s="97" t="inlineStr">
+        <is>
+          <t>% of GRIT-tested skills covered in live course content — Learning–GRIT delta → 0</t>
+        </is>
+      </c>
+      <c r="I29" s="95" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J29" s="97" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="K29" s="97" t="inlineStr">
+        <is>
+          <t>Learning Domains</t>
+        </is>
+      </c>
+      <c r="L29" s="99" t="n">
+        <v>100</v>
+      </c>
+      <c r="M29" s="100" t="n"/>
+      <c r="N29" s="101">
+        <f>IF(AND(ISNUMBER(L29),ISNUMBER(M29)),L29-M29,"")</f>
+        <v/>
+      </c>
+      <c r="O29" s="97" t="inlineStr"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="102" t="n"/>
+      <c r="B30" s="103" t="n"/>
+      <c r="C30" s="104" t="inlineStr">
+        <is>
+          <t>GRIT-feature KPIs — org-owned, pending definition with the GRIT owner (Sundar); rows enter the tracker when defined.</t>
+        </is>
+      </c>
+      <c r="D30" s="102" t="n"/>
+      <c r="E30" s="102" t="n"/>
+      <c r="F30" s="102" t="n"/>
+      <c r="G30" s="102" t="n"/>
+      <c r="H30" s="102" t="n"/>
+      <c r="I30" s="102" t="n"/>
+      <c r="J30" s="102" t="n"/>
+      <c r="K30" s="102" t="n"/>
+      <c r="L30" s="102" t="n"/>
+      <c r="M30" s="102" t="n"/>
+      <c r="N30" s="102" t="n"/>
+      <c r="O30" s="102" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="105" t="n"/>
+      <c r="B31" s="106" t="inlineStr">
+        <is>
+          <t>KRA 5 — Employability
+B3 80% · B4 80%</t>
+        </is>
+      </c>
+      <c r="C31" s="107" t="inlineStr">
+        <is>
+          <t>Employability mapping deliberately not forced — skill mastery is the long lever; rows enter the tracker when the mapping is agreed.</t>
+        </is>
+      </c>
+      <c r="D31" s="105" t="n"/>
+      <c r="E31" s="105" t="n"/>
+      <c r="F31" s="105" t="n"/>
+      <c r="G31" s="105" t="n"/>
+      <c r="H31" s="105" t="n"/>
+      <c r="I31" s="105" t="n"/>
+      <c r="J31" s="105" t="n"/>
+      <c r="K31" s="105" t="n"/>
+      <c r="L31" s="105" t="n"/>
+      <c r="M31" s="105" t="n"/>
+      <c r="N31" s="105" t="n"/>
+      <c r="O31" s="105" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="I4:I11"/>
+    <mergeCell ref="K4:K11"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="F4:F11"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="H4:H11"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="O12:O13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C30:O30"/>
+    <mergeCell ref="B3:B14"/>
+    <mergeCell ref="C4:C11"/>
+    <mergeCell ref="B31"/>
+    <mergeCell ref="O4:O11"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="D4:D11"/>
+    <mergeCell ref="J4:J11"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="C31:O31"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="B15:B24"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Category re-map: org 7 + Program Delivery / University Alignment / Platform Reliability
CSI (a team) and Developer Platform (a lane) were sitting on the category
axis; replaced by three what-it-measures categories per Pavan's approval.
Tracker col C + all 27 KPI-name prefixes re-derived; one-pager §4/§5/§9
re-grouped, lane totals unchanged. Operating view sync deferred.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C3" s="55" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Program Delivery</t>
         </is>
       </c>
       <c r="D3" s="53" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="G3" s="55" t="inlineStr">
         <is>
-          <t>Delivery:NIAT::Program Delivery Gap</t>
+          <t>Program Delivery:NIAT::Program Delivery Gap</t>
         </is>
       </c>
       <c r="H3" s="55" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="C16" s="69" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D16" s="67" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="G16" s="69" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Content Issue Resolution Efficiency</t>
+          <t>Content Efficiency:All::Content Issue Resolution Efficiency</t>
         </is>
       </c>
       <c r="H16" s="69" t="inlineStr">
@@ -2394,7 +2394,7 @@
       <c r="B17" s="75" t="n"/>
       <c r="C17" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D17" s="74" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="G17" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Content Issue Recurrence</t>
+          <t>Content Efficiency:All::Content Issue Recurrence</t>
         </is>
       </c>
       <c r="H17" s="76" t="inlineStr">
@@ -2473,7 +2473,7 @@
       <c r="B18" s="75" t="n"/>
       <c r="C18" s="76" t="inlineStr">
         <is>
-          <t>Business Impact</t>
+          <t>Content Effectiveness</t>
         </is>
       </c>
       <c r="D18" s="74" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="G18" s="76" t="inlineStr">
         <is>
-          <t>Business Impact:All::Learning Environment Satisfaction</t>
+          <t>Content Effectiveness:All::Learning Environment Satisfaction</t>
         </is>
       </c>
       <c r="H18" s="76" t="inlineStr">
@@ -2548,7 +2548,7 @@
       <c r="B19" s="75" t="n"/>
       <c r="C19" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Platform Reliability</t>
         </is>
       </c>
       <c r="D19" s="74" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="G19" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Availability &amp; Saturation Detection</t>
+          <t>Platform Reliability:All::Availability &amp; Saturation Detection</t>
         </is>
       </c>
       <c r="H19" s="76" t="inlineStr">
@@ -2623,7 +2623,7 @@
       <c r="B20" s="75" t="n"/>
       <c r="C20" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Platform Reliability</t>
         </is>
       </c>
       <c r="D20" s="74" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="G20" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Tail-Latency User Impact</t>
+          <t>Platform Reliability:All::Tail-Latency User Impact</t>
         </is>
       </c>
       <c r="H20" s="76" t="inlineStr">
@@ -2702,7 +2702,7 @@
       <c r="B21" s="75" t="n"/>
       <c r="C21" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Platform Reliability</t>
         </is>
       </c>
       <c r="D21" s="74" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="G21" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Platform Issue Resolution Efficiency</t>
+          <t>Platform Reliability:All::Platform Issue Resolution Efficiency</t>
         </is>
       </c>
       <c r="H21" s="76" t="inlineStr">
@@ -2777,7 +2777,7 @@
       <c r="B22" s="75" t="n"/>
       <c r="C22" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Platform Reliability</t>
         </is>
       </c>
       <c r="D22" s="74" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G22" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:All::Platform Issue Recurrence</t>
+          <t>Platform Reliability:All::Platform Issue Recurrence</t>
         </is>
       </c>
       <c r="H22" s="76" t="inlineStr">
@@ -2856,7 +2856,7 @@
       <c r="B23" s="75" t="n"/>
       <c r="C23" s="76" t="inlineStr">
         <is>
-          <t>Business Impact</t>
+          <t>Program Delivery</t>
         </is>
       </c>
       <c r="D23" s="74" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="G23" s="76" t="inlineStr">
         <is>
-          <t>Business Impact:NIAT::Journey Step Health</t>
+          <t>Program Delivery:NIAT::Journey Step Health</t>
         </is>
       </c>
       <c r="H23" s="76" t="inlineStr">
@@ -2933,7 +2933,7 @@
       <c r="B24" s="75" t="n"/>
       <c r="C24" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D24" s="74" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G24" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:NIAT::Product Issue Resolution Efficiency</t>
+          <t>Content Efficiency:NIAT::Product Issue Resolution Efficiency</t>
         </is>
       </c>
       <c r="H24" s="76" t="inlineStr">
@@ -3010,7 +3010,7 @@
       <c r="B25" s="75" t="n"/>
       <c r="C25" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D25" s="74" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="G25" s="76" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:NIAT::Product Issue Recurrence</t>
+          <t>Content Efficiency:NIAT::Product Issue Recurrence</t>
         </is>
       </c>
       <c r="H25" s="76" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="C26" s="83" t="inlineStr">
         <is>
-          <t>Business Impact</t>
+          <t>University Alignment</t>
         </is>
       </c>
       <c r="D26" s="81" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="G26" s="83" t="inlineStr">
         <is>
-          <t>Business Impact:NIAT:B3::BOS Credit Acceptance</t>
+          <t>University Alignment:NIAT:B3::BOS Credit Acceptance</t>
         </is>
       </c>
       <c r="H26" s="83" t="inlineStr">
@@ -3181,7 +3181,7 @@
       <c r="F27" s="90" t="n"/>
       <c r="G27" s="91" t="inlineStr">
         <is>
-          <t>Business Impact:NIAT:B4::BOS Credit Acceptance</t>
+          <t>University Alignment:NIAT:B4::BOS Credit Acceptance</t>
         </is>
       </c>
       <c r="H27" s="90" t="n"/>
@@ -3232,7 +3232,7 @@
       <c r="B29" s="89" t="n"/>
       <c r="C29" s="91" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>University Alignment</t>
         </is>
       </c>
       <c r="D29" s="88" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="G29" s="91" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:NIAT::University Communication TAT</t>
+          <t>University Alignment:NIAT::University Communication TAT</t>
         </is>
       </c>
       <c r="H29" s="91" t="inlineStr">
@@ -3311,7 +3311,7 @@
       <c r="B30" s="89" t="n"/>
       <c r="C30" s="91" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Relevance</t>
         </is>
       </c>
       <c r="D30" s="88" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G30" s="91" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:NIAT::University Curriculum &amp; Framework Compliance</t>
+          <t>Content Relevance:NIAT::University Curriculum &amp; Framework Compliance</t>
         </is>
       </c>
       <c r="H30" s="91" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="C31" s="97" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability</t>
+          <t>Content Relevance</t>
         </is>
       </c>
       <c r="D31" s="95" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="G31" s="97" t="inlineStr">
         <is>
-          <t>Quality &amp; Reliability:NIAT::Industry Update Adherence</t>
+          <t>Content Relevance:NIAT::Industry Update Adherence</t>
         </is>
       </c>
       <c r="H31" s="97" t="inlineStr">
@@ -3744,7 +3744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3955,6 +3955,18 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="55" customHeight="1">
+      <c r="A20" s="48" t="inlineStr">
+        <is>
+          <t>Metric categories (col C)</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>Org Head-Abstract vocabulary — Business Impact · Content Effectiveness · Content Velocity · Content Efficiency · Content Relevance · Stakeholder Alignment · Executive Ops — plus three department extensions: Program Delivery · University Alignment · Platform Reliability. Category = what the KPI measures; Lane (col L) = who is accountable; Functions (col K) = who does the work.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cadence fixes: PDG weekly; Alignment monthly vs biweekly skill assessments
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -1769,7 +1769,7 @@
       </c>
       <c r="N3" s="55" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Weekly</t>
         </is>
       </c>
       <c r="O3" s="57" t="n">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H12" s="62" t="inlineStr">
         <is>
-          <t>|avg module-quiz score − avg skill-assessment score| — the taught-vs-tested gap</t>
+          <t>|avg module-quiz score − avg biweekly skill-assessment score| — the taught-vs-tested gap</t>
         </is>
       </c>
       <c r="I12" s="62" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="N12" s="62" t="inlineStr">
         <is>
-          <t>Per cycle</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="O12" s="64" t="n">

</xml_diff>

<commit_message>
CROSS-FUNCTION marker (was CROSS-DEPT) + lane legend on both artifacts
Product Issue rows: resolution spans functions, not departments — tag,
legend, and both descriptions renamed everywhere (builder, json, xlsx,
tracker HTML, one-pager §5/§6/tag legend). Lanes explained: tracker
key-point + Legend B3 glosses; one-pager §2 Lanes row + axis one-liner
(category = what · lane = accountable · function = does the work).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -2948,7 +2948,7 @@
       </c>
       <c r="F24" s="77" t="inlineStr">
         <is>
-          <t>Product Issue Resolution Efficiency  [CROSS-DEPT]</t>
+          <t>Product Issue Resolution Efficiency  [CROSS-FUNCTION]</t>
         </is>
       </c>
       <c r="G24" s="76" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="H24" s="76" t="inlineStr">
         <is>
-          <t>% of student-reported product issues resolved within TAT — resolved across departments, we route; fix live + students notified</t>
+          <t>% of student-reported product issues resolved within TAT — resolved across functions, we route; fix live + students notified</t>
         </is>
       </c>
       <c r="I24" s="76" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="F25" s="77" t="inlineStr">
         <is>
-          <t>Product Issue Recurrence  [CROSS-DEPT]</t>
+          <t>Product Issue Recurrence  [CROSS-FUNCTION]</t>
         </is>
       </c>
       <c r="G25" s="76" t="inlineStr">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="34" customHeight="1">
+    <row r="3" ht="70" customHeight="1">
       <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Lane (KPI owner)</t>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B3" s="33" t="inlineStr">
         <is>
-          <t>A lane is an accountability grouping of KPIs, NOT a team — the lane lead answers for the number at review. Lanes: Learning Domains · Learning Platform · Developer Platform · Agentic Content Platform · Product Learning Experience.</t>
+          <t>A lane is an accountability grouping of KPIs, NOT a team — the lane lead answers for the number at review. Learning Domains (domain curriculum, pedagogy &amp; question banks) · Learning Platform (shared study / practice / revision / assessment capabilities) · Product Learning Experience (product-specific learning experiences + university delivery &amp; compliance) · Agentic Content Platform (AI platforms &amp; automation for content production) · Developer Platform (IDE, compiler &amp; platform services) · Shared/PMO (department-wide programs). Category (col C) = what it measures · Lane (col L) = who is accountable · Functions (col K) = who does the work.</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Markers</t>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>[ORG] org-owned scoreboard, tracked not owned · [CROSS-DEPT] resolved across departments, we route · [SAMPLE] illustrative numbers until baselines land · [CASCADE] same KPI feeds two KRAs.</t>
+          <t>[ORG] org-owned scoreboard, tracked not owned · [CROSS-FUNCTION] resolved across functions, we route · [SAMPLE] illustrative numbers until baselines land · [CASCADE] same KPI feeds two KRAs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team-view tabs (CSI + FS&CS) + JSH/PDG existence-vs-health + §11 step owners
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Tracker FY26-27" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Index" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSI Team View" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FullStack &amp; CS Core View" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +77,28 @@
       <color rgb="FF777777"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="27">
     <fill>
       <patternFill/>
     </fill>
@@ -196,8 +218,18 @@
         <fgColor rgb="FFFCEBF1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A78D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1BAF7A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="59">
+  <borders count="60">
     <border>
       <left/>
       <right/>
@@ -912,11 +944,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF555555"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1198,6 +1244,58 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="22" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1702,7 +1800,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="84" customHeight="1">
+    <row r="3" ht="110" customHeight="1">
       <c r="A3" s="53" t="n">
         <v>1</v>
       </c>
@@ -1739,12 +1837,12 @@
       </c>
       <c r="H3" s="55" t="inlineStr">
         <is>
-          <t>% deviation of the executed schedule vs the designed schedule, across the journey steps (lectures, quizzes, practice releases, assets)</t>
+          <t>% deviation of the executed schedule vs the designed schedule, across the journey steps (lectures, quizzes, practice releases, assets) — existence only: a step that never runs counts here, not in Journey Step Health</t>
         </is>
       </c>
       <c r="I3" s="55" t="inlineStr">
         <is>
-          <t>lecture schedule adherence · classroom-quiz conduction &amp; attendance · practice release schedule · module-quiz schedule adherence &amp; integrity · skill-assessment schedule adherence (conducted by Program Ops) · learning assets (PPT + recorded video) ready &amp; loaded ≥1 month ahead</t>
+          <t>lecture schedule adherence (Program Ops) · classroom-quiz conduction &amp; attendance (Instructors) · practice release schedule (Program Ops + Learning Domains) · module-quiz schedule adherence &amp; integrity (Program Ops) · skill-assessment schedule adherence (Program Ops conducts) · learning assets (PPT + recorded video) ready &amp; loaded ≥1 month ahead (Instructors-dept SLA)</t>
         </is>
       </c>
       <c r="J3" s="55" t="inlineStr">
@@ -1782,7 +1880,7 @@
       </c>
       <c r="R3" s="55" t="inlineStr">
         <is>
-          <t>CASCADE — feeds KRA 1 + KRA 3, tracked once (no double count). Lower is better — variance reads inverted.</t>
+          <t>CASCADE — feeds KRA 1 + KRA 3, tracked once (no double count). Lower is better — variance reads inverted. Assembled KPI — each dependent step carries a named owner (col I); we orchestrate, route, escalate: red 2 consecutive weeks → HOD-to-HOD.</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="45" customHeight="1">
+    <row r="23" ht="110" customHeight="1">
       <c r="A23" s="74" t="n">
         <v>20</v>
       </c>
@@ -2881,12 +2979,12 @@
       </c>
       <c r="H23" s="76" t="inlineStr">
         <is>
-          <t>% of the 11 journey steps green — NIAT first, then per product</t>
+          <t>% of the journey steps that ran this month finishing green (one-pager §11 thresholds) — NIAT first, then per product. Health of what ran: a step that never ran counts in PDG, not here</t>
         </is>
       </c>
       <c r="I23" s="76" t="inlineStr">
         <is>
-          <t>the 11 journey steps — attendance · class runs · classroom quiz · practice · revision · module quiz · skill assessment … (one-pager §11)</t>
+          <t>the 11 journey steps, each with a named owner (§11 owner column) — attendance (Program Ops) · class runs (Program Ops + Instructors) · classroom quiz (Instructors) · quiz performance (Learning Domains) · practice availability (Program Ops + LD/ACP) · practice return &amp; completion (LP lane) · revision (LP lane) · module quiz (Program Ops) · skill assessment (Program Ops) · SA preparedness (Learning Domains)</t>
         </is>
       </c>
       <c r="J23" s="76" t="inlineStr">
@@ -2922,7 +3020,7 @@
       </c>
       <c r="R23" s="76" t="inlineStr">
         <is>
-          <t>Q1 baseline sets the budget — blank until then (org-tracker precedent).</t>
+          <t>Q1 baseline sets the budget — blank until then (org-tracker precedent). Assembled KPI — steps owned per col I (§11 owner column); we orchestrate, route, escalate.</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3967,7 +4065,3319 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="48" t="inlineStr">
+        <is>
+          <t>Team views (tabs 4–5)</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>Functional Operating Views — one satellite tab per team, docked to the tracker, never merged. Section A mirrors the tracker rows the team is on the hook for (live formulas — numbers are edited on the tracker tab only). Section B = KPIs the team owns, budgets &amp; actuals here, each with a Ladders-to call: direct (an org KRA number) · enabling (a dept §5 KPI) · hygiene (guardrail, no ladder by design). Section C = asks of counterparties. Pilots: CSI team · FullStack &amp; CS Core.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF2A78D6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="115" t="inlineStr">
+        <is>
+          <t>CSI team — Functional Operating View · FY 2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="116" t="inlineStr">
+        <is>
+          <t>Curriculum Systems &amp; Infrastructure — Product Learning Experience lane. Section A mirrors the department tracker (live formulas — numbers are edited on the KPI Tracker tab only) · Section B is owned here, budgets &amp; actuals live on this tab · Section C = asks of counterparties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="117" t="inlineStr">
+        <is>
+          <t>S. No</t>
+        </is>
+      </c>
+      <c r="B3" s="117" t="inlineStr">
+        <is>
+          <t>Sect</t>
+        </is>
+      </c>
+      <c r="C3" s="117" t="inlineStr">
+        <is>
+          <t>Metric category</t>
+        </is>
+      </c>
+      <c r="D3" s="117" t="inlineStr">
+        <is>
+          <t>KPI name</t>
+        </is>
+      </c>
+      <c r="E3" s="117" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F3" s="117" t="inlineStr">
+        <is>
+          <t>Ladders to</t>
+        </is>
+      </c>
+      <c r="G3" s="117" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H3" s="117" t="inlineStr">
+        <is>
+          <t>Freq</t>
+        </is>
+      </c>
+      <c r="I3" s="117" t="inlineStr">
+        <is>
+          <t>Budgeted</t>
+        </is>
+      </c>
+      <c r="J3" s="117" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="K3" s="117" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="L3" s="117" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="118" t="inlineStr">
+        <is>
+          <t>A — Inherited: org-KRA rows this team is on the hook for (live mirror — numbers live on the KPI Tracker tab; edit there)</t>
+        </is>
+      </c>
+      <c r="B4" s="119" t="n"/>
+      <c r="C4" s="119" t="n"/>
+      <c r="D4" s="119" t="n"/>
+      <c r="E4" s="119" t="n"/>
+      <c r="F4" s="119" t="n"/>
+      <c r="G4" s="119" t="n"/>
+      <c r="H4" s="119" t="n"/>
+      <c r="I4" s="119" t="n"/>
+      <c r="J4" s="119" t="n"/>
+      <c r="K4" s="119" t="n"/>
+      <c r="L4" s="119" t="n"/>
+    </row>
+    <row r="5" ht="71" customHeight="1">
+      <c r="A5" s="120" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B5" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="121">
+        <f>IF('KPI Tracker FY26-27'!C3="","",'KPI Tracker FY26-27'!C3)</f>
+        <v/>
+      </c>
+      <c r="D5" s="122">
+        <f>IF('KPI Tracker FY26-27'!G3="","",'KPI Tracker FY26-27'!G3)</f>
+        <v/>
+      </c>
+      <c r="E5" s="121">
+        <f>IF('KPI Tracker FY26-27'!H3="","",'KPI Tracker FY26-27'!H3)</f>
+        <v/>
+      </c>
+      <c r="F5" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G5" s="120">
+        <f>IF('KPI Tracker FY26-27'!M3="","",'KPI Tracker FY26-27'!M3)</f>
+        <v/>
+      </c>
+      <c r="H5" s="120">
+        <f>IF('KPI Tracker FY26-27'!N3="","",'KPI Tracker FY26-27'!N3)</f>
+        <v/>
+      </c>
+      <c r="I5" s="120">
+        <f>IF('KPI Tracker FY26-27'!O3="","",'KPI Tracker FY26-27'!O3)</f>
+        <v/>
+      </c>
+      <c r="J5" s="120">
+        <f>IF('KPI Tracker FY26-27'!P3="","",'KPI Tracker FY26-27'!P3)</f>
+        <v/>
+      </c>
+      <c r="K5" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q3="","",'KPI Tracker FY26-27'!Q3)</f>
+        <v/>
+      </c>
+      <c r="L5" s="121">
+        <f>IF('KPI Tracker FY26-27'!R3="","",'KPI Tracker FY26-27'!R3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="120" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="B6" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="121">
+        <f>IF('KPI Tracker FY26-27'!C23="","",'KPI Tracker FY26-27'!C23)</f>
+        <v/>
+      </c>
+      <c r="D6" s="122">
+        <f>IF('KPI Tracker FY26-27'!G23="","",'KPI Tracker FY26-27'!G23)</f>
+        <v/>
+      </c>
+      <c r="E6" s="121">
+        <f>IF('KPI Tracker FY26-27'!H23="","",'KPI Tracker FY26-27'!H23)</f>
+        <v/>
+      </c>
+      <c r="F6" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G6" s="120">
+        <f>IF('KPI Tracker FY26-27'!M23="","",'KPI Tracker FY26-27'!M23)</f>
+        <v/>
+      </c>
+      <c r="H6" s="120">
+        <f>IF('KPI Tracker FY26-27'!N23="","",'KPI Tracker FY26-27'!N23)</f>
+        <v/>
+      </c>
+      <c r="I6" s="120">
+        <f>IF('KPI Tracker FY26-27'!O23="","",'KPI Tracker FY26-27'!O23)</f>
+        <v/>
+      </c>
+      <c r="J6" s="120">
+        <f>IF('KPI Tracker FY26-27'!P23="","",'KPI Tracker FY26-27'!P23)</f>
+        <v/>
+      </c>
+      <c r="K6" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q23="","",'KPI Tracker FY26-27'!Q23)</f>
+        <v/>
+      </c>
+      <c r="L6" s="121">
+        <f>IF('KPI Tracker FY26-27'!R23="","",'KPI Tracker FY26-27'!R23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="120" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B7" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" s="121">
+        <f>IF('KPI Tracker FY26-27'!C24="","",'KPI Tracker FY26-27'!C24)</f>
+        <v/>
+      </c>
+      <c r="D7" s="122">
+        <f>IF('KPI Tracker FY26-27'!G24="","",'KPI Tracker FY26-27'!G24)</f>
+        <v/>
+      </c>
+      <c r="E7" s="121">
+        <f>IF('KPI Tracker FY26-27'!H24="","",'KPI Tracker FY26-27'!H24)</f>
+        <v/>
+      </c>
+      <c r="F7" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G7" s="120">
+        <f>IF('KPI Tracker FY26-27'!M24="","",'KPI Tracker FY26-27'!M24)</f>
+        <v/>
+      </c>
+      <c r="H7" s="120">
+        <f>IF('KPI Tracker FY26-27'!N24="","",'KPI Tracker FY26-27'!N24)</f>
+        <v/>
+      </c>
+      <c r="I7" s="120">
+        <f>IF('KPI Tracker FY26-27'!O24="","",'KPI Tracker FY26-27'!O24)</f>
+        <v/>
+      </c>
+      <c r="J7" s="120">
+        <f>IF('KPI Tracker FY26-27'!P24="","",'KPI Tracker FY26-27'!P24)</f>
+        <v/>
+      </c>
+      <c r="K7" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q24="","",'KPI Tracker FY26-27'!Q24)</f>
+        <v/>
+      </c>
+      <c r="L7" s="121">
+        <f>IF('KPI Tracker FY26-27'!R24="","",'KPI Tracker FY26-27'!R24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="120" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B8" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" s="121">
+        <f>IF('KPI Tracker FY26-27'!C25="","",'KPI Tracker FY26-27'!C25)</f>
+        <v/>
+      </c>
+      <c r="D8" s="122">
+        <f>IF('KPI Tracker FY26-27'!G25="","",'KPI Tracker FY26-27'!G25)</f>
+        <v/>
+      </c>
+      <c r="E8" s="121">
+        <f>IF('KPI Tracker FY26-27'!H25="","",'KPI Tracker FY26-27'!H25)</f>
+        <v/>
+      </c>
+      <c r="F8" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G8" s="120">
+        <f>IF('KPI Tracker FY26-27'!M25="","",'KPI Tracker FY26-27'!M25)</f>
+        <v/>
+      </c>
+      <c r="H8" s="120">
+        <f>IF('KPI Tracker FY26-27'!N25="","",'KPI Tracker FY26-27'!N25)</f>
+        <v/>
+      </c>
+      <c r="I8" s="120">
+        <f>IF('KPI Tracker FY26-27'!O25="","",'KPI Tracker FY26-27'!O25)</f>
+        <v/>
+      </c>
+      <c r="J8" s="120">
+        <f>IF('KPI Tracker FY26-27'!P25="","",'KPI Tracker FY26-27'!P25)</f>
+        <v/>
+      </c>
+      <c r="K8" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q25="","",'KPI Tracker FY26-27'!Q25)</f>
+        <v/>
+      </c>
+      <c r="L8" s="121">
+        <f>IF('KPI Tracker FY26-27'!R25="","",'KPI Tracker FY26-27'!R25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="120" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B9" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" s="121">
+        <f>IF('KPI Tracker FY26-27'!C26="","",'KPI Tracker FY26-27'!C26)</f>
+        <v/>
+      </c>
+      <c r="D9" s="122">
+        <f>IF('KPI Tracker FY26-27'!G26="","",'KPI Tracker FY26-27'!G26)</f>
+        <v/>
+      </c>
+      <c r="E9" s="121">
+        <f>IF('KPI Tracker FY26-27'!H26="","",'KPI Tracker FY26-27'!H26)</f>
+        <v/>
+      </c>
+      <c r="F9" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G9" s="120">
+        <f>IF('KPI Tracker FY26-27'!M26="","",'KPI Tracker FY26-27'!M26)</f>
+        <v/>
+      </c>
+      <c r="H9" s="120">
+        <f>IF('KPI Tracker FY26-27'!N26="","",'KPI Tracker FY26-27'!N26)</f>
+        <v/>
+      </c>
+      <c r="I9" s="120">
+        <f>IF('KPI Tracker FY26-27'!O26="","",'KPI Tracker FY26-27'!O26)</f>
+        <v/>
+      </c>
+      <c r="J9" s="120">
+        <f>IF('KPI Tracker FY26-27'!P26="","",'KPI Tracker FY26-27'!P26)</f>
+        <v/>
+      </c>
+      <c r="K9" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q26="","",'KPI Tracker FY26-27'!Q26)</f>
+        <v/>
+      </c>
+      <c r="L9" s="121">
+        <f>IF('KPI Tracker FY26-27'!R26="","",'KPI Tracker FY26-27'!R26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="120" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B10" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C10" s="121">
+        <f>IF('KPI Tracker FY26-27'!C26="","",'KPI Tracker FY26-27'!C26)</f>
+        <v/>
+      </c>
+      <c r="D10" s="122">
+        <f>IF('KPI Tracker FY26-27'!G27="","",'KPI Tracker FY26-27'!G27)</f>
+        <v/>
+      </c>
+      <c r="E10" s="121">
+        <f>IF('KPI Tracker FY26-27'!H26="","",'KPI Tracker FY26-27'!H26)</f>
+        <v/>
+      </c>
+      <c r="F10" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G10" s="120">
+        <f>IF('KPI Tracker FY26-27'!M26="","",'KPI Tracker FY26-27'!M26)</f>
+        <v/>
+      </c>
+      <c r="H10" s="120">
+        <f>IF('KPI Tracker FY26-27'!N26="","",'KPI Tracker FY26-27'!N26)</f>
+        <v/>
+      </c>
+      <c r="I10" s="120">
+        <f>IF('KPI Tracker FY26-27'!O27="","",'KPI Tracker FY26-27'!O27)</f>
+        <v/>
+      </c>
+      <c r="J10" s="120">
+        <f>IF('KPI Tracker FY26-27'!P27="","",'KPI Tracker FY26-27'!P27)</f>
+        <v/>
+      </c>
+      <c r="K10" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q27="","",'KPI Tracker FY26-27'!Q27)</f>
+        <v/>
+      </c>
+      <c r="L10" s="121">
+        <f>IF('KPI Tracker FY26-27'!R26="","",'KPI Tracker FY26-27'!R26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="120" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="B11" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C11" s="121">
+        <f>IF('KPI Tracker FY26-27'!C29="","",'KPI Tracker FY26-27'!C29)</f>
+        <v/>
+      </c>
+      <c r="D11" s="122">
+        <f>IF('KPI Tracker FY26-27'!G29="","",'KPI Tracker FY26-27'!G29)</f>
+        <v/>
+      </c>
+      <c r="E11" s="121">
+        <f>IF('KPI Tracker FY26-27'!H29="","",'KPI Tracker FY26-27'!H29)</f>
+        <v/>
+      </c>
+      <c r="F11" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G11" s="120">
+        <f>IF('KPI Tracker FY26-27'!M29="","",'KPI Tracker FY26-27'!M29)</f>
+        <v/>
+      </c>
+      <c r="H11" s="120">
+        <f>IF('KPI Tracker FY26-27'!N29="","",'KPI Tracker FY26-27'!N29)</f>
+        <v/>
+      </c>
+      <c r="I11" s="120">
+        <f>IF('KPI Tracker FY26-27'!O29="","",'KPI Tracker FY26-27'!O29)</f>
+        <v/>
+      </c>
+      <c r="J11" s="120">
+        <f>IF('KPI Tracker FY26-27'!P29="","",'KPI Tracker FY26-27'!P29)</f>
+        <v/>
+      </c>
+      <c r="K11" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q29="","",'KPI Tracker FY26-27'!Q29)</f>
+        <v/>
+      </c>
+      <c r="L11" s="121">
+        <f>IF('KPI Tracker FY26-27'!R29="","",'KPI Tracker FY26-27'!R29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="120" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+      <c r="B12" s="120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C12" s="121">
+        <f>IF('KPI Tracker FY26-27'!C30="","",'KPI Tracker FY26-27'!C30)</f>
+        <v/>
+      </c>
+      <c r="D12" s="122">
+        <f>IF('KPI Tracker FY26-27'!G30="","",'KPI Tracker FY26-27'!G30)</f>
+        <v/>
+      </c>
+      <c r="E12" s="121">
+        <f>IF('KPI Tracker FY26-27'!H30="","",'KPI Tracker FY26-27'!H30)</f>
+        <v/>
+      </c>
+      <c r="F12" s="121" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G12" s="120">
+        <f>IF('KPI Tracker FY26-27'!M30="","",'KPI Tracker FY26-27'!M30)</f>
+        <v/>
+      </c>
+      <c r="H12" s="120">
+        <f>IF('KPI Tracker FY26-27'!N30="","",'KPI Tracker FY26-27'!N30)</f>
+        <v/>
+      </c>
+      <c r="I12" s="120">
+        <f>IF('KPI Tracker FY26-27'!O30="","",'KPI Tracker FY26-27'!O30)</f>
+        <v/>
+      </c>
+      <c r="J12" s="120">
+        <f>IF('KPI Tracker FY26-27'!P30="","",'KPI Tracker FY26-27'!P30)</f>
+        <v/>
+      </c>
+      <c r="K12" s="120">
+        <f>IF('KPI Tracker FY26-27'!Q30="","",'KPI Tracker FY26-27'!Q30)</f>
+        <v/>
+      </c>
+      <c r="L12" s="121">
+        <f>IF('KPI Tracker FY26-27'!R30="","",'KPI Tracker FY26-27'!R30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="118" t="inlineStr">
+        <is>
+          <t>B — Owned: functional KPIs this team runs (budgets &amp; actuals live here) — Ladders-to key: direct = an org-KRA number · enabling = a dept §5 KPI · hygiene = guardrail by design</t>
+        </is>
+      </c>
+      <c r="B13" s="119" t="n"/>
+      <c r="C13" s="119" t="n"/>
+      <c r="D13" s="119" t="n"/>
+      <c r="E13" s="119" t="n"/>
+      <c r="F13" s="119" t="n"/>
+      <c r="G13" s="119" t="n"/>
+      <c r="H13" s="119" t="n"/>
+      <c r="I13" s="119" t="n"/>
+      <c r="J13" s="119" t="n"/>
+      <c r="K13" s="119" t="n"/>
+      <c r="L13" s="119" t="n"/>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C14" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D14" s="125" t="inlineStr">
+        <is>
+          <t>Cost per BOS Approval (NIAT)</t>
+        </is>
+      </c>
+      <c r="E14" s="124" t="inlineStr">
+        <is>
+          <t>Average cost incurred per approved BOS across university partners. Includes CSI team payroll and non-payroll costs (travel, liaison activities) attributed to BOS approval work.</t>
+        </is>
+      </c>
+      <c r="F14" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per BOS Approval (§5 Content Efficiency) — the economics of the KRA-3 BOS engine</t>
+        </is>
+      </c>
+      <c r="G14" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H14" s="123" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I14" s="123" t="n"/>
+      <c r="J14" s="123" t="n"/>
+      <c r="K14" s="126">
+        <f>IF(AND(ISNUMBER(I14),ISNUMBER(J14)),I14-J14,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="124" t="inlineStr">
+        <is>
+          <t>Q1 ref: B ₹14,040 (quarterly).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="123" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C15" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D15" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Vernacular Content Hour (NIAT + Academy)</t>
+        </is>
+      </c>
+      <c r="E15" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to produce one hour of vernacular-language content, tracked centrally by the CSI team. Includes CSI payroll and AI tooling costs attributed to vernacular production.</t>
+        </is>
+      </c>
+      <c r="F15" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per Vernacular Content Hour (§5 Content Efficiency) — central track; FS&amp;CS Core carries the production-side twin</t>
+        </is>
+      </c>
+      <c r="G15" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H15" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I15" s="123" t="n"/>
+      <c r="J15" s="123" t="n"/>
+      <c r="K15" s="126">
+        <f>IF(AND(ISNUMBER(I15),ISNUMBER(J15)),I15-J15,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="124" t="inlineStr"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="123" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C16" s="124" t="inlineStr">
+        <is>
+          <t>Executive Ops</t>
+        </is>
+      </c>
+      <c r="D16" s="125" t="inlineStr">
+        <is>
+          <t>Operations &amp; Growth Cost</t>
+        </is>
+      </c>
+      <c r="E16" s="124" t="inlineStr">
+        <is>
+          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+        </is>
+      </c>
+      <c r="F16" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="G16" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H16" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I16" s="123" t="n"/>
+      <c r="J16" s="123" t="n"/>
+      <c r="K16" s="126">
+        <f>IF(AND(ISNUMBER(I16),ISNUMBER(J16)),I16-J16,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="124" t="inlineStr"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="118" t="inlineStr">
+        <is>
+          <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
+        </is>
+      </c>
+      <c r="B17" s="119" t="n"/>
+      <c r="C17" s="119" t="n"/>
+      <c r="D17" s="119" t="n"/>
+      <c r="E17" s="119" t="n"/>
+      <c r="F17" s="119" t="n"/>
+      <c r="G17" s="119" t="n"/>
+      <c r="H17" s="119" t="n"/>
+      <c r="I17" s="119" t="n"/>
+      <c r="J17" s="119" t="n"/>
+      <c r="K17" s="119" t="n"/>
+      <c r="L17" s="119" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="120" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="120" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C18" s="121" t="inlineStr">
+        <is>
+          <t>Program Ops</t>
+        </is>
+      </c>
+      <c r="D18" s="122" t="inlineStr">
+        <is>
+          <t>Conduction adherence</t>
+        </is>
+      </c>
+      <c r="E18" s="121" t="inlineStr">
+        <is>
+          <t>Zero schedule deviation on lectures / quizzes / assessments + attendance drive — feeds Program Delivery Gap &amp; Journey Step Health (§7 ask; exact thresholds pending).</t>
+        </is>
+      </c>
+      <c r="F18" s="121" t="n"/>
+      <c r="G18" s="120" t="n"/>
+      <c r="H18" s="120" t="n"/>
+      <c r="I18" s="120" t="n"/>
+      <c r="J18" s="120" t="n"/>
+      <c r="K18" s="120" t="n"/>
+      <c r="L18" s="121" t="n"/>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="120" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C19" s="121" t="inlineStr">
+        <is>
+          <t>Instructors dept</t>
+        </is>
+      </c>
+      <c r="D19" s="122" t="inlineStr">
+        <is>
+          <t>Learning-assets SLA</t>
+        </is>
+      </c>
+      <c r="E19" s="121" t="inlineStr">
+        <is>
+          <t>PPT + recorded video ready &amp; loaded ≥1 month ahead of delivery — feeds the assets leg of Program Delivery Gap.</t>
+        </is>
+      </c>
+      <c r="F19" s="121" t="n"/>
+      <c r="G19" s="120" t="n"/>
+      <c r="H19" s="120" t="n"/>
+      <c r="I19" s="120" t="n"/>
+      <c r="J19" s="120" t="n"/>
+      <c r="K19" s="120" t="n"/>
+      <c r="L19" s="121" t="n"/>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="120" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C20" s="121" t="inlineStr">
+        <is>
+          <t>Univ Relations</t>
+        </is>
+      </c>
+      <c r="D20" s="122" t="inlineStr">
+        <is>
+          <t>University response windows</t>
+        </is>
+      </c>
+      <c r="E20" s="121" t="inlineStr">
+        <is>
+          <t>BOS meeting windows + response SLAs on university communications — feeds BOS Credit Acceptance &amp; University Communication TAT.</t>
+        </is>
+      </c>
+      <c r="F20" s="121" t="n"/>
+      <c r="G20" s="120" t="n"/>
+      <c r="H20" s="120" t="n"/>
+      <c r="I20" s="120" t="n"/>
+      <c r="J20" s="120" t="n"/>
+      <c r="K20" s="120" t="n"/>
+      <c r="L20" s="121" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="E18:L18"/>
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="E19:L19"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF1BAF7A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="127" t="inlineStr">
+        <is>
+          <t>FullStack &amp; CS Core — Functional Operating View · FY 2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="116" t="inlineStr">
+        <is>
+          <t>Learning Domains lane — Content function. Section A mirrors the department tracker (live formulas — numbers are edited on the KPI Tracker tab only) · Section B is owned here, budgets &amp; actuals live on this tab · Section C = asks of counterparties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="128" t="inlineStr">
+        <is>
+          <t>S. No</t>
+        </is>
+      </c>
+      <c r="B3" s="128" t="inlineStr">
+        <is>
+          <t>Sect</t>
+        </is>
+      </c>
+      <c r="C3" s="128" t="inlineStr">
+        <is>
+          <t>Metric category</t>
+        </is>
+      </c>
+      <c r="D3" s="128" t="inlineStr">
+        <is>
+          <t>KPI name</t>
+        </is>
+      </c>
+      <c r="E3" s="128" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F3" s="128" t="inlineStr">
+        <is>
+          <t>Ladders to</t>
+        </is>
+      </c>
+      <c r="G3" s="128" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H3" s="128" t="inlineStr">
+        <is>
+          <t>Freq</t>
+        </is>
+      </c>
+      <c r="I3" s="128" t="inlineStr">
+        <is>
+          <t>Budgeted</t>
+        </is>
+      </c>
+      <c r="J3" s="128" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="K3" s="128" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="L3" s="128" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="129" t="inlineStr">
+        <is>
+          <t>A — Inherited: org-KRA rows this team is on the hook for (live mirror — numbers live on the KPI Tracker tab; edit there)</t>
+        </is>
+      </c>
+      <c r="B4" s="119" t="n"/>
+      <c r="C4" s="119" t="n"/>
+      <c r="D4" s="119" t="n"/>
+      <c r="E4" s="119" t="n"/>
+      <c r="F4" s="119" t="n"/>
+      <c r="G4" s="119" t="n"/>
+      <c r="H4" s="119" t="n"/>
+      <c r="I4" s="119" t="n"/>
+      <c r="J4" s="119" t="n"/>
+      <c r="K4" s="119" t="n"/>
+      <c r="L4" s="119" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="130" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B5" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D5" s="132">
+        <f>IF('KPI Tracker FY26-27'!G4="","",'KPI Tracker FY26-27'!G4)</f>
+        <v/>
+      </c>
+      <c r="E5" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F5" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G5" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H5" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I5" s="130">
+        <f>IF('KPI Tracker FY26-27'!O4="","",'KPI Tracker FY26-27'!O4)</f>
+        <v/>
+      </c>
+      <c r="J5" s="130">
+        <f>IF('KPI Tracker FY26-27'!P4="","",'KPI Tracker FY26-27'!P4)</f>
+        <v/>
+      </c>
+      <c r="K5" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q4="","",'KPI Tracker FY26-27'!Q4)</f>
+        <v/>
+      </c>
+      <c r="L5" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="130" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B6" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D6" s="132">
+        <f>IF('KPI Tracker FY26-27'!G5="","",'KPI Tracker FY26-27'!G5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F6" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G6" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H6" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I6" s="130">
+        <f>IF('KPI Tracker FY26-27'!O5="","",'KPI Tracker FY26-27'!O5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="130">
+        <f>IF('KPI Tracker FY26-27'!P5="","",'KPI Tracker FY26-27'!P5)</f>
+        <v/>
+      </c>
+      <c r="K6" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q5="","",'KPI Tracker FY26-27'!Q5)</f>
+        <v/>
+      </c>
+      <c r="L6" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="130" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B7" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D7" s="132">
+        <f>IF('KPI Tracker FY26-27'!G6="","",'KPI Tracker FY26-27'!G6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F7" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G7" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H7" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I7" s="130">
+        <f>IF('KPI Tracker FY26-27'!O6="","",'KPI Tracker FY26-27'!O6)</f>
+        <v/>
+      </c>
+      <c r="J7" s="130">
+        <f>IF('KPI Tracker FY26-27'!P6="","",'KPI Tracker FY26-27'!P6)</f>
+        <v/>
+      </c>
+      <c r="K7" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q6="","",'KPI Tracker FY26-27'!Q6)</f>
+        <v/>
+      </c>
+      <c r="L7" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="130" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="B8" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D8" s="132">
+        <f>IF('KPI Tracker FY26-27'!G7="","",'KPI Tracker FY26-27'!G7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F8" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G8" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H8" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I8" s="130">
+        <f>IF('KPI Tracker FY26-27'!O7="","",'KPI Tracker FY26-27'!O7)</f>
+        <v/>
+      </c>
+      <c r="J8" s="130">
+        <f>IF('KPI Tracker FY26-27'!P7="","",'KPI Tracker FY26-27'!P7)</f>
+        <v/>
+      </c>
+      <c r="K8" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q7="","",'KPI Tracker FY26-27'!Q7)</f>
+        <v/>
+      </c>
+      <c r="L8" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="130" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="B9" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D9" s="132">
+        <f>IF('KPI Tracker FY26-27'!G8="","",'KPI Tracker FY26-27'!G8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F9" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G9" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H9" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I9" s="130">
+        <f>IF('KPI Tracker FY26-27'!O8="","",'KPI Tracker FY26-27'!O8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="130">
+        <f>IF('KPI Tracker FY26-27'!P8="","",'KPI Tracker FY26-27'!P8)</f>
+        <v/>
+      </c>
+      <c r="K9" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q8="","",'KPI Tracker FY26-27'!Q8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="130" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="B10" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C10" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D10" s="132">
+        <f>IF('KPI Tracker FY26-27'!G9="","",'KPI Tracker FY26-27'!G9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F10" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G10" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H10" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I10" s="130">
+        <f>IF('KPI Tracker FY26-27'!O9="","",'KPI Tracker FY26-27'!O9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="130">
+        <f>IF('KPI Tracker FY26-27'!P9="","",'KPI Tracker FY26-27'!P9)</f>
+        <v/>
+      </c>
+      <c r="K10" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q9="","",'KPI Tracker FY26-27'!Q9)</f>
+        <v/>
+      </c>
+      <c r="L10" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="130" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="B11" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C11" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D11" s="132">
+        <f>IF('KPI Tracker FY26-27'!G10="","",'KPI Tracker FY26-27'!G10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F11" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G11" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H11" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I11" s="130">
+        <f>IF('KPI Tracker FY26-27'!O10="","",'KPI Tracker FY26-27'!O10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="130">
+        <f>IF('KPI Tracker FY26-27'!P10="","",'KPI Tracker FY26-27'!P10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q10="","",'KPI Tracker FY26-27'!Q10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="130" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="B12" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C12" s="131">
+        <f>IF('KPI Tracker FY26-27'!C4="","",'KPI Tracker FY26-27'!C4)</f>
+        <v/>
+      </c>
+      <c r="D12" s="132">
+        <f>IF('KPI Tracker FY26-27'!G11="","",'KPI Tracker FY26-27'!G11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="131">
+        <f>IF('KPI Tracker FY26-27'!H4="","",'KPI Tracker FY26-27'!H4)</f>
+        <v/>
+      </c>
+      <c r="F12" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G12" s="130">
+        <f>IF('KPI Tracker FY26-27'!M4="","",'KPI Tracker FY26-27'!M4)</f>
+        <v/>
+      </c>
+      <c r="H12" s="130">
+        <f>IF('KPI Tracker FY26-27'!N4="","",'KPI Tracker FY26-27'!N4)</f>
+        <v/>
+      </c>
+      <c r="I12" s="130">
+        <f>IF('KPI Tracker FY26-27'!O11="","",'KPI Tracker FY26-27'!O11)</f>
+        <v/>
+      </c>
+      <c r="J12" s="130">
+        <f>IF('KPI Tracker FY26-27'!P11="","",'KPI Tracker FY26-27'!P11)</f>
+        <v/>
+      </c>
+      <c r="K12" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q11="","",'KPI Tracker FY26-27'!Q11)</f>
+        <v/>
+      </c>
+      <c r="L12" s="131">
+        <f>IF('KPI Tracker FY26-27'!R4="","",'KPI Tracker FY26-27'!R4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="130" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B13" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C13" s="131">
+        <f>IF('KPI Tracker FY26-27'!C12="","",'KPI Tracker FY26-27'!C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="132">
+        <f>IF('KPI Tracker FY26-27'!G12="","",'KPI Tracker FY26-27'!G12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="131">
+        <f>IF('KPI Tracker FY26-27'!H12="","",'KPI Tracker FY26-27'!H12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G13" s="130">
+        <f>IF('KPI Tracker FY26-27'!M12="","",'KPI Tracker FY26-27'!M12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="130">
+        <f>IF('KPI Tracker FY26-27'!N12="","",'KPI Tracker FY26-27'!N12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="130">
+        <f>IF('KPI Tracker FY26-27'!O12="","",'KPI Tracker FY26-27'!O12)</f>
+        <v/>
+      </c>
+      <c r="J13" s="130">
+        <f>IF('KPI Tracker FY26-27'!P12="","",'KPI Tracker FY26-27'!P12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q12="","",'KPI Tracker FY26-27'!Q12)</f>
+        <v/>
+      </c>
+      <c r="L13" s="131">
+        <f>IF('KPI Tracker FY26-27'!R12="","",'KPI Tracker FY26-27'!R12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="130" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B14" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C14" s="131">
+        <f>IF('KPI Tracker FY26-27'!C12="","",'KPI Tracker FY26-27'!C12)</f>
+        <v/>
+      </c>
+      <c r="D14" s="132">
+        <f>IF('KPI Tracker FY26-27'!G13="","",'KPI Tracker FY26-27'!G13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="131">
+        <f>IF('KPI Tracker FY26-27'!H12="","",'KPI Tracker FY26-27'!H12)</f>
+        <v/>
+      </c>
+      <c r="F14" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G14" s="130">
+        <f>IF('KPI Tracker FY26-27'!M12="","",'KPI Tracker FY26-27'!M12)</f>
+        <v/>
+      </c>
+      <c r="H14" s="130">
+        <f>IF('KPI Tracker FY26-27'!N12="","",'KPI Tracker FY26-27'!N12)</f>
+        <v/>
+      </c>
+      <c r="I14" s="130">
+        <f>IF('KPI Tracker FY26-27'!O13="","",'KPI Tracker FY26-27'!O13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="130">
+        <f>IF('KPI Tracker FY26-27'!P13="","",'KPI Tracker FY26-27'!P13)</f>
+        <v/>
+      </c>
+      <c r="K14" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q13="","",'KPI Tracker FY26-27'!Q13)</f>
+        <v/>
+      </c>
+      <c r="L14" s="131">
+        <f>IF('KPI Tracker FY26-27'!R12="","",'KPI Tracker FY26-27'!R12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="130" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B15" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C15" s="131">
+        <f>IF('KPI Tracker FY26-27'!C14="","",'KPI Tracker FY26-27'!C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="132">
+        <f>IF('KPI Tracker FY26-27'!G14="","",'KPI Tracker FY26-27'!G14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="131">
+        <f>IF('KPI Tracker FY26-27'!H14="","",'KPI Tracker FY26-27'!H14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="131" t="inlineStr">
+        <is>
+          <t>inherited — team-sheet twin</t>
+        </is>
+      </c>
+      <c r="G15" s="130">
+        <f>IF('KPI Tracker FY26-27'!M14="","",'KPI Tracker FY26-27'!M14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="130">
+        <f>IF('KPI Tracker FY26-27'!N14="","",'KPI Tracker FY26-27'!N14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="130">
+        <f>IF('KPI Tracker FY26-27'!O14="","",'KPI Tracker FY26-27'!O14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="130">
+        <f>IF('KPI Tracker FY26-27'!P14="","",'KPI Tracker FY26-27'!P14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q14="","",'KPI Tracker FY26-27'!Q14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="131">
+        <f>IF('KPI Tracker FY26-27'!R14="","",'KPI Tracker FY26-27'!R14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="130" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B16" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C16" s="131">
+        <f>IF('KPI Tracker FY26-27'!C16="","",'KPI Tracker FY26-27'!C16)</f>
+        <v/>
+      </c>
+      <c r="D16" s="132">
+        <f>IF('KPI Tracker FY26-27'!G16="","",'KPI Tracker FY26-27'!G16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="131">
+        <f>IF('KPI Tracker FY26-27'!H16="","",'KPI Tracker FY26-27'!H16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G16" s="130">
+        <f>IF('KPI Tracker FY26-27'!M16="","",'KPI Tracker FY26-27'!M16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="130">
+        <f>IF('KPI Tracker FY26-27'!N16="","",'KPI Tracker FY26-27'!N16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="130">
+        <f>IF('KPI Tracker FY26-27'!O16="","",'KPI Tracker FY26-27'!O16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="130">
+        <f>IF('KPI Tracker FY26-27'!P16="","",'KPI Tracker FY26-27'!P16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q16="","",'KPI Tracker FY26-27'!Q16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="131">
+        <f>IF('KPI Tracker FY26-27'!R16="","",'KPI Tracker FY26-27'!R16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="130" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="B17" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C17" s="131">
+        <f>IF('KPI Tracker FY26-27'!C17="","",'KPI Tracker FY26-27'!C17)</f>
+        <v/>
+      </c>
+      <c r="D17" s="132">
+        <f>IF('KPI Tracker FY26-27'!G17="","",'KPI Tracker FY26-27'!G17)</f>
+        <v/>
+      </c>
+      <c r="E17" s="131">
+        <f>IF('KPI Tracker FY26-27'!H17="","",'KPI Tracker FY26-27'!H17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G17" s="130">
+        <f>IF('KPI Tracker FY26-27'!M17="","",'KPI Tracker FY26-27'!M17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="130">
+        <f>IF('KPI Tracker FY26-27'!N17="","",'KPI Tracker FY26-27'!N17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="130">
+        <f>IF('KPI Tracker FY26-27'!O17="","",'KPI Tracker FY26-27'!O17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="130">
+        <f>IF('KPI Tracker FY26-27'!P17="","",'KPI Tracker FY26-27'!P17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q17="","",'KPI Tracker FY26-27'!Q17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="131">
+        <f>IF('KPI Tracker FY26-27'!R17="","",'KPI Tracker FY26-27'!R17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="130" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B18" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C18" s="131">
+        <f>IF('KPI Tracker FY26-27'!C18="","",'KPI Tracker FY26-27'!C18)</f>
+        <v/>
+      </c>
+      <c r="D18" s="132">
+        <f>IF('KPI Tracker FY26-27'!G18="","",'KPI Tracker FY26-27'!G18)</f>
+        <v/>
+      </c>
+      <c r="E18" s="131">
+        <f>IF('KPI Tracker FY26-27'!H18="","",'KPI Tracker FY26-27'!H18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="131" t="inlineStr">
+        <is>
+          <t>inherited — team-sheet twin</t>
+        </is>
+      </c>
+      <c r="G18" s="130">
+        <f>IF('KPI Tracker FY26-27'!M18="","",'KPI Tracker FY26-27'!M18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="130">
+        <f>IF('KPI Tracker FY26-27'!N18="","",'KPI Tracker FY26-27'!N18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="130">
+        <f>IF('KPI Tracker FY26-27'!O18="","",'KPI Tracker FY26-27'!O18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="130">
+        <f>IF('KPI Tracker FY26-27'!P18="","",'KPI Tracker FY26-27'!P18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q18="","",'KPI Tracker FY26-27'!Q18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="131">
+        <f>IF('KPI Tracker FY26-27'!R18="","",'KPI Tracker FY26-27'!R18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="130" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B19" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C19" s="131">
+        <f>IF('KPI Tracker FY26-27'!C26="","",'KPI Tracker FY26-27'!C26)</f>
+        <v/>
+      </c>
+      <c r="D19" s="132">
+        <f>IF('KPI Tracker FY26-27'!G26="","",'KPI Tracker FY26-27'!G26)</f>
+        <v/>
+      </c>
+      <c r="E19" s="131">
+        <f>IF('KPI Tracker FY26-27'!H26="","",'KPI Tracker FY26-27'!H26)</f>
+        <v/>
+      </c>
+      <c r="F19" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G19" s="130">
+        <f>IF('KPI Tracker FY26-27'!M26="","",'KPI Tracker FY26-27'!M26)</f>
+        <v/>
+      </c>
+      <c r="H19" s="130">
+        <f>IF('KPI Tracker FY26-27'!N26="","",'KPI Tracker FY26-27'!N26)</f>
+        <v/>
+      </c>
+      <c r="I19" s="130">
+        <f>IF('KPI Tracker FY26-27'!O26="","",'KPI Tracker FY26-27'!O26)</f>
+        <v/>
+      </c>
+      <c r="J19" s="130">
+        <f>IF('KPI Tracker FY26-27'!P26="","",'KPI Tracker FY26-27'!P26)</f>
+        <v/>
+      </c>
+      <c r="K19" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q26="","",'KPI Tracker FY26-27'!Q26)</f>
+        <v/>
+      </c>
+      <c r="L19" s="131">
+        <f>IF('KPI Tracker FY26-27'!R26="","",'KPI Tracker FY26-27'!R26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="130" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B20" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" s="131">
+        <f>IF('KPI Tracker FY26-27'!C26="","",'KPI Tracker FY26-27'!C26)</f>
+        <v/>
+      </c>
+      <c r="D20" s="132">
+        <f>IF('KPI Tracker FY26-27'!G27="","",'KPI Tracker FY26-27'!G27)</f>
+        <v/>
+      </c>
+      <c r="E20" s="131">
+        <f>IF('KPI Tracker FY26-27'!H26="","",'KPI Tracker FY26-27'!H26)</f>
+        <v/>
+      </c>
+      <c r="F20" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G20" s="130">
+        <f>IF('KPI Tracker FY26-27'!M26="","",'KPI Tracker FY26-27'!M26)</f>
+        <v/>
+      </c>
+      <c r="H20" s="130">
+        <f>IF('KPI Tracker FY26-27'!N26="","",'KPI Tracker FY26-27'!N26)</f>
+        <v/>
+      </c>
+      <c r="I20" s="130">
+        <f>IF('KPI Tracker FY26-27'!O27="","",'KPI Tracker FY26-27'!O27)</f>
+        <v/>
+      </c>
+      <c r="J20" s="130">
+        <f>IF('KPI Tracker FY26-27'!P27="","",'KPI Tracker FY26-27'!P27)</f>
+        <v/>
+      </c>
+      <c r="K20" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q27="","",'KPI Tracker FY26-27'!Q27)</f>
+        <v/>
+      </c>
+      <c r="L20" s="131">
+        <f>IF('KPI Tracker FY26-27'!R26="","",'KPI Tracker FY26-27'!R26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="130" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+      <c r="B21" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C21" s="131">
+        <f>IF('KPI Tracker FY26-27'!C30="","",'KPI Tracker FY26-27'!C30)</f>
+        <v/>
+      </c>
+      <c r="D21" s="132">
+        <f>IF('KPI Tracker FY26-27'!G30="","",'KPI Tracker FY26-27'!G30)</f>
+        <v/>
+      </c>
+      <c r="E21" s="131">
+        <f>IF('KPI Tracker FY26-27'!H30="","",'KPI Tracker FY26-27'!H30)</f>
+        <v/>
+      </c>
+      <c r="F21" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G21" s="130">
+        <f>IF('KPI Tracker FY26-27'!M30="","",'KPI Tracker FY26-27'!M30)</f>
+        <v/>
+      </c>
+      <c r="H21" s="130">
+        <f>IF('KPI Tracker FY26-27'!N30="","",'KPI Tracker FY26-27'!N30)</f>
+        <v/>
+      </c>
+      <c r="I21" s="130">
+        <f>IF('KPI Tracker FY26-27'!O30="","",'KPI Tracker FY26-27'!O30)</f>
+        <v/>
+      </c>
+      <c r="J21" s="130">
+        <f>IF('KPI Tracker FY26-27'!P30="","",'KPI Tracker FY26-27'!P30)</f>
+        <v/>
+      </c>
+      <c r="K21" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q30="","",'KPI Tracker FY26-27'!Q30)</f>
+        <v/>
+      </c>
+      <c r="L21" s="131">
+        <f>IF('KPI Tracker FY26-27'!R30="","",'KPI Tracker FY26-27'!R30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="130" t="inlineStr">
+        <is>
+          <t>T27</t>
+        </is>
+      </c>
+      <c r="B22" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C22" s="131">
+        <f>IF('KPI Tracker FY26-27'!C31="","",'KPI Tracker FY26-27'!C31)</f>
+        <v/>
+      </c>
+      <c r="D22" s="132">
+        <f>IF('KPI Tracker FY26-27'!G31="","",'KPI Tracker FY26-27'!G31)</f>
+        <v/>
+      </c>
+      <c r="E22" s="131">
+        <f>IF('KPI Tracker FY26-27'!H31="","",'KPI Tracker FY26-27'!H31)</f>
+        <v/>
+      </c>
+      <c r="F22" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="G22" s="130">
+        <f>IF('KPI Tracker FY26-27'!M31="","",'KPI Tracker FY26-27'!M31)</f>
+        <v/>
+      </c>
+      <c r="H22" s="130">
+        <f>IF('KPI Tracker FY26-27'!N31="","",'KPI Tracker FY26-27'!N31)</f>
+        <v/>
+      </c>
+      <c r="I22" s="130">
+        <f>IF('KPI Tracker FY26-27'!O31="","",'KPI Tracker FY26-27'!O31)</f>
+        <v/>
+      </c>
+      <c r="J22" s="130">
+        <f>IF('KPI Tracker FY26-27'!P31="","",'KPI Tracker FY26-27'!P31)</f>
+        <v/>
+      </c>
+      <c r="K22" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q31="","",'KPI Tracker FY26-27'!Q31)</f>
+        <v/>
+      </c>
+      <c r="L22" s="131">
+        <f>IF('KPI Tracker FY26-27'!R31="","",'KPI Tracker FY26-27'!R31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="129" t="inlineStr">
+        <is>
+          <t>B — Owned: functional KPIs this team runs (budgets &amp; actuals live here) — Ladders-to key: direct = an org-KRA number · enabling = a dept §5 KPI · hygiene = guardrail by design</t>
+        </is>
+      </c>
+      <c r="B23" s="119" t="n"/>
+      <c r="C23" s="119" t="n"/>
+      <c r="D23" s="119" t="n"/>
+      <c r="E23" s="119" t="n"/>
+      <c r="F23" s="119" t="n"/>
+      <c r="G23" s="119" t="n"/>
+      <c r="H23" s="119" t="n"/>
+      <c r="I23" s="119" t="n"/>
+      <c r="J23" s="119" t="n"/>
+      <c r="K23" s="119" t="n"/>
+      <c r="L23" s="119" t="n"/>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C24" s="124" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D24" s="125" t="inlineStr">
+        <is>
+          <t>Summative Skill Assessment Achievement Rate</t>
+        </is>
+      </c>
+      <c r="E24" s="124" t="inlineStr">
+        <is>
+          <t>Students scoring above the defined passing threshold in summative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
+        </is>
+      </c>
+      <c r="F24" s="124" t="inlineStr">
+        <is>
+          <t>direct → org KRA 1 — the summative achievement number itself (org scoreboard; the tracker reads it via module-quiz Bands + Alignment)</t>
+        </is>
+      </c>
+      <c r="G24" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H24" s="123" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I24" s="123" t="n"/>
+      <c r="J24" s="123" t="n"/>
+      <c r="K24" s="126">
+        <f>IF(AND(ISNUMBER(I24),ISNUMBER(J24)),I24-J24,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="124" t="inlineStr">
+        <is>
+          <t>Q1 ref: B 35 (quarterly) · default threshold 70%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="123" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C25" s="124" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D25" s="125" t="inlineStr">
+        <is>
+          <t>Formative Skill Assessment Achievement Rate</t>
+        </is>
+      </c>
+      <c r="E25" s="124" t="inlineStr">
+        <is>
+          <t>Students scoring above the defined passing threshold in formative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
+        </is>
+      </c>
+      <c r="F25" s="124" t="inlineStr">
+        <is>
+          <t>enabling → Summative SA Achievement (row above) + tracker Content–Assessment Alignment — the early-warning formative read</t>
+        </is>
+      </c>
+      <c r="G25" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H25" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I25" s="123" t="n"/>
+      <c r="J25" s="123" t="n"/>
+      <c r="K25" s="126">
+        <f>IF(AND(ISNUMBER(I25),ISNUMBER(J25)),I25-J25,"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 23 · A 33.4 — 75% cap used as the Skill Assessments cut-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="123" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C26" s="124" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D26" s="125" t="inlineStr">
+        <is>
+          <t>Graded Assessment Achievement Rate (NIAT)</t>
+        </is>
+      </c>
+      <c r="E26" s="124" t="inlineStr">
+        <is>
+          <t>Students scoring above the defined passing threshold in university-conducted graded assessments — Mid-1, Mid-2 and End Semester exams — delivered in collaboration with the university.</t>
+        </is>
+      </c>
+      <c r="F26" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Business Impact (§5) — university-conducted exams: NIAT SPI &amp; university trust</t>
+        </is>
+      </c>
+      <c r="G26" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H26" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I26" s="123" t="n"/>
+      <c r="J26" s="123" t="n"/>
+      <c r="K26" s="126">
+        <f>IF(AND(ISNUMBER(I26),ISNUMBER(J26)),I26-J26,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="124" t="inlineStr"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="123" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C27" s="124" t="inlineStr">
+        <is>
+          <t>Business Impact</t>
+        </is>
+      </c>
+      <c r="D27" s="125" t="inlineStr">
+        <is>
+          <t>Weekly Active Users (Launchpad)</t>
+        </is>
+      </c>
+      <c r="E27" s="124" t="inlineStr">
+        <is>
+          <t>Total prospective learner leads generated in the period through content-driven channels (organic, referral, campaigns, partnerships).</t>
+        </is>
+      </c>
+      <c r="F27" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Business Impact (§5) — Launchpad top-of-funnel</t>
+        </is>
+      </c>
+      <c r="G27" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H27" s="123" t="inlineStr">
+        <is>
+          <t>Monthly (wkly avg)</t>
+        </is>
+      </c>
+      <c r="I27" s="123" t="n"/>
+      <c r="J27" s="123" t="n"/>
+      <c r="K27" s="126">
+        <f>IF(AND(ISNUMBER(I27),ISNUMBER(J27)),I27-J27,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="124" t="inlineStr"/>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="123" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C28" s="124" t="inlineStr">
+        <is>
+          <t>Content Effectiveness</t>
+        </is>
+      </c>
+      <c r="D28" s="125" t="inlineStr">
+        <is>
+          <t>Learning Engagement Effort (LE)</t>
+        </is>
+      </c>
+      <c r="E28" s="124" t="inlineStr">
+        <is>
+          <t>How much a learner meaningfully engages with learning material, adjusted for effort intensity and persistence. Passive time (video, cheatsheets) weighted at 0.5.</t>
+        </is>
+      </c>
+      <c r="F28" s="124" t="inlineStr">
+        <is>
+          <t>enabling → tracker Engagement-Matrix Cell Migration — LE is the effort axis of the matrix</t>
+        </is>
+      </c>
+      <c r="G28" s="123" t="inlineStr">
+        <is>
+          <t>Min (wtd)</t>
+        </is>
+      </c>
+      <c r="H28" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I28" s="123" t="n"/>
+      <c r="J28" s="123" t="n"/>
+      <c r="K28" s="126">
+        <f>IF(AND(ISNUMBER(I28),ISNUMBER(J28)),I28-J28,"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="124" t="inlineStr"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="123" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C29" s="124" t="inlineStr">
+        <is>
+          <t>Content Effectiveness</t>
+        </is>
+      </c>
+      <c r="D29" s="125" t="inlineStr">
+        <is>
+          <t>Course Completion Rate</t>
+        </is>
+      </c>
+      <c r="E29" s="124" t="inlineStr">
+        <is>
+          <t>% of enrolled learners who complete a course in full. Encompasses all unit types — video, practice, projects and assessments.</t>
+        </is>
+      </c>
+      <c r="F29" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Effectiveness (§5)</t>
+        </is>
+      </c>
+      <c r="G29" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H29" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I29" s="123" t="n"/>
+      <c r="J29" s="123" t="n"/>
+      <c r="K29" s="126">
+        <f>IF(AND(ISNUMBER(I29),ISNUMBER(J29)),I29-J29,"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="124" t="inlineStr"/>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="123" t="n">
+        <v>7</v>
+      </c>
+      <c r="B30" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C30" s="124" t="inlineStr">
+        <is>
+          <t>Content Effectiveness</t>
+        </is>
+      </c>
+      <c r="D30" s="125" t="inlineStr">
+        <is>
+          <t>Pedagogy Initiative Impact</t>
+        </is>
+      </c>
+      <c r="E30" s="124" t="inlineStr">
+        <is>
+          <t>Implemented pedagogy initiatives with measurable learning-outcome improvement. Outcome baseline must be defined and agreed before the initiative is launched.</t>
+        </is>
+      </c>
+      <c r="F30" s="124" t="inlineStr">
+        <is>
+          <t>enabling → LE + module-quiz Bands — pedagogy initiatives move the learning numbers</t>
+        </is>
+      </c>
+      <c r="G30" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H30" s="123" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I30" s="123" t="n"/>
+      <c r="J30" s="123" t="n"/>
+      <c r="K30" s="126">
+        <f>IF(AND(ISNUMBER(I30),ISNUMBER(J30)),I30-J30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="124" t="inlineStr"/>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="123" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C31" s="124" t="inlineStr">
+        <is>
+          <t>Content Effectiveness</t>
+        </is>
+      </c>
+      <c r="D31" s="125" t="inlineStr">
+        <is>
+          <t>Learner Accessed Content Completion Rate</t>
+        </is>
+      </c>
+      <c r="E31" s="124" t="inlineStr">
+        <is>
+          <t>Video units: for each learner, % of video units they opened that they also completed; averaged across learners. Excludes units with zero opens.</t>
+        </is>
+      </c>
+      <c r="F31" s="124" t="inlineStr">
+        <is>
+          <t>enabling → Course Completion Rate — the video-unit leg</t>
+        </is>
+      </c>
+      <c r="G31" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H31" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I31" s="123" t="n"/>
+      <c r="J31" s="123" t="n"/>
+      <c r="K31" s="126">
+        <f>IF(AND(ISNUMBER(I31),ISNUMBER(J31)),I31-J31,"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="124" t="inlineStr"/>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="123" t="n">
+        <v>9</v>
+      </c>
+      <c r="B32" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C32" s="124" t="inlineStr">
+        <is>
+          <t>Content Effectiveness</t>
+        </is>
+      </c>
+      <c r="D32" s="125" t="inlineStr">
+        <is>
+          <t>Practice Attempt-to-Completion Rate</t>
+        </is>
+      </c>
+      <c r="E32" s="124" t="inlineStr">
+        <is>
+          <t>Practice units: for each learner, % of coding/project exercises attempted that they also completed. Surfaces environment friction (IDE, playground, cloud setup) vs difficulty-related drop-off.</t>
+        </is>
+      </c>
+      <c r="F32" s="124" t="inlineStr">
+        <is>
+          <t>enabling → tracker Journey Step Health steps 6–7 (practice return &amp; completion) + Learning Environment Satisfaction</t>
+        </is>
+      </c>
+      <c r="G32" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H32" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I32" s="123" t="n"/>
+      <c r="J32" s="123" t="n"/>
+      <c r="K32" s="126">
+        <f>IF(AND(ISNUMBER(I32),ISNUMBER(J32)),I32-J32,"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 38.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="123" t="n">
+        <v>10</v>
+      </c>
+      <c r="B33" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C33" s="124" t="inlineStr">
+        <is>
+          <t>Content Velocity</t>
+        </is>
+      </c>
+      <c r="D33" s="125" t="inlineStr">
+        <is>
+          <t>Learning Content Hours Delivered</t>
+        </is>
+      </c>
+      <c r="E33" s="124" t="inlineStr">
+        <is>
+          <t>Total learning content hours created per month across all formats (video, text, interactive). Content serving multiple products counted once.</t>
+        </is>
+      </c>
+      <c r="F33" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Velocity (§5) — capacity for B4 &amp; new stacks</t>
+        </is>
+      </c>
+      <c r="G33" s="123" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="H33" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I33" s="123" t="n"/>
+      <c r="J33" s="123" t="n"/>
+      <c r="K33" s="126">
+        <f>IF(AND(ISNUMBER(I33),ISNUMBER(J33)),I33-J33,"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 50 · A 46.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="58" customHeight="1">
+      <c r="A34" s="123" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C34" s="124" t="inlineStr">
+        <is>
+          <t>Content Velocity</t>
+        </is>
+      </c>
+      <c r="D34" s="125" t="inlineStr">
+        <is>
+          <t>Vernacular Content Hours Delivered</t>
+        </is>
+      </c>
+      <c r="E34" s="124" t="inlineStr">
+        <is>
+          <t>Total vernacular-language learning content hours created per month. Tracked separately from English hours — effort per vernacular hour differs significantly.</t>
+        </is>
+      </c>
+      <c r="F34" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Velocity (§5) — vernacular capacity</t>
+        </is>
+      </c>
+      <c r="G34" s="123" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="H34" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I34" s="123" t="n"/>
+      <c r="J34" s="123" t="n"/>
+      <c r="K34" s="126">
+        <f>IF(AND(ISNUMBER(I34),ISNUMBER(J34)),I34-J34,"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0 — no vernacular slate yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="123" t="n">
+        <v>12</v>
+      </c>
+      <c r="B35" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C35" s="124" t="inlineStr">
+        <is>
+          <t>Content Velocity</t>
+        </is>
+      </c>
+      <c r="D35" s="125" t="inlineStr">
+        <is>
+          <t>Practice &amp; Assessment Content Pieces Delivered</t>
+        </is>
+      </c>
+      <c r="E35" s="124" t="inlineStr">
+        <is>
+          <t>Total practice and assessment pieces delivered monthly across owned domains (MCQs, coding questions, projects, case studies).</t>
+        </is>
+      </c>
+      <c r="F35" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Velocity (§5) — practice depth behind Journey Step Health steps 5–7</t>
+        </is>
+      </c>
+      <c r="G35" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H35" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I35" s="123" t="n"/>
+      <c r="J35" s="123" t="n"/>
+      <c r="K35" s="126">
+        <f>IF(AND(ISNUMBER(I35),ISNUMBER(J35)),I35-J35,"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 1,600 · A 1,499 (Aug B: 1,000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="123" t="n">
+        <v>13</v>
+      </c>
+      <c r="B36" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C36" s="124" t="inlineStr">
+        <is>
+          <t>Content Velocity</t>
+        </is>
+      </c>
+      <c r="D36" s="125" t="inlineStr">
+        <is>
+          <t>Branding Content Assets Delivered</t>
+        </is>
+      </c>
+      <c r="E36" s="124" t="inlineStr">
+        <is>
+          <t>Total branded content pieces produced monthly (thumbnails, banners, promo assets).</t>
+        </is>
+      </c>
+      <c r="F36" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Velocity (§5)</t>
+        </is>
+      </c>
+      <c r="G36" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H36" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I36" s="123" t="n"/>
+      <c r="J36" s="123" t="n"/>
+      <c r="K36" s="126">
+        <f>IF(AND(ISNUMBER(I36),ISNUMBER(J36)),I36-J36,"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="58" customHeight="1">
+      <c r="A37" s="123" t="n">
+        <v>14</v>
+      </c>
+      <c r="B37" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C37" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D37" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Learning Hour Produced</t>
+        </is>
+      </c>
+      <c r="E37" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to produce one hour of learning content. Includes people, tools and infra involved in creation. Tracks creation efficiency — not delivery cost.</t>
+        </is>
+      </c>
+      <c r="F37" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per Learning Hour (§5 Content Efficiency)</t>
+        </is>
+      </c>
+      <c r="G37" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H37" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I37" s="123" t="n"/>
+      <c r="J37" s="123" t="n"/>
+      <c r="K37" s="126">
+        <f>IF(AND(ISNUMBER(I37),ISNUMBER(J37)),I37-J37,"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B ₹10,000 · A ₹6,803 — 46 h across 4 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="58" customHeight="1">
+      <c r="A38" s="123" t="n">
+        <v>15</v>
+      </c>
+      <c r="B38" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C38" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D38" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Vernacular Content Hour</t>
+        </is>
+      </c>
+      <c r="E38" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to produce one hour of vernacular-language content. Includes team bandwidth involved in creation (contract basis, tools &amp; infrastructure).</t>
+        </is>
+      </c>
+      <c r="F38" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per Vernacular Content Hour (§5) — production-side twin of CSI's central track</t>
+        </is>
+      </c>
+      <c r="G38" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H38" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I38" s="123" t="n"/>
+      <c r="J38" s="123" t="n"/>
+      <c r="K38" s="126">
+        <f>IF(AND(ISNUMBER(I38),ISNUMBER(J38)),I38-J38,"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="123" t="n">
+        <v>16</v>
+      </c>
+      <c r="B39" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C39" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D39" s="125" t="inlineStr">
+        <is>
+          <t>Cost per MCQ Generated</t>
+        </is>
+      </c>
+      <c r="E39" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to develop one objective question, including both manual and AI-assisted production.</t>
+        </is>
+      </c>
+      <c r="F39" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per MCQ (§5 Content Efficiency)</t>
+        </is>
+      </c>
+      <c r="G39" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H39" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I39" s="123" t="n"/>
+      <c r="J39" s="123" t="n"/>
+      <c r="K39" s="126">
+        <f>IF(AND(ISNUMBER(I39),ISNUMBER(J39)),I39-J39,"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B ₹40 · A ₹26 — 1,347 MCQs across 2 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="123" t="n">
+        <v>17</v>
+      </c>
+      <c r="B40" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C40" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D40" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Coding Question</t>
+        </is>
+      </c>
+      <c r="E40" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to develop one coding question, including test-case design and evaluation-engine configuration.</t>
+        </is>
+      </c>
+      <c r="F40" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per Coding Question (§5 Content Efficiency)</t>
+        </is>
+      </c>
+      <c r="G40" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H40" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I40" s="123" t="n"/>
+      <c r="J40" s="123" t="n"/>
+      <c r="K40" s="126">
+        <f>IF(AND(ISNUMBER(I40),ISNUMBER(J40)),I40-J40,"")</f>
+        <v/>
+      </c>
+      <c r="L40" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B ₹400 · A ₹163 — 131 coding questions across 3 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="123" t="n">
+        <v>18</v>
+      </c>
+      <c r="B41" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C41" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D41" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Branding Content Asset</t>
+        </is>
+      </c>
+      <c r="E41" s="124" t="inlineStr">
+        <is>
+          <t>Average cost to create one branded content piece.</t>
+        </is>
+      </c>
+      <c r="F41" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Cost per Branding Asset (§5 Content Efficiency)</t>
+        </is>
+      </c>
+      <c r="G41" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H41" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I41" s="123" t="n"/>
+      <c r="J41" s="123" t="n"/>
+      <c r="K41" s="126">
+        <f>IF(AND(ISNUMBER(I41),ISNUMBER(J41)),I41-J41,"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="58" customHeight="1">
+      <c r="A42" s="123" t="n">
+        <v>19</v>
+      </c>
+      <c r="B42" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C42" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D42" s="125" t="inlineStr">
+        <is>
+          <t>Platform Runtime Cost per Active Learner</t>
+        </is>
+      </c>
+      <c r="E42" s="124" t="inlineStr">
+        <is>
+          <t>Total platform delivery costs (cloud compute, code-execution infra, cloud IDE hosting, GenAI API calls) divided by active learners in the period. Tracks delivery-cost efficiency as usage scales.</t>
+        </is>
+      </c>
+      <c r="F42" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Platform Runtime Cost per Active Learner (§5) — the team's share of delivery cost</t>
+        </is>
+      </c>
+      <c r="G42" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H42" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I42" s="123" t="n"/>
+      <c r="J42" s="123" t="n"/>
+      <c r="K42" s="126">
+        <f>IF(AND(ISNUMBER(I42),ISNUMBER(J42)),I42-J42,"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="124" t="inlineStr"/>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="123" t="n">
+        <v>20</v>
+      </c>
+      <c r="B43" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C43" s="124" t="inlineStr">
+        <is>
+          <t>Content Efficiency</t>
+        </is>
+      </c>
+      <c r="D43" s="125" t="inlineStr">
+        <is>
+          <t>R&amp;D Initiative Impact</t>
+        </is>
+      </c>
+      <c r="E43" s="124" t="inlineStr">
+        <is>
+          <t>Implemented R&amp;D initiatives — including adoption of agentic AI solutions and automation pipelines — with measurable content-production improvement.</t>
+        </is>
+      </c>
+      <c r="F43" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept R&amp;D Initiative Impact + Agentic Production Coverage (§5)</t>
+        </is>
+      </c>
+      <c r="G43" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H43" s="123" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I43" s="123" t="n"/>
+      <c r="J43" s="123" t="n"/>
+      <c r="K43" s="126">
+        <f>IF(AND(ISNUMBER(I43),ISNUMBER(J43)),I43-J43,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="58" customHeight="1">
+      <c r="A44" s="123" t="n">
+        <v>21</v>
+      </c>
+      <c r="B44" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C44" s="124" t="inlineStr">
+        <is>
+          <t>Content Relevance</t>
+        </is>
+      </c>
+      <c r="D44" s="125" t="inlineStr">
+        <is>
+          <t>Tech Stack Freshness Rate</t>
+        </is>
+      </c>
+      <c r="E44" s="124" t="inlineStr">
+        <is>
+          <t>% of tools, frameworks, libraries and environments referenced in content (and configured in IDEs, playgrounds, cloud setups) matching the current stable or LTS version at audit.</t>
+        </is>
+      </c>
+      <c r="F44" s="124" t="inlineStr">
+        <is>
+          <t>enabling → tracker Industry Update Adherence — the freshness audit behind relevance</t>
+        </is>
+      </c>
+      <c r="G44" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H44" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I44" s="123" t="n"/>
+      <c r="J44" s="123" t="n"/>
+      <c r="K44" s="126">
+        <f>IF(AND(ISNUMBER(I44),ISNUMBER(J44)),I44-J44,"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 100 · A 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="123" t="n">
+        <v>22</v>
+      </c>
+      <c r="B45" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C45" s="124" t="inlineStr">
+        <is>
+          <t>Stakeholder Alignment</t>
+        </is>
+      </c>
+      <c r="D45" s="125" t="inlineStr">
+        <is>
+          <t>Stakeholder Content Request Fulfillment Rate</t>
+        </is>
+      </c>
+      <c r="E45" s="124" t="inlineStr">
+        <is>
+          <t>Requests from Sales, Placements, Program Ops, Assessments and Instructors fulfilled within agreed timeframes across all products.</t>
+        </is>
+      </c>
+      <c r="F45" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Stakeholder Alignment (§5)</t>
+        </is>
+      </c>
+      <c r="G45" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H45" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I45" s="123" t="n"/>
+      <c r="J45" s="123" t="n"/>
+      <c r="K45" s="126">
+        <f>IF(AND(ISNUMBER(I45),ISNUMBER(J45)),I45-J45,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 90 · A 90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="58" customHeight="1">
+      <c r="A46" s="123" t="n">
+        <v>23</v>
+      </c>
+      <c r="B46" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C46" s="124" t="inlineStr">
+        <is>
+          <t>Stakeholder Alignment</t>
+        </is>
+      </c>
+      <c r="D46" s="125" t="inlineStr">
+        <is>
+          <t>Cross-functional Sprint Delivery Rate</t>
+        </is>
+      </c>
+      <c r="E46" s="124" t="inlineStr">
+        <is>
+          <t>% of committed tickets across Product, Pedagogy, Engineering, UI/UX and DA/DE — scoped and approved by this team — delivered within the committed sprint.</t>
+        </is>
+      </c>
+      <c r="F46" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Stakeholder Alignment (§5)</t>
+        </is>
+      </c>
+      <c r="G46" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H46" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I46" s="123" t="n"/>
+      <c r="J46" s="123" t="n"/>
+      <c r="K46" s="126">
+        <f>IF(AND(ISNUMBER(I46),ISNUMBER(J46)),I46-J46,"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 100 · A 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1">
+      <c r="A47" s="123" t="n">
+        <v>24</v>
+      </c>
+      <c r="B47" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C47" s="124" t="inlineStr">
+        <is>
+          <t>Executive Ops</t>
+        </is>
+      </c>
+      <c r="D47" s="125" t="inlineStr">
+        <is>
+          <t>Operations &amp; Growth Cost</t>
+        </is>
+      </c>
+      <c r="E47" s="124" t="inlineStr">
+        <is>
+          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+        </is>
+      </c>
+      <c r="F47" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="G47" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H47" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I47" s="123" t="n"/>
+      <c r="J47" s="123" t="n"/>
+      <c r="K47" s="126">
+        <f>IF(AND(ISNUMBER(I47),ISNUMBER(J47)),I47-J47,"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: A ₹300,863.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="58" customHeight="1">
+      <c r="A48" s="123" t="n">
+        <v>25</v>
+      </c>
+      <c r="B48" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C48" s="124" t="inlineStr">
+        <is>
+          <t>Executive Ops</t>
+        </is>
+      </c>
+      <c r="D48" s="125" t="inlineStr">
+        <is>
+          <t>Creative Resource Utilisation Rate</t>
+        </is>
+      </c>
+      <c r="E48" s="124" t="inlineStr">
+        <is>
+          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
+        </is>
+      </c>
+      <c r="F48" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
+        </is>
+      </c>
+      <c r="G48" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H48" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I48" s="123" t="n"/>
+      <c r="J48" s="123" t="n"/>
+      <c r="K48" s="126">
+        <f>IF(AND(ISNUMBER(I48),ISNUMBER(J48)),I48-J48,"")</f>
+        <v/>
+      </c>
+      <c r="L48" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: A 100% — fully utilised, at times stretched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="129" t="inlineStr">
+        <is>
+          <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
+        </is>
+      </c>
+      <c r="B49" s="119" t="n"/>
+      <c r="C49" s="119" t="n"/>
+      <c r="D49" s="119" t="n"/>
+      <c r="E49" s="119" t="n"/>
+      <c r="F49" s="119" t="n"/>
+      <c r="G49" s="119" t="n"/>
+      <c r="H49" s="119" t="n"/>
+      <c r="I49" s="119" t="n"/>
+      <c r="J49" s="119" t="n"/>
+      <c r="K49" s="119" t="n"/>
+      <c r="L49" s="119" t="n"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C50" s="131" t="inlineStr">
+        <is>
+          <t>Assessments team</t>
+        </is>
+      </c>
+      <c r="D50" s="132" t="inlineStr">
+        <is>
+          <t>Assessment blueprints per cycle</t>
+        </is>
+      </c>
+      <c r="E50" s="131" t="inlineStr">
+        <is>
+          <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
+        </is>
+      </c>
+      <c r="F50" s="131" t="n"/>
+      <c r="G50" s="130" t="n"/>
+      <c r="H50" s="130" t="n"/>
+      <c r="I50" s="130" t="n"/>
+      <c r="J50" s="130" t="n"/>
+      <c r="K50" s="130" t="n"/>
+      <c r="L50" s="131" t="n"/>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="130" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C51" s="131" t="inlineStr">
+        <is>
+          <t>Learning Platform / DA-DEs</t>
+        </is>
+      </c>
+      <c r="D51" s="132" t="inlineStr">
+        <is>
+          <t>Engagement &amp; LE dashboards</t>
+        </is>
+      </c>
+      <c r="E51" s="131" t="inlineStr">
+        <is>
+          <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here.</t>
+        </is>
+      </c>
+      <c r="F51" s="131" t="n"/>
+      <c r="G51" s="130" t="n"/>
+      <c r="H51" s="130" t="n"/>
+      <c r="I51" s="130" t="n"/>
+      <c r="J51" s="130" t="n"/>
+      <c r="K51" s="130" t="n"/>
+      <c r="L51" s="131" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="130" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C52" s="131" t="inlineStr">
+        <is>
+          <t>Instructors dept + Program Ops</t>
+        </is>
+      </c>
+      <c r="D52" s="132" t="inlineStr">
+        <is>
+          <t>Classroom signal loop</t>
+        </is>
+      </c>
+      <c r="E52" s="131" t="inlineStr">
+        <is>
+          <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
+        </is>
+      </c>
+      <c r="F52" s="131" t="n"/>
+      <c r="G52" s="130" t="n"/>
+      <c r="H52" s="130" t="n"/>
+      <c r="I52" s="130" t="n"/>
+      <c r="J52" s="130" t="n"/>
+      <c r="K52" s="130" t="n"/>
+      <c r="L52" s="131" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="E50:L50"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="E51:L51"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="E52:L52"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
FS Section B rulings: retire LE + Course Completion rows, pin PII to domain SME
LE = effort axis of the engagement matrix, not a budgeted KPI (already
inside Cell Migration). Course Completion = conduction-driven, demoted to
read-only cut in the dashboards ask. PII stays SME-owned with Pedagogy
Experts contributing; PII + LACCR ladders re-pointed off the retired rows.
FS view now A 18 / B 23 / C 3.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -5156,7 +5156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6661,27 +6661,27 @@
       </c>
       <c r="F28" s="125" t="inlineStr">
         <is>
-          <t>Learning Engagement Effort (LE)</t>
+          <t>Pedagogy Initiative Impact</t>
         </is>
       </c>
       <c r="G28" s="124" t="inlineStr">
         <is>
-          <t>How much a learner meaningfully engages with learning material, adjusted for effort intensity and persistence. Passive time (video, cheatsheets) weighted at 0.5.</t>
+          <t>Implemented pedagogy initiatives with measurable learning-outcome improvement. Outcome baseline must be defined and agreed before the initiative is launched.</t>
         </is>
       </c>
       <c r="H28" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Engagement-Matrix Cell Migration — LE is the effort axis of the matrix</t>
+          <t>enabling → module-quiz Bands + org KRA 2 Academics CSAT — pedagogy initiatives move the learning numbers</t>
         </is>
       </c>
       <c r="I28" s="123" t="inlineStr">
         <is>
-          <t>Min (wtd)</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J28" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K28" s="123" t="n"/>
@@ -6690,7 +6690,11 @@
         <f>IF(AND(ISNUMBER(K28),ISNUMBER(L28)),K28-L28,"")</f>
         <v/>
       </c>
-      <c r="N28" s="124" t="inlineStr"/>
+      <c r="N28" s="124" t="inlineStr">
+        <is>
+          <t>Owned by the domain SME on this team; embedded Pedagogy Experts contribute to the initiatives.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="123" t="n">
@@ -6718,17 +6722,17 @@
       </c>
       <c r="F29" s="125" t="inlineStr">
         <is>
-          <t>Course Completion Rate</t>
+          <t>Learner Accessed Content Completion Rate</t>
         </is>
       </c>
       <c r="G29" s="124" t="inlineStr">
         <is>
-          <t>% of enrolled learners who complete a course in full. Encompasses all unit types — video, practice, projects and assessments.</t>
+          <t>Video units: for each learner, % of video units they opened that they also completed; averaged across learners. Excludes units with zero opens.</t>
         </is>
       </c>
       <c r="H29" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Effectiveness (§5)</t>
+          <t>enabling → tracker Engagement-Matrix Cell Migration — video-stickiness leg of the value axis; access-conditioned, so conduction effects are stripped</t>
         </is>
       </c>
       <c r="I29" s="123" t="inlineStr">
@@ -6775,27 +6779,27 @@
       </c>
       <c r="F30" s="125" t="inlineStr">
         <is>
-          <t>Pedagogy Initiative Impact</t>
+          <t>Practice Attempt-to-Completion Rate</t>
         </is>
       </c>
       <c r="G30" s="124" t="inlineStr">
         <is>
-          <t>Implemented pedagogy initiatives with measurable learning-outcome improvement. Outcome baseline must be defined and agreed before the initiative is launched.</t>
+          <t>Practice units: for each learner, % of coding/project exercises attempted that they also completed. Surfaces environment friction (IDE, playground, cloud setup) vs difficulty-related drop-off.</t>
         </is>
       </c>
       <c r="H30" s="124" t="inlineStr">
         <is>
-          <t>enabling → LE + module-quiz Bands — pedagogy initiatives move the learning numbers</t>
+          <t>enabling → tracker Journey Step Health steps 6–7 (practice return &amp; completion) + Learning Environment Satisfaction</t>
         </is>
       </c>
       <c r="I30" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J30" s="123" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K30" s="123" t="n"/>
@@ -6804,7 +6808,11 @@
         <f>IF(AND(ISNUMBER(K30),ISNUMBER(L30)),K30-L30,"")</f>
         <v/>
       </c>
-      <c r="N30" s="124" t="inlineStr"/>
+      <c r="N30" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 38.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="123" t="n">
@@ -6817,7 +6825,7 @@
       </c>
       <c r="C31" s="124" t="inlineStr">
         <is>
-          <t>Content Effectiveness</t>
+          <t>Content Velocity</t>
         </is>
       </c>
       <c r="D31" s="123" t="inlineStr">
@@ -6832,22 +6840,22 @@
       </c>
       <c r="F31" s="125" t="inlineStr">
         <is>
-          <t>Learner Accessed Content Completion Rate</t>
+          <t>Learning Content Hours Delivered</t>
         </is>
       </c>
       <c r="G31" s="124" t="inlineStr">
         <is>
-          <t>Video units: for each learner, % of video units they opened that they also completed; averaged across learners. Excludes units with zero opens.</t>
+          <t>Total learning content hours created per month across all formats (video, text, interactive). Content serving multiple products counted once.</t>
         </is>
       </c>
       <c r="H31" s="124" t="inlineStr">
         <is>
-          <t>enabling → Course Completion Rate — the video-unit leg</t>
+          <t>enabling → dept Content Velocity (§5) — capacity for B4 &amp; new stacks</t>
         </is>
       </c>
       <c r="I31" s="123" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="J31" s="123" t="inlineStr">
@@ -6861,7 +6869,11 @@
         <f>IF(AND(ISNUMBER(K31),ISNUMBER(L31)),K31-L31,"")</f>
         <v/>
       </c>
-      <c r="N31" s="124" t="inlineStr"/>
+      <c r="N31" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 50 · A 46.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="58" customHeight="1">
       <c r="A32" s="123" t="n">
@@ -6874,7 +6886,7 @@
       </c>
       <c r="C32" s="124" t="inlineStr">
         <is>
-          <t>Content Effectiveness</t>
+          <t>Content Velocity</t>
         </is>
       </c>
       <c r="D32" s="123" t="inlineStr">
@@ -6889,22 +6901,22 @@
       </c>
       <c r="F32" s="125" t="inlineStr">
         <is>
-          <t>Practice Attempt-to-Completion Rate</t>
+          <t>Vernacular Content Hours Delivered</t>
         </is>
       </c>
       <c r="G32" s="124" t="inlineStr">
         <is>
-          <t>Practice units: for each learner, % of coding/project exercises attempted that they also completed. Surfaces environment friction (IDE, playground, cloud setup) vs difficulty-related drop-off.</t>
+          <t>Total vernacular-language learning content hours created per month. Tracked separately from English hours — effort per vernacular hour differs significantly.</t>
         </is>
       </c>
       <c r="H32" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Journey Step Health steps 6–7 (practice return &amp; completion) + Learning Environment Satisfaction</t>
+          <t>enabling → dept Content Velocity (§5) — vernacular capacity</t>
         </is>
       </c>
       <c r="I32" s="123" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="J32" s="123" t="inlineStr">
@@ -6920,7 +6932,7 @@
       </c>
       <c r="N32" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 38.</t>
+          <t>Q1 Jul: B 0 — no vernacular slate yet.</t>
         </is>
       </c>
     </row>
@@ -6950,22 +6962,22 @@
       </c>
       <c r="F33" s="125" t="inlineStr">
         <is>
-          <t>Learning Content Hours Delivered</t>
+          <t>Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
       </c>
       <c r="G33" s="124" t="inlineStr">
         <is>
-          <t>Total learning content hours created per month across all formats (video, text, interactive). Content serving multiple products counted once.</t>
+          <t>Total practice and assessment pieces delivered monthly across owned domains (MCQs, coding questions, projects, case studies).</t>
         </is>
       </c>
       <c r="H33" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — capacity for B4 &amp; new stacks</t>
+          <t>enabling → dept Content Velocity (§5) — practice depth behind Journey Step Health steps 5–7</t>
         </is>
       </c>
       <c r="I33" s="123" t="inlineStr">
         <is>
-          <t>Hours</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J33" s="123" t="inlineStr">
@@ -6981,11 +6993,11 @@
       </c>
       <c r="N33" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 50 · A 46.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="58" customHeight="1">
+          <t>Q1 Jul: B 1,600 · A 1,499 (Aug B: 1,000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="123" t="n">
         <v>11</v>
       </c>
@@ -7011,22 +7023,22 @@
       </c>
       <c r="F34" s="125" t="inlineStr">
         <is>
-          <t>Vernacular Content Hours Delivered</t>
+          <t>Branding Content Assets Delivered</t>
         </is>
       </c>
       <c r="G34" s="124" t="inlineStr">
         <is>
-          <t>Total vernacular-language learning content hours created per month. Tracked separately from English hours — effort per vernacular hour differs significantly.</t>
+          <t>Total branded content pieces produced monthly (thumbnails, banners, promo assets).</t>
         </is>
       </c>
       <c r="H34" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — vernacular capacity</t>
+          <t>enabling → dept Content Velocity (§5)</t>
         </is>
       </c>
       <c r="I34" s="123" t="inlineStr">
         <is>
-          <t>Hours</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J34" s="123" t="inlineStr">
@@ -7042,11 +7054,11 @@
       </c>
       <c r="N34" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 — no vernacular slate yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="45" customHeight="1">
+          <t>Q1 Jul: B 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="58" customHeight="1">
       <c r="A35" s="123" t="n">
         <v>12</v>
       </c>
@@ -7057,7 +7069,7 @@
       </c>
       <c r="C35" s="124" t="inlineStr">
         <is>
-          <t>Content Velocity</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D35" s="123" t="inlineStr">
@@ -7072,22 +7084,22 @@
       </c>
       <c r="F35" s="125" t="inlineStr">
         <is>
-          <t>Practice &amp; Assessment Content Pieces Delivered</t>
+          <t>Cost per Learning Hour Produced</t>
         </is>
       </c>
       <c r="G35" s="124" t="inlineStr">
         <is>
-          <t>Total practice and assessment pieces delivered monthly across owned domains (MCQs, coding questions, projects, case studies).</t>
+          <t>Average cost to produce one hour of learning content. Includes people, tools and infra involved in creation. Tracks creation efficiency — not delivery cost.</t>
         </is>
       </c>
       <c r="H35" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — practice depth behind Journey Step Health steps 5–7</t>
+          <t>enabling → dept Cost per Learning Hour (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I35" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="J35" s="123" t="inlineStr">
@@ -7103,11 +7115,11 @@
       </c>
       <c r="N35" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 1,600 · A 1,499 (Aug B: 1,000).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="32" customHeight="1">
+          <t>Q1 Jul: B ₹10,000 · A ₹6,803 — 46 h across 4 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="58" customHeight="1">
       <c r="A36" s="123" t="n">
         <v>13</v>
       </c>
@@ -7118,7 +7130,7 @@
       </c>
       <c r="C36" s="124" t="inlineStr">
         <is>
-          <t>Content Velocity</t>
+          <t>Content Efficiency</t>
         </is>
       </c>
       <c r="D36" s="123" t="inlineStr">
@@ -7133,22 +7145,22 @@
       </c>
       <c r="F36" s="125" t="inlineStr">
         <is>
-          <t>Branding Content Assets Delivered</t>
+          <t>Cost per Vernacular Content Hour</t>
         </is>
       </c>
       <c r="G36" s="124" t="inlineStr">
         <is>
-          <t>Total branded content pieces produced monthly (thumbnails, banners, promo assets).</t>
+          <t>Average cost to produce one hour of vernacular-language content. Includes team bandwidth involved in creation (contract basis, tools &amp; infrastructure).</t>
         </is>
       </c>
       <c r="H36" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5)</t>
+          <t>enabling → dept Cost per Vernacular Content Hour (§5) — production-side twin of CSI's central track</t>
         </is>
       </c>
       <c r="I36" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="J36" s="123" t="inlineStr">
@@ -7164,11 +7176,11 @@
       </c>
       <c r="N36" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="58" customHeight="1">
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="123" t="n">
         <v>14</v>
       </c>
@@ -7194,17 +7206,17 @@
       </c>
       <c r="F37" s="125" t="inlineStr">
         <is>
-          <t>Cost per Learning Hour Produced</t>
+          <t>Cost per MCQ Generated</t>
         </is>
       </c>
       <c r="G37" s="124" t="inlineStr">
         <is>
-          <t>Average cost to produce one hour of learning content. Includes people, tools and infra involved in creation. Tracks creation efficiency — not delivery cost.</t>
+          <t>Average cost to develop one objective question, including both manual and AI-assisted production.</t>
         </is>
       </c>
       <c r="H37" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Learning Hour (§5 Content Efficiency)</t>
+          <t>enabling → dept Cost per MCQ (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I37" s="123" t="inlineStr">
@@ -7225,11 +7237,11 @@
       </c>
       <c r="N37" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B ₹10,000 · A ₹6,803 — 46 h across 4 products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="58" customHeight="1">
+          <t>Q1 Jul: B ₹40 · A ₹26 — 1,347 MCQs across 2 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
       <c r="A38" s="123" t="n">
         <v>15</v>
       </c>
@@ -7255,17 +7267,17 @@
       </c>
       <c r="F38" s="125" t="inlineStr">
         <is>
-          <t>Cost per Vernacular Content Hour</t>
+          <t>Cost per Coding Question</t>
         </is>
       </c>
       <c r="G38" s="124" t="inlineStr">
         <is>
-          <t>Average cost to produce one hour of vernacular-language content. Includes team bandwidth involved in creation (contract basis, tools &amp; infrastructure).</t>
+          <t>Average cost to develop one coding question, including test-case design and evaluation-engine configuration.</t>
         </is>
       </c>
       <c r="H38" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Vernacular Content Hour (§5) — production-side twin of CSI's central track</t>
+          <t>enabling → dept Cost per Coding Question (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I38" s="123" t="inlineStr">
@@ -7286,7 +7298,7 @@
       </c>
       <c r="N38" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 · A 0.</t>
+          <t>Q1 Jul: B ₹400 · A ₹163 — 131 coding questions across 3 products.</t>
         </is>
       </c>
     </row>
@@ -7316,17 +7328,17 @@
       </c>
       <c r="F39" s="125" t="inlineStr">
         <is>
-          <t>Cost per MCQ Generated</t>
+          <t>Cost per Branding Content Asset</t>
         </is>
       </c>
       <c r="G39" s="124" t="inlineStr">
         <is>
-          <t>Average cost to develop one objective question, including both manual and AI-assisted production.</t>
+          <t>Average cost to create one branded content piece.</t>
         </is>
       </c>
       <c r="H39" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per MCQ (§5 Content Efficiency)</t>
+          <t>enabling → dept Cost per Branding Asset (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I39" s="123" t="inlineStr">
@@ -7347,11 +7359,11 @@
       </c>
       <c r="N39" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B ₹40 · A ₹26 — 1,347 MCQs across 2 products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="45" customHeight="1">
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="58" customHeight="1">
       <c r="A40" s="123" t="n">
         <v>17</v>
       </c>
@@ -7377,17 +7389,17 @@
       </c>
       <c r="F40" s="125" t="inlineStr">
         <is>
-          <t>Cost per Coding Question</t>
+          <t>Platform Runtime Cost per Active Learner</t>
         </is>
       </c>
       <c r="G40" s="124" t="inlineStr">
         <is>
-          <t>Average cost to develop one coding question, including test-case design and evaluation-engine configuration.</t>
+          <t>Total platform delivery costs (cloud compute, code-execution infra, cloud IDE hosting, GenAI API calls) divided by active learners in the period. Tracks delivery-cost efficiency as usage scales.</t>
         </is>
       </c>
       <c r="H40" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Coding Question (§5 Content Efficiency)</t>
+          <t>enabling → dept Platform Runtime Cost per Active Learner (§5) — the team's share of delivery cost</t>
         </is>
       </c>
       <c r="I40" s="123" t="inlineStr">
@@ -7406,13 +7418,9 @@
         <f>IF(AND(ISNUMBER(K40),ISNUMBER(L40)),K40-L40,"")</f>
         <v/>
       </c>
-      <c r="N40" s="124" t="inlineStr">
-        <is>
-          <t>Q1 Jul: B ₹400 · A ₹163 — 131 coding questions across 3 products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="32" customHeight="1">
+      <c r="N40" s="124" t="inlineStr"/>
+    </row>
+    <row r="41" ht="45" customHeight="1">
       <c r="A41" s="123" t="n">
         <v>18</v>
       </c>
@@ -7438,27 +7446,27 @@
       </c>
       <c r="F41" s="125" t="inlineStr">
         <is>
-          <t>Cost per Branding Content Asset</t>
+          <t>R&amp;D Initiative Impact</t>
         </is>
       </c>
       <c r="G41" s="124" t="inlineStr">
         <is>
-          <t>Average cost to create one branded content piece.</t>
+          <t>Implemented R&amp;D initiatives — including adoption of agentic AI solutions and automation pipelines — with measurable content-production improvement.</t>
         </is>
       </c>
       <c r="H41" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Branding Asset (§5 Content Efficiency)</t>
+          <t>enabling → dept R&amp;D Initiative Impact (§5) + tracker row Agentic Production Coverage</t>
         </is>
       </c>
       <c r="I41" s="123" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J41" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K41" s="123" t="n"/>
@@ -7484,7 +7492,7 @@
       </c>
       <c r="C42" s="124" t="inlineStr">
         <is>
-          <t>Content Efficiency</t>
+          <t>Content Relevance</t>
         </is>
       </c>
       <c r="D42" s="123" t="inlineStr">
@@ -7499,22 +7507,22 @@
       </c>
       <c r="F42" s="125" t="inlineStr">
         <is>
-          <t>Platform Runtime Cost per Active Learner</t>
+          <t>Tech Stack Freshness Rate</t>
         </is>
       </c>
       <c r="G42" s="124" t="inlineStr">
         <is>
-          <t>Total platform delivery costs (cloud compute, code-execution infra, cloud IDE hosting, GenAI API calls) divided by active learners in the period. Tracks delivery-cost efficiency as usage scales.</t>
+          <t>% of tools, frameworks, libraries and environments referenced in content (and configured in IDEs, playgrounds, cloud setups) matching the current stable or LTS version at audit.</t>
         </is>
       </c>
       <c r="H42" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Platform Runtime Cost per Active Learner (§5) — the team's share of delivery cost</t>
+          <t>enabling → tracker Industry Update Adherence — the freshness audit behind relevance</t>
         </is>
       </c>
       <c r="I42" s="123" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J42" s="123" t="inlineStr">
@@ -7528,7 +7536,11 @@
         <f>IF(AND(ISNUMBER(K42),ISNUMBER(L42)),K42-L42,"")</f>
         <v/>
       </c>
-      <c r="N42" s="124" t="inlineStr"/>
+      <c r="N42" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 100 · A 100.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="123" t="n">
@@ -7541,7 +7553,7 @@
       </c>
       <c r="C43" s="124" t="inlineStr">
         <is>
-          <t>Content Efficiency</t>
+          <t>Stakeholder Alignment</t>
         </is>
       </c>
       <c r="D43" s="123" t="inlineStr">
@@ -7556,27 +7568,27 @@
       </c>
       <c r="F43" s="125" t="inlineStr">
         <is>
-          <t>R&amp;D Initiative Impact</t>
+          <t>Stakeholder Content Request Fulfillment Rate</t>
         </is>
       </c>
       <c r="G43" s="124" t="inlineStr">
         <is>
-          <t>Implemented R&amp;D initiatives — including adoption of agentic AI solutions and automation pipelines — with measurable content-production improvement.</t>
+          <t>Requests from Sales, Placements, Program Ops, Assessments and Instructors fulfilled within agreed timeframes across all products.</t>
         </is>
       </c>
       <c r="H43" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept R&amp;D Initiative Impact (§5) + tracker row Agentic Production Coverage</t>
+          <t>enabling → dept Stakeholder Alignment (§5)</t>
         </is>
       </c>
       <c r="I43" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J43" s="123" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K43" s="123" t="n"/>
@@ -7587,7 +7599,7 @@
       </c>
       <c r="N43" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 · A 0.</t>
+          <t>Q1 Jul: B 90 · A 90.</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7614,7 @@
       </c>
       <c r="C44" s="124" t="inlineStr">
         <is>
-          <t>Content Relevance</t>
+          <t>Stakeholder Alignment</t>
         </is>
       </c>
       <c r="D44" s="123" t="inlineStr">
@@ -7617,17 +7629,17 @@
       </c>
       <c r="F44" s="125" t="inlineStr">
         <is>
-          <t>Tech Stack Freshness Rate</t>
+          <t>Cross-functional Sprint Delivery Rate</t>
         </is>
       </c>
       <c r="G44" s="124" t="inlineStr">
         <is>
-          <t>% of tools, frameworks, libraries and environments referenced in content (and configured in IDEs, playgrounds, cloud setups) matching the current stable or LTS version at audit.</t>
+          <t>% of committed tickets across Product, Pedagogy, Engineering, UI/UX and DA/DE — scoped and approved by this team — delivered within the committed sprint.</t>
         </is>
       </c>
       <c r="H44" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Industry Update Adherence — the freshness audit behind relevance</t>
+          <t>enabling → dept Stakeholder Alignment (§5)</t>
         </is>
       </c>
       <c r="I44" s="123" t="inlineStr">
@@ -7663,7 +7675,7 @@
       </c>
       <c r="C45" s="124" t="inlineStr">
         <is>
-          <t>Stakeholder Alignment</t>
+          <t>Executive Ops</t>
         </is>
       </c>
       <c r="D45" s="123" t="inlineStr">
@@ -7678,22 +7690,22 @@
       </c>
       <c r="F45" s="125" t="inlineStr">
         <is>
-          <t>Stakeholder Content Request Fulfillment Rate</t>
+          <t>Operations &amp; Growth Cost</t>
         </is>
       </c>
       <c r="G45" s="124" t="inlineStr">
         <is>
-          <t>Requests from Sales, Placements, Program Ops, Assessments and Instructors fulfilled within agreed timeframes across all products.</t>
+          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
         </is>
       </c>
       <c r="H45" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Stakeholder Alignment (§5)</t>
+          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
         </is>
       </c>
       <c r="I45" s="123" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="J45" s="123" t="inlineStr">
@@ -7709,7 +7721,7 @@
       </c>
       <c r="N45" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 90 · A 90.</t>
+          <t>Q1 Jul: A ₹300,863.</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7736,7 @@
       </c>
       <c r="C46" s="124" t="inlineStr">
         <is>
-          <t>Stakeholder Alignment</t>
+          <t>Executive Ops</t>
         </is>
       </c>
       <c r="D46" s="123" t="inlineStr">
@@ -7739,17 +7751,17 @@
       </c>
       <c r="F46" s="125" t="inlineStr">
         <is>
-          <t>Cross-functional Sprint Delivery Rate</t>
+          <t>Creative Resource Utilisation Rate</t>
         </is>
       </c>
       <c r="G46" s="124" t="inlineStr">
         <is>
-          <t>% of committed tickets across Product, Pedagogy, Engineering, UI/UX and DA/DE — scoped and approved by this team — delivered within the committed sprint.</t>
+          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
         </is>
       </c>
       <c r="H46" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Stakeholder Alignment (§5)</t>
+          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
         </is>
       </c>
       <c r="I46" s="123" t="inlineStr">
@@ -7770,155 +7782,101 @@
       </c>
       <c r="N46" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 100 · A 100.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="45" customHeight="1">
-      <c r="A47" s="123" t="n">
-        <v>24</v>
-      </c>
-      <c r="B47" s="123" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C47" s="124" t="inlineStr">
-        <is>
-          <t>Executive Ops</t>
-        </is>
-      </c>
-      <c r="D47" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="E47" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F47" s="125" t="inlineStr">
-        <is>
-          <t>Operations &amp; Growth Cost</t>
-        </is>
-      </c>
-      <c r="G47" s="124" t="inlineStr">
-        <is>
-          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
-        </is>
-      </c>
-      <c r="H47" s="124" t="inlineStr">
-        <is>
-          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
-        </is>
-      </c>
-      <c r="I47" s="123" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="J47" s="123" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K47" s="123" t="n"/>
-      <c r="L47" s="123" t="n"/>
-      <c r="M47" s="126">
-        <f>IF(AND(ISNUMBER(K47),ISNUMBER(L47)),K47-L47,"")</f>
-        <v/>
-      </c>
-      <c r="N47" s="124" t="inlineStr">
-        <is>
-          <t>Q1 Jul: A ₹300,863.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="58" customHeight="1">
-      <c r="A48" s="123" t="n">
-        <v>25</v>
-      </c>
-      <c r="B48" s="123" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C48" s="124" t="inlineStr">
-        <is>
-          <t>Executive Ops</t>
-        </is>
-      </c>
-      <c r="D48" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="E48" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F48" s="125" t="inlineStr">
-        <is>
-          <t>Creative Resource Utilisation Rate</t>
-        </is>
-      </c>
-      <c r="G48" s="124" t="inlineStr">
-        <is>
-          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
-        </is>
-      </c>
-      <c r="H48" s="124" t="inlineStr">
-        <is>
-          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
-        </is>
-      </c>
-      <c r="I48" s="123" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="J48" s="123" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="K48" s="123" t="n"/>
-      <c r="L48" s="123" t="n"/>
-      <c r="M48" s="126">
-        <f>IF(AND(ISNUMBER(K48),ISNUMBER(L48)),K48-L48,"")</f>
-        <v/>
-      </c>
-      <c r="N48" s="124" t="inlineStr">
-        <is>
           <t>Q1 Jul: A 100% — fully utilised, at times stretched.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="129" t="inlineStr">
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="129" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B49" s="119" t="n"/>
-      <c r="C49" s="119" t="n"/>
-      <c r="D49" s="119" t="n"/>
-      <c r="E49" s="119" t="n"/>
-      <c r="F49" s="119" t="n"/>
-      <c r="G49" s="119" t="n"/>
-      <c r="H49" s="119" t="n"/>
-      <c r="I49" s="119" t="n"/>
-      <c r="J49" s="119" t="n"/>
-      <c r="K49" s="119" t="n"/>
-      <c r="L49" s="119" t="n"/>
-      <c r="M49" s="119" t="n"/>
-      <c r="N49" s="119" t="n"/>
+      <c r="B47" s="119" t="n"/>
+      <c r="C47" s="119" t="n"/>
+      <c r="D47" s="119" t="n"/>
+      <c r="E47" s="119" t="n"/>
+      <c r="F47" s="119" t="n"/>
+      <c r="G47" s="119" t="n"/>
+      <c r="H47" s="119" t="n"/>
+      <c r="I47" s="119" t="n"/>
+      <c r="J47" s="119" t="n"/>
+      <c r="K47" s="119" t="n"/>
+      <c r="L47" s="119" t="n"/>
+      <c r="M47" s="119" t="n"/>
+      <c r="N47" s="119" t="n"/>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C48" s="131" t="inlineStr">
+        <is>
+          <t>Assessments team</t>
+        </is>
+      </c>
+      <c r="D48" s="130" t="n"/>
+      <c r="E48" s="130" t="n"/>
+      <c r="F48" s="132" t="inlineStr">
+        <is>
+          <t>Assessment blueprints per cycle</t>
+        </is>
+      </c>
+      <c r="G48" s="131" t="inlineStr">
+        <is>
+          <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
+        </is>
+      </c>
+      <c r="H48" s="131" t="n"/>
+      <c r="I48" s="130" t="n"/>
+      <c r="J48" s="130" t="n"/>
+      <c r="K48" s="130" t="n"/>
+      <c r="L48" s="130" t="n"/>
+      <c r="M48" s="130" t="n"/>
+      <c r="N48" s="131" t="n"/>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="130" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C49" s="131" t="inlineStr">
+        <is>
+          <t>Learning Platform / DA-DEs</t>
+        </is>
+      </c>
+      <c r="D49" s="130" t="n"/>
+      <c r="E49" s="130" t="n"/>
+      <c r="F49" s="132" t="inlineStr">
+        <is>
+          <t>Engagement &amp; LE dashboards</t>
+        </is>
+      </c>
+      <c r="G49" s="131" t="inlineStr">
+        <is>
+          <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here. Course-completion cuts included as a read-only view: completion is conduction-driven (Program Ops); the team's owned stickiness KPIs are Learner-Accessed Completion + Practice Attempt-to-Completion.</t>
+        </is>
+      </c>
+      <c r="H49" s="131" t="n"/>
+      <c r="I49" s="130" t="n"/>
+      <c r="J49" s="130" t="n"/>
+      <c r="K49" s="130" t="n"/>
+      <c r="L49" s="130" t="n"/>
+      <c r="M49" s="130" t="n"/>
+      <c r="N49" s="131" t="n"/>
     </row>
     <row r="50" ht="40" customHeight="1">
       <c r="A50" s="130" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B50" s="130" t="inlineStr">
         <is>
@@ -7927,19 +7885,19 @@
       </c>
       <c r="C50" s="131" t="inlineStr">
         <is>
-          <t>Assessments team</t>
+          <t>Instructors dept + Program Ops</t>
         </is>
       </c>
       <c r="D50" s="130" t="n"/>
       <c r="E50" s="130" t="n"/>
       <c r="F50" s="132" t="inlineStr">
         <is>
-          <t>Assessment blueprints per cycle</t>
+          <t>Classroom signal loop</t>
         </is>
       </c>
       <c r="G50" s="131" t="inlineStr">
         <is>
-          <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
+          <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
         </is>
       </c>
       <c r="H50" s="131" t="n"/>
@@ -7950,82 +7908,14 @@
       <c r="M50" s="130" t="n"/>
       <c r="N50" s="131" t="n"/>
     </row>
-    <row r="51" ht="40" customHeight="1">
-      <c r="A51" s="130" t="n">
-        <v>2</v>
-      </c>
-      <c r="B51" s="130" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C51" s="131" t="inlineStr">
-        <is>
-          <t>Learning Platform / DA-DEs</t>
-        </is>
-      </c>
-      <c r="D51" s="130" t="n"/>
-      <c r="E51" s="130" t="n"/>
-      <c r="F51" s="132" t="inlineStr">
-        <is>
-          <t>Engagement &amp; LE dashboards</t>
-        </is>
-      </c>
-      <c r="G51" s="131" t="inlineStr">
-        <is>
-          <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here.</t>
-        </is>
-      </c>
-      <c r="H51" s="131" t="n"/>
-      <c r="I51" s="130" t="n"/>
-      <c r="J51" s="130" t="n"/>
-      <c r="K51" s="130" t="n"/>
-      <c r="L51" s="130" t="n"/>
-      <c r="M51" s="130" t="n"/>
-      <c r="N51" s="131" t="n"/>
-    </row>
-    <row r="52" ht="40" customHeight="1">
-      <c r="A52" s="130" t="n">
-        <v>3</v>
-      </c>
-      <c r="B52" s="130" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C52" s="131" t="inlineStr">
-        <is>
-          <t>Instructors dept + Program Ops</t>
-        </is>
-      </c>
-      <c r="D52" s="130" t="n"/>
-      <c r="E52" s="130" t="n"/>
-      <c r="F52" s="132" t="inlineStr">
-        <is>
-          <t>Classroom signal loop</t>
-        </is>
-      </c>
-      <c r="G52" s="131" t="inlineStr">
-        <is>
-          <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
-        </is>
-      </c>
-      <c r="H52" s="131" t="n"/>
-      <c r="I52" s="130" t="n"/>
-      <c r="J52" s="130" t="n"/>
-      <c r="K52" s="130" t="n"/>
-      <c r="L52" s="130" t="n"/>
-      <c r="M52" s="130" t="n"/>
-      <c r="N52" s="131" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="G51:N51"/>
-    <mergeCell ref="G52:N52"/>
+    <mergeCell ref="G49:N49"/>
+    <mergeCell ref="G48:N48"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="G50:N50"/>
-    <mergeCell ref="A49:N49"/>
+    <mergeCell ref="A47:N47"/>
     <mergeCell ref="A23:N23"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Domain Product Enablement: FS Section B rows + LP build ask + boundary legend
Section-B-first per ruling: eval-env coverage + domain capability delivery,
raised by domain SMEs, built by PMs + Engineering, accountability in
Learning Domains. Legend 23 records the generic-vs-domain and ACP
boundaries; Packaging Teams named Content Systems & Infra.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -3945,7 +3945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="B4" s="33" t="inlineStr">
         <is>
-          <t>The teams that actively build the learning system (HOD one-pager §2 key terms): Content, Engineering, Product Managers, Pedagogy Experts, DA/DEs, Graphic Designers, Video Editors, Product Designers, Packaging Teams, SDIs — plus the CSI team on delivery- and university-facing rows. Draft for red-pen.</t>
+          <t>The teams that actively build the learning system (HOD one-pager §2 key terms): Content, Engineering, Product Managers, Pedagogy Experts, DA/DEs, Graphic Designers, Video Editors, Product Designers, Packaging Teams (Content Systems &amp; Infra), SDIs — plus the CSI team on delivery- and university-facing rows. Draft for red-pen.</t>
         </is>
       </c>
     </row>
@@ -4189,6 +4189,18 @@
       <c r="B22" s="49" t="inlineStr">
         <is>
           <t>Worked by (primary) — staffing, never ownership (col L stays the accountability; many-to-many): Learning Domains — Content domain teams + Pedagogy Experts (lesson-plan design, the in-classroom experience) + DA/DEs · Learning Platform — Product Managers + Engineering + DA/DEs · Product Learning Experience — CSI team + Product Managers + Pedagogy Experts (journey design) · Agentic Content Platform — Content–Central + DA/DEs · Developer Platform — Engineering · Shared/PMO — PMO. Program Ops, Instructors dept and Mentors are counterparties reached through asks (§7 / team-view Section C), not lane staff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t>Domain product boundary</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>Domain-specific product work — evaluation environments and domain-specific learning-platform capabilities, incl. domain-specific learner-facing AI tutors/agents — is raised and accepted by domain SMEs, built by Product Managers + Engineering, and its KPIs sit in the domain team's Section B under Domain Product Enablement (Learning Domains accountability). Generic/reusable capabilities rest with the Learning Platform lane, product-owned. ACP boundary: ACP = content-facing production pipelines · domain product work = learner-facing systems. Section-B-first: an org-tracker row waits until the environment registry sets a baseline.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7664,7 +7676,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="45" customHeight="1">
+    <row r="45" ht="84" customHeight="1">
       <c r="A45" s="123" t="n">
         <v>22</v>
       </c>
@@ -7675,7 +7687,7 @@
       </c>
       <c r="C45" s="124" t="inlineStr">
         <is>
-          <t>Executive Ops</t>
+          <t>Domain Product Enablement</t>
         </is>
       </c>
       <c r="D45" s="123" t="inlineStr">
@@ -7690,27 +7702,27 @@
       </c>
       <c r="F45" s="125" t="inlineStr">
         <is>
-          <t>Operations &amp; Growth Cost</t>
+          <t>Evaluation Environment Coverage</t>
         </is>
       </c>
       <c r="G45" s="124" t="inlineStr">
         <is>
-          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+          <t>% of practice/assessment item types in this domain's live curriculum with a production-ready evaluation environment (code judges, test harnesses, notebook/cloud envs). Domain configuration — item types, test cases, judges — by this team's SMEs; platform build by Product Managers + Engineering.</t>
         </is>
       </c>
       <c r="H45" s="124" t="inlineStr">
         <is>
-          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
+          <t>enabling → Practice Attempt-to-Completion (environment-friction leg) + tracker Journey Step Health steps 6–7 + Learning Environment Satisfaction</t>
         </is>
       </c>
       <c r="I45" s="123" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J45" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K45" s="123" t="n"/>
@@ -7721,11 +7733,11 @@
       </c>
       <c r="N45" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: A ₹300,863.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="58" customHeight="1">
+          <t>Baseline first: build the item-type × environment registry, then set the budget (APC precedent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="71" customHeight="1">
       <c r="A46" s="123" t="n">
         <v>23</v>
       </c>
@@ -7736,7 +7748,7 @@
       </c>
       <c r="C46" s="124" t="inlineStr">
         <is>
-          <t>Executive Ops</t>
+          <t>Domain Product Enablement</t>
         </is>
       </c>
       <c r="D46" s="123" t="inlineStr">
@@ -7751,17 +7763,17 @@
       </c>
       <c r="F46" s="125" t="inlineStr">
         <is>
-          <t>Creative Resource Utilisation Rate</t>
+          <t>Domain Capability Delivery</t>
         </is>
       </c>
       <c r="G46" s="124" t="inlineStr">
         <is>
-          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
+          <t>Domain-specific learning-platform capabilities shipped vs committed per cycle. Raised and specified by this team's SMEs; built by Product Managers + Engineering; accountability stays here — the ask and the acceptance are domain-owned.</t>
         </is>
       </c>
       <c r="H46" s="124" t="inlineStr">
         <is>
-          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
+          <t>enabling → dept Platform Capability Configuration Coverage (§5) + the LP capability registry</t>
         </is>
       </c>
       <c r="I46" s="123" t="inlineStr">
@@ -7771,7 +7783,7 @@
       </c>
       <c r="J46" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K46" s="123" t="n"/>
@@ -7782,101 +7794,155 @@
       </c>
       <c r="N46" s="124" t="inlineStr">
         <is>
+          <t>Generic/reusable capabilities rest with the Learning Platform lane (product-owned), not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1">
+      <c r="A47" s="123" t="n">
+        <v>24</v>
+      </c>
+      <c r="B47" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C47" s="124" t="inlineStr">
+        <is>
+          <t>Executive Ops</t>
+        </is>
+      </c>
+      <c r="D47" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E47" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F47" s="125" t="inlineStr">
+        <is>
+          <t>Operations &amp; Growth Cost</t>
+        </is>
+      </c>
+      <c r="G47" s="124" t="inlineStr">
+        <is>
+          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+        </is>
+      </c>
+      <c r="H47" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — team run-cost guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I47" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="J47" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K47" s="123" t="n"/>
+      <c r="L47" s="123" t="n"/>
+      <c r="M47" s="126">
+        <f>IF(AND(ISNUMBER(K47),ISNUMBER(L47)),K47-L47,"")</f>
+        <v/>
+      </c>
+      <c r="N47" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: A ₹300,863.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="58" customHeight="1">
+      <c r="A48" s="123" t="n">
+        <v>25</v>
+      </c>
+      <c r="B48" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C48" s="124" t="inlineStr">
+        <is>
+          <t>Executive Ops</t>
+        </is>
+      </c>
+      <c r="D48" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E48" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F48" s="125" t="inlineStr">
+        <is>
+          <t>Creative Resource Utilisation Rate</t>
+        </is>
+      </c>
+      <c r="G48" s="124" t="inlineStr">
+        <is>
+          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
+        </is>
+      </c>
+      <c r="H48" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I48" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J48" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K48" s="123" t="n"/>
+      <c r="L48" s="123" t="n"/>
+      <c r="M48" s="126">
+        <f>IF(AND(ISNUMBER(K48),ISNUMBER(L48)),K48-L48,"")</f>
+        <v/>
+      </c>
+      <c r="N48" s="124" t="inlineStr">
+        <is>
           <t>Q1 Jul: A 100% — fully utilised, at times stretched.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="129" t="inlineStr">
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="129" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B47" s="119" t="n"/>
-      <c r="C47" s="119" t="n"/>
-      <c r="D47" s="119" t="n"/>
-      <c r="E47" s="119" t="n"/>
-      <c r="F47" s="119" t="n"/>
-      <c r="G47" s="119" t="n"/>
-      <c r="H47" s="119" t="n"/>
-      <c r="I47" s="119" t="n"/>
-      <c r="J47" s="119" t="n"/>
-      <c r="K47" s="119" t="n"/>
-      <c r="L47" s="119" t="n"/>
-      <c r="M47" s="119" t="n"/>
-      <c r="N47" s="119" t="n"/>
-    </row>
-    <row r="48" ht="40" customHeight="1">
-      <c r="A48" s="130" t="n">
-        <v>1</v>
-      </c>
-      <c r="B48" s="130" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C48" s="131" t="inlineStr">
-        <is>
-          <t>Assessments team</t>
-        </is>
-      </c>
-      <c r="D48" s="130" t="n"/>
-      <c r="E48" s="130" t="n"/>
-      <c r="F48" s="132" t="inlineStr">
-        <is>
-          <t>Assessment blueprints per cycle</t>
-        </is>
-      </c>
-      <c r="G48" s="131" t="inlineStr">
-        <is>
-          <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
-        </is>
-      </c>
-      <c r="H48" s="131" t="n"/>
-      <c r="I48" s="130" t="n"/>
-      <c r="J48" s="130" t="n"/>
-      <c r="K48" s="130" t="n"/>
-      <c r="L48" s="130" t="n"/>
-      <c r="M48" s="130" t="n"/>
-      <c r="N48" s="131" t="n"/>
-    </row>
-    <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="130" t="n">
-        <v>2</v>
-      </c>
-      <c r="B49" s="130" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C49" s="131" t="inlineStr">
-        <is>
-          <t>Learning Platform / DA-DEs</t>
-        </is>
-      </c>
-      <c r="D49" s="130" t="n"/>
-      <c r="E49" s="130" t="n"/>
-      <c r="F49" s="132" t="inlineStr">
-        <is>
-          <t>Engagement &amp; LE dashboards</t>
-        </is>
-      </c>
-      <c r="G49" s="131" t="inlineStr">
-        <is>
-          <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here. Course-completion cuts included as a read-only view: completion is conduction-driven (Program Ops); the team's owned stickiness KPIs are Learner-Accessed Completion + Practice Attempt-to-Completion.</t>
-        </is>
-      </c>
-      <c r="H49" s="131" t="n"/>
-      <c r="I49" s="130" t="n"/>
-      <c r="J49" s="130" t="n"/>
-      <c r="K49" s="130" t="n"/>
-      <c r="L49" s="130" t="n"/>
-      <c r="M49" s="130" t="n"/>
-      <c r="N49" s="131" t="n"/>
+      <c r="B49" s="119" t="n"/>
+      <c r="C49" s="119" t="n"/>
+      <c r="D49" s="119" t="n"/>
+      <c r="E49" s="119" t="n"/>
+      <c r="F49" s="119" t="n"/>
+      <c r="G49" s="119" t="n"/>
+      <c r="H49" s="119" t="n"/>
+      <c r="I49" s="119" t="n"/>
+      <c r="J49" s="119" t="n"/>
+      <c r="K49" s="119" t="n"/>
+      <c r="L49" s="119" t="n"/>
+      <c r="M49" s="119" t="n"/>
+      <c r="N49" s="119" t="n"/>
     </row>
     <row r="50" ht="40" customHeight="1">
       <c r="A50" s="130" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B50" s="130" t="inlineStr">
         <is>
@@ -7885,19 +7951,19 @@
       </c>
       <c r="C50" s="131" t="inlineStr">
         <is>
-          <t>Instructors dept + Program Ops</t>
+          <t>Assessments team</t>
         </is>
       </c>
       <c r="D50" s="130" t="n"/>
       <c r="E50" s="130" t="n"/>
       <c r="F50" s="132" t="inlineStr">
         <is>
-          <t>Classroom signal loop</t>
+          <t>Assessment blueprints per cycle</t>
         </is>
       </c>
       <c r="G50" s="131" t="inlineStr">
         <is>
-          <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
+          <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
         </is>
       </c>
       <c r="H50" s="131" t="n"/>
@@ -7908,15 +7974,118 @@
       <c r="M50" s="130" t="n"/>
       <c r="N50" s="131" t="n"/>
     </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="130" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C51" s="131" t="inlineStr">
+        <is>
+          <t>Learning Platform / DA-DEs</t>
+        </is>
+      </c>
+      <c r="D51" s="130" t="n"/>
+      <c r="E51" s="130" t="n"/>
+      <c r="F51" s="132" t="inlineStr">
+        <is>
+          <t>Engagement &amp; LE dashboards</t>
+        </is>
+      </c>
+      <c r="G51" s="131" t="inlineStr">
+        <is>
+          <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here. Course-completion cuts included as a read-only view: completion is conduction-driven (Program Ops); the team's owned stickiness KPIs are Learner-Accessed Completion + Practice Attempt-to-Completion.</t>
+        </is>
+      </c>
+      <c r="H51" s="131" t="n"/>
+      <c r="I51" s="130" t="n"/>
+      <c r="J51" s="130" t="n"/>
+      <c r="K51" s="130" t="n"/>
+      <c r="L51" s="130" t="n"/>
+      <c r="M51" s="130" t="n"/>
+      <c r="N51" s="131" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="130" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C52" s="131" t="inlineStr">
+        <is>
+          <t>Learning Platform (PMs + Engineering)</t>
+        </is>
+      </c>
+      <c r="D52" s="130" t="n"/>
+      <c r="E52" s="130" t="n"/>
+      <c r="F52" s="132" t="inlineStr">
+        <is>
+          <t>Domain-specific capability build</t>
+        </is>
+      </c>
+      <c r="G52" s="131" t="inlineStr">
+        <is>
+          <t>Build slots for domain-raised capabilities and evaluation environments — SMEs here raise and accept; PMs + Engineering build. Boundary: generic/reusable capability = Learning Platform lane (product-owned) · domain-specific instance = KPI here, in Learning Domains · ACP = content-facing production pipelines, domain product work = learner-facing systems.</t>
+        </is>
+      </c>
+      <c r="H52" s="131" t="n"/>
+      <c r="I52" s="130" t="n"/>
+      <c r="J52" s="130" t="n"/>
+      <c r="K52" s="130" t="n"/>
+      <c r="L52" s="130" t="n"/>
+      <c r="M52" s="130" t="n"/>
+      <c r="N52" s="131" t="n"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="130" t="n">
+        <v>4</v>
+      </c>
+      <c r="B53" s="130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C53" s="131" t="inlineStr">
+        <is>
+          <t>Instructors dept + Program Ops</t>
+        </is>
+      </c>
+      <c r="D53" s="130" t="n"/>
+      <c r="E53" s="130" t="n"/>
+      <c r="F53" s="132" t="inlineStr">
+        <is>
+          <t>Classroom signal loop</t>
+        </is>
+      </c>
+      <c r="G53" s="131" t="inlineStr">
+        <is>
+          <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
+        </is>
+      </c>
+      <c r="H53" s="131" t="n"/>
+      <c r="I53" s="130" t="n"/>
+      <c r="J53" s="130" t="n"/>
+      <c r="K53" s="130" t="n"/>
+      <c r="L53" s="130" t="n"/>
+      <c r="M53" s="130" t="n"/>
+      <c r="N53" s="131" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="G49:N49"/>
-    <mergeCell ref="G48:N48"/>
+  <mergeCells count="9">
+    <mergeCell ref="G51:N51"/>
+    <mergeCell ref="G52:N52"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="G50:N50"/>
-    <mergeCell ref="A47:N47"/>
+    <mergeCell ref="A49:N49"/>
     <mergeCell ref="A23:N23"/>
+    <mergeCell ref="G53:N53"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Retire R&D Initiative Impact; APC absorbs it + FS Section A at 90
- R&D II removed from FS Section B, one-pager §5/§9 (totals 47), role-cards chips
- APC cascaded into FS Section A via twins (A 19 / B 24 / C 4)
- EEC/DCD v1 + pre-agreed funnel trigger; PII → Learning-Value Uplift outcome form
- Legend row 24 "Metric evolution (pre-agreed)"; all outputs rebuilt; 4 artifacts republished

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -2568,7 +2568,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="84" customHeight="1">
+    <row r="18" ht="136" customHeight="1">
       <c r="A18" s="74" t="n">
         <v>15</v>
       </c>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="R18" s="76" t="inlineStr">
         <is>
-          <t>ACP's tracker row now CIRE/CIR sit with Learning Domains — this lane builds the pipes; the issue KPIs score the fixes. Target 90% blended (§5); read with cost-per-item + Content Issue Recurrence. Functions cell draft for red-pen.</t>
+          <t>ACP's tracker row now CIRE/CIR sit with Learning Domains — this lane builds the pipes; the issue KPIs score the fixes. Target 90% blended (§5); read with cost-per-item + Content Issue Recurrence. Functions cell draft for red-pen. Absorbs the retired R&amp;D Initiative Impact — initiative counting folds into coverage % + cost-per-item + recurrence; mirrored in FS &amp; CS Core Section A at the same 90.</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4201,6 +4201,18 @@
       <c r="B23" s="49" t="inlineStr">
         <is>
           <t>Domain-specific product work — evaluation environments and domain-specific learning-platform capabilities, incl. domain-specific learner-facing AI tutors/agents — is raised and accepted by domain SMEs, built by Product Managers + Engineering, and its KPIs sit in the domain team's Section B under Domain Product Enablement (Learning Domains accountability). Generic/reusable capabilities rest with the Learning Platform lane, product-owned. ACP boundary: ACP = content-facing production pipelines · domain product work = learner-facing systems. Section-B-first: an org-tracker row waits until the environment registry sets a baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="48" t="inlineStr">
+        <is>
+          <t>Metric evolution (pre-agreed)</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>Forward moves recorded so the sheet evolves without relitigating. (1) R&amp;D Initiative Impact — retired Aug 2026, absorbed by Agentic Production Coverage (org row, mirrored in FS &amp; CS Core Section A at 90) + the cost-per-item rows + Content Issue Recurrence; initiative counting is no longer a KPI anywhere. (2) Evaluation Environment Coverage + Domain Capability Delivery — at ~90% registry coverage or after two review cycles, the pair folds into one funnel KPI: raised → accepted → delivered rate + TAT, with capabilities-raised/quarter as a non-budgeted context line. (3) Pedagogy Initiative Impact — becomes Domain Learning-Value Uplift (ability/band improvement across the domain's courses per cycle, HE×HV machinery, semester/quarter windows) once per-course ability instruments are confirmed.</t>
         </is>
       </c>
     </row>
@@ -6086,10 +6098,10 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="84" customHeight="1">
       <c r="A18" s="130" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B18" s="130" t="inlineStr">
@@ -6098,23 +6110,23 @@
         </is>
       </c>
       <c r="C18" s="131">
-        <f>IF('KPI Tracker FY26-27'!C19="","",'KPI Tracker FY26-27'!C19)</f>
+        <f>IF('KPI Tracker FY26-27'!C18="","",'KPI Tracker FY26-27'!C18)</f>
         <v/>
       </c>
       <c r="D18" s="130">
-        <f>IF('KPI Tracker FY26-27'!D19="","",'KPI Tracker FY26-27'!D19)</f>
+        <f>IF('KPI Tracker FY26-27'!D18="","",'KPI Tracker FY26-27'!D18)</f>
         <v/>
       </c>
       <c r="E18" s="130">
-        <f>IF('KPI Tracker FY26-27'!E19="","",'KPI Tracker FY26-27'!E19)</f>
+        <f>IF('KPI Tracker FY26-27'!E18="","",'KPI Tracker FY26-27'!E18)</f>
         <v/>
       </c>
       <c r="F18" s="132">
-        <f>IF('KPI Tracker FY26-27'!G19="","",'KPI Tracker FY26-27'!G19)</f>
+        <f>IF('KPI Tracker FY26-27'!G18="","",'KPI Tracker FY26-27'!G18)</f>
         <v/>
       </c>
       <c r="G18" s="131">
-        <f>IF('KPI Tracker FY26-27'!H19="","",'KPI Tracker FY26-27'!H19)</f>
+        <f>IF('KPI Tracker FY26-27'!H18="","",'KPI Tracker FY26-27'!H18)</f>
         <v/>
       </c>
       <c r="H18" s="131" t="inlineStr">
@@ -6123,34 +6135,34 @@
         </is>
       </c>
       <c r="I18" s="130">
-        <f>IF('KPI Tracker FY26-27'!M19="","",'KPI Tracker FY26-27'!M19)</f>
+        <f>IF('KPI Tracker FY26-27'!M18="","",'KPI Tracker FY26-27'!M18)</f>
         <v/>
       </c>
       <c r="J18" s="130">
-        <f>IF('KPI Tracker FY26-27'!N19="","",'KPI Tracker FY26-27'!N19)</f>
+        <f>IF('KPI Tracker FY26-27'!N18="","",'KPI Tracker FY26-27'!N18)</f>
         <v/>
       </c>
       <c r="K18" s="130">
-        <f>IF('KPI Tracker FY26-27'!O19="","",'KPI Tracker FY26-27'!O19)</f>
+        <f>IF('KPI Tracker FY26-27'!O18="","",'KPI Tracker FY26-27'!O18)</f>
         <v/>
       </c>
       <c r="L18" s="130">
-        <f>IF('KPI Tracker FY26-27'!P19="","",'KPI Tracker FY26-27'!P19)</f>
+        <f>IF('KPI Tracker FY26-27'!P18="","",'KPI Tracker FY26-27'!P18)</f>
         <v/>
       </c>
       <c r="M18" s="130">
-        <f>IF('KPI Tracker FY26-27'!Q19="","",'KPI Tracker FY26-27'!Q19)</f>
+        <f>IF('KPI Tracker FY26-27'!Q18="","",'KPI Tracker FY26-27'!Q18)</f>
         <v/>
       </c>
       <c r="N18" s="131">
-        <f>IF('KPI Tracker FY26-27'!R19="","",'KPI Tracker FY26-27'!R19)</f>
+        <f>IF('KPI Tracker FY26-27'!R18="","",'KPI Tracker FY26-27'!R18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="130" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B19" s="130" t="inlineStr">
@@ -6159,59 +6171,59 @@
         </is>
       </c>
       <c r="C19" s="131">
-        <f>IF('KPI Tracker FY26-27'!C27="","",'KPI Tracker FY26-27'!C27)</f>
+        <f>IF('KPI Tracker FY26-27'!C19="","",'KPI Tracker FY26-27'!C19)</f>
         <v/>
       </c>
       <c r="D19" s="130">
-        <f>IF('KPI Tracker FY26-27'!D27="","",'KPI Tracker FY26-27'!D27)</f>
+        <f>IF('KPI Tracker FY26-27'!D19="","",'KPI Tracker FY26-27'!D19)</f>
         <v/>
       </c>
       <c r="E19" s="130">
-        <f>IF('KPI Tracker FY26-27'!E27="","",'KPI Tracker FY26-27'!E27)</f>
+        <f>IF('KPI Tracker FY26-27'!E19="","",'KPI Tracker FY26-27'!E19)</f>
         <v/>
       </c>
       <c r="F19" s="132">
-        <f>IF('KPI Tracker FY26-27'!G27="","",'KPI Tracker FY26-27'!G27)</f>
+        <f>IF('KPI Tracker FY26-27'!G19="","",'KPI Tracker FY26-27'!G19)</f>
         <v/>
       </c>
       <c r="G19" s="131">
-        <f>IF('KPI Tracker FY26-27'!H27="","",'KPI Tracker FY26-27'!H27)</f>
+        <f>IF('KPI Tracker FY26-27'!H19="","",'KPI Tracker FY26-27'!H19)</f>
         <v/>
       </c>
       <c r="H19" s="131" t="inlineStr">
         <is>
-          <t>inherited — via Functions (col K)</t>
+          <t>inherited — team-sheet twin</t>
         </is>
       </c>
       <c r="I19" s="130">
-        <f>IF('KPI Tracker FY26-27'!M27="","",'KPI Tracker FY26-27'!M27)</f>
+        <f>IF('KPI Tracker FY26-27'!M19="","",'KPI Tracker FY26-27'!M19)</f>
         <v/>
       </c>
       <c r="J19" s="130">
-        <f>IF('KPI Tracker FY26-27'!N27="","",'KPI Tracker FY26-27'!N27)</f>
+        <f>IF('KPI Tracker FY26-27'!N19="","",'KPI Tracker FY26-27'!N19)</f>
         <v/>
       </c>
       <c r="K19" s="130">
-        <f>IF('KPI Tracker FY26-27'!O27="","",'KPI Tracker FY26-27'!O27)</f>
+        <f>IF('KPI Tracker FY26-27'!O19="","",'KPI Tracker FY26-27'!O19)</f>
         <v/>
       </c>
       <c r="L19" s="130">
-        <f>IF('KPI Tracker FY26-27'!P27="","",'KPI Tracker FY26-27'!P27)</f>
+        <f>IF('KPI Tracker FY26-27'!P19="","",'KPI Tracker FY26-27'!P19)</f>
         <v/>
       </c>
       <c r="M19" s="130">
-        <f>IF('KPI Tracker FY26-27'!Q27="","",'KPI Tracker FY26-27'!Q27)</f>
+        <f>IF('KPI Tracker FY26-27'!Q19="","",'KPI Tracker FY26-27'!Q19)</f>
         <v/>
       </c>
       <c r="N19" s="131">
-        <f>IF('KPI Tracker FY26-27'!R27="","",'KPI Tracker FY26-27'!R27)</f>
+        <f>IF('KPI Tracker FY26-27'!R19="","",'KPI Tracker FY26-27'!R19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="130" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="B20" s="130" t="inlineStr">
@@ -6228,11 +6240,11 @@
         <v/>
       </c>
       <c r="E20" s="130">
-        <f>IF('KPI Tracker FY26-27'!E28="","",'KPI Tracker FY26-27'!E28)</f>
+        <f>IF('KPI Tracker FY26-27'!E27="","",'KPI Tracker FY26-27'!E27)</f>
         <v/>
       </c>
       <c r="F20" s="132">
-        <f>IF('KPI Tracker FY26-27'!G28="","",'KPI Tracker FY26-27'!G28)</f>
+        <f>IF('KPI Tracker FY26-27'!G27="","",'KPI Tracker FY26-27'!G27)</f>
         <v/>
       </c>
       <c r="G20" s="131">
@@ -6253,15 +6265,15 @@
         <v/>
       </c>
       <c r="K20" s="130">
-        <f>IF('KPI Tracker FY26-27'!O28="","",'KPI Tracker FY26-27'!O28)</f>
+        <f>IF('KPI Tracker FY26-27'!O27="","",'KPI Tracker FY26-27'!O27)</f>
         <v/>
       </c>
       <c r="L20" s="130">
-        <f>IF('KPI Tracker FY26-27'!P28="","",'KPI Tracker FY26-27'!P28)</f>
+        <f>IF('KPI Tracker FY26-27'!P27="","",'KPI Tracker FY26-27'!P27)</f>
         <v/>
       </c>
       <c r="M20" s="130">
-        <f>IF('KPI Tracker FY26-27'!Q28="","",'KPI Tracker FY26-27'!Q28)</f>
+        <f>IF('KPI Tracker FY26-27'!Q27="","",'KPI Tracker FY26-27'!Q27)</f>
         <v/>
       </c>
       <c r="N20" s="131">
@@ -6272,7 +6284,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="130" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="B21" s="130" t="inlineStr">
@@ -6281,23 +6293,23 @@
         </is>
       </c>
       <c r="C21" s="131">
-        <f>IF('KPI Tracker FY26-27'!C31="","",'KPI Tracker FY26-27'!C31)</f>
+        <f>IF('KPI Tracker FY26-27'!C27="","",'KPI Tracker FY26-27'!C27)</f>
         <v/>
       </c>
       <c r="D21" s="130">
-        <f>IF('KPI Tracker FY26-27'!D31="","",'KPI Tracker FY26-27'!D31)</f>
+        <f>IF('KPI Tracker FY26-27'!D27="","",'KPI Tracker FY26-27'!D27)</f>
         <v/>
       </c>
       <c r="E21" s="130">
-        <f>IF('KPI Tracker FY26-27'!E31="","",'KPI Tracker FY26-27'!E31)</f>
+        <f>IF('KPI Tracker FY26-27'!E28="","",'KPI Tracker FY26-27'!E28)</f>
         <v/>
       </c>
       <c r="F21" s="132">
-        <f>IF('KPI Tracker FY26-27'!G31="","",'KPI Tracker FY26-27'!G31)</f>
+        <f>IF('KPI Tracker FY26-27'!G28="","",'KPI Tracker FY26-27'!G28)</f>
         <v/>
       </c>
       <c r="G21" s="131">
-        <f>IF('KPI Tracker FY26-27'!H31="","",'KPI Tracker FY26-27'!H31)</f>
+        <f>IF('KPI Tracker FY26-27'!H27="","",'KPI Tracker FY26-27'!H27)</f>
         <v/>
       </c>
       <c r="H21" s="131" t="inlineStr">
@@ -6306,175 +6318,175 @@
         </is>
       </c>
       <c r="I21" s="130">
-        <f>IF('KPI Tracker FY26-27'!M31="","",'KPI Tracker FY26-27'!M31)</f>
+        <f>IF('KPI Tracker FY26-27'!M27="","",'KPI Tracker FY26-27'!M27)</f>
         <v/>
       </c>
       <c r="J21" s="130">
-        <f>IF('KPI Tracker FY26-27'!N31="","",'KPI Tracker FY26-27'!N31)</f>
+        <f>IF('KPI Tracker FY26-27'!N27="","",'KPI Tracker FY26-27'!N27)</f>
         <v/>
       </c>
       <c r="K21" s="130">
-        <f>IF('KPI Tracker FY26-27'!O31="","",'KPI Tracker FY26-27'!O31)</f>
+        <f>IF('KPI Tracker FY26-27'!O28="","",'KPI Tracker FY26-27'!O28)</f>
         <v/>
       </c>
       <c r="L21" s="130">
-        <f>IF('KPI Tracker FY26-27'!P31="","",'KPI Tracker FY26-27'!P31)</f>
+        <f>IF('KPI Tracker FY26-27'!P28="","",'KPI Tracker FY26-27'!P28)</f>
         <v/>
       </c>
       <c r="M21" s="130">
-        <f>IF('KPI Tracker FY26-27'!Q31="","",'KPI Tracker FY26-27'!Q31)</f>
+        <f>IF('KPI Tracker FY26-27'!Q28="","",'KPI Tracker FY26-27'!Q28)</f>
         <v/>
       </c>
       <c r="N21" s="131">
-        <f>IF('KPI Tracker FY26-27'!R31="","",'KPI Tracker FY26-27'!R31)</f>
+        <f>IF('KPI Tracker FY26-27'!R27="","",'KPI Tracker FY26-27'!R27)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="130" t="inlineStr">
         <is>
+          <t>T27</t>
+        </is>
+      </c>
+      <c r="B22" s="130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C22" s="131">
+        <f>IF('KPI Tracker FY26-27'!C31="","",'KPI Tracker FY26-27'!C31)</f>
+        <v/>
+      </c>
+      <c r="D22" s="130">
+        <f>IF('KPI Tracker FY26-27'!D31="","",'KPI Tracker FY26-27'!D31)</f>
+        <v/>
+      </c>
+      <c r="E22" s="130">
+        <f>IF('KPI Tracker FY26-27'!E31="","",'KPI Tracker FY26-27'!E31)</f>
+        <v/>
+      </c>
+      <c r="F22" s="132">
+        <f>IF('KPI Tracker FY26-27'!G31="","",'KPI Tracker FY26-27'!G31)</f>
+        <v/>
+      </c>
+      <c r="G22" s="131">
+        <f>IF('KPI Tracker FY26-27'!H31="","",'KPI Tracker FY26-27'!H31)</f>
+        <v/>
+      </c>
+      <c r="H22" s="131" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K)</t>
+        </is>
+      </c>
+      <c r="I22" s="130">
+        <f>IF('KPI Tracker FY26-27'!M31="","",'KPI Tracker FY26-27'!M31)</f>
+        <v/>
+      </c>
+      <c r="J22" s="130">
+        <f>IF('KPI Tracker FY26-27'!N31="","",'KPI Tracker FY26-27'!N31)</f>
+        <v/>
+      </c>
+      <c r="K22" s="130">
+        <f>IF('KPI Tracker FY26-27'!O31="","",'KPI Tracker FY26-27'!O31)</f>
+        <v/>
+      </c>
+      <c r="L22" s="130">
+        <f>IF('KPI Tracker FY26-27'!P31="","",'KPI Tracker FY26-27'!P31)</f>
+        <v/>
+      </c>
+      <c r="M22" s="130">
+        <f>IF('KPI Tracker FY26-27'!Q31="","",'KPI Tracker FY26-27'!Q31)</f>
+        <v/>
+      </c>
+      <c r="N22" s="131">
+        <f>IF('KPI Tracker FY26-27'!R31="","",'KPI Tracker FY26-27'!R31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="130" t="inlineStr">
+        <is>
           <t>T28</t>
         </is>
       </c>
-      <c r="B22" s="130" t="inlineStr">
+      <c r="B23" s="130" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C22" s="131">
+      <c r="C23" s="131">
         <f>IF('KPI Tracker FY26-27'!C32="","",'KPI Tracker FY26-27'!C32)</f>
         <v/>
       </c>
-      <c r="D22" s="130">
+      <c r="D23" s="130">
         <f>IF('KPI Tracker FY26-27'!D32="","",'KPI Tracker FY26-27'!D32)</f>
         <v/>
       </c>
-      <c r="E22" s="130">
+      <c r="E23" s="130">
         <f>IF('KPI Tracker FY26-27'!E32="","",'KPI Tracker FY26-27'!E32)</f>
         <v/>
       </c>
-      <c r="F22" s="132">
+      <c r="F23" s="132">
         <f>IF('KPI Tracker FY26-27'!G32="","",'KPI Tracker FY26-27'!G32)</f>
         <v/>
       </c>
-      <c r="G22" s="131">
+      <c r="G23" s="131">
         <f>IF('KPI Tracker FY26-27'!H32="","",'KPI Tracker FY26-27'!H32)</f>
         <v/>
       </c>
-      <c r="H22" s="131" t="inlineStr">
+      <c r="H23" s="131" t="inlineStr">
         <is>
           <t>inherited — via Functions (col K)</t>
         </is>
       </c>
-      <c r="I22" s="130">
+      <c r="I23" s="130">
         <f>IF('KPI Tracker FY26-27'!M32="","",'KPI Tracker FY26-27'!M32)</f>
         <v/>
       </c>
-      <c r="J22" s="130">
+      <c r="J23" s="130">
         <f>IF('KPI Tracker FY26-27'!N32="","",'KPI Tracker FY26-27'!N32)</f>
         <v/>
       </c>
-      <c r="K22" s="130">
+      <c r="K23" s="130">
         <f>IF('KPI Tracker FY26-27'!O32="","",'KPI Tracker FY26-27'!O32)</f>
         <v/>
       </c>
-      <c r="L22" s="130">
+      <c r="L23" s="130">
         <f>IF('KPI Tracker FY26-27'!P32="","",'KPI Tracker FY26-27'!P32)</f>
         <v/>
       </c>
-      <c r="M22" s="130">
+      <c r="M23" s="130">
         <f>IF('KPI Tracker FY26-27'!Q32="","",'KPI Tracker FY26-27'!Q32)</f>
         <v/>
       </c>
-      <c r="N22" s="131">
+      <c r="N23" s="131">
         <f>IF('KPI Tracker FY26-27'!R32="","",'KPI Tracker FY26-27'!R32)</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="129" t="inlineStr">
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="129" t="inlineStr">
         <is>
           <t>B — Owned: functional KPIs this team runs (budgets &amp; actuals live here) — Ladders-to key: direct = an org-KRA number · enabling = a dept §5 KPI · hygiene = guardrail by design</t>
         </is>
       </c>
-      <c r="B23" s="119" t="n"/>
-      <c r="C23" s="119" t="n"/>
-      <c r="D23" s="119" t="n"/>
-      <c r="E23" s="119" t="n"/>
-      <c r="F23" s="119" t="n"/>
-      <c r="G23" s="119" t="n"/>
-      <c r="H23" s="119" t="n"/>
-      <c r="I23" s="119" t="n"/>
-      <c r="J23" s="119" t="n"/>
-      <c r="K23" s="119" t="n"/>
-      <c r="L23" s="119" t="n"/>
-      <c r="M23" s="119" t="n"/>
-      <c r="N23" s="119" t="n"/>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="123" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C24" s="124" t="inlineStr">
-        <is>
-          <t>Business Impact</t>
-        </is>
-      </c>
-      <c r="D24" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="E24" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F24" s="125" t="inlineStr">
-        <is>
-          <t>Summative Skill Assessment Achievement Rate</t>
-        </is>
-      </c>
-      <c r="G24" s="124" t="inlineStr">
-        <is>
-          <t>Students scoring above the defined passing threshold in summative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
-        </is>
-      </c>
-      <c r="H24" s="124" t="inlineStr">
-        <is>
-          <t>direct → org KRA 1 — the summative achievement number itself (org scoreboard; the tracker reads it via module-quiz Bands + Alignment)</t>
-        </is>
-      </c>
-      <c r="I24" s="123" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="J24" s="123" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="K24" s="123" t="n"/>
-      <c r="L24" s="123" t="n"/>
-      <c r="M24" s="126">
-        <f>IF(AND(ISNUMBER(K24),ISNUMBER(L24)),K24-L24,"")</f>
-        <v/>
-      </c>
-      <c r="N24" s="124" t="inlineStr">
-        <is>
-          <t>Q1 ref: B 35 (quarterly) · default threshold 70%.</t>
-        </is>
-      </c>
+      <c r="B24" s="119" t="n"/>
+      <c r="C24" s="119" t="n"/>
+      <c r="D24" s="119" t="n"/>
+      <c r="E24" s="119" t="n"/>
+      <c r="F24" s="119" t="n"/>
+      <c r="G24" s="119" t="n"/>
+      <c r="H24" s="119" t="n"/>
+      <c r="I24" s="119" t="n"/>
+      <c r="J24" s="119" t="n"/>
+      <c r="K24" s="119" t="n"/>
+      <c r="L24" s="119" t="n"/>
+      <c r="M24" s="119" t="n"/>
+      <c r="N24" s="119" t="n"/>
     </row>
     <row r="25" ht="58" customHeight="1">
       <c r="A25" s="123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="123" t="inlineStr">
         <is>
@@ -6498,17 +6510,17 @@
       </c>
       <c r="F25" s="125" t="inlineStr">
         <is>
-          <t>Formative Skill Assessment Achievement Rate</t>
+          <t>Summative Skill Assessment Achievement Rate</t>
         </is>
       </c>
       <c r="G25" s="124" t="inlineStr">
         <is>
-          <t>Students scoring above the defined passing threshold in formative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
+          <t>Students scoring above the defined passing threshold in summative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
         </is>
       </c>
       <c r="H25" s="124" t="inlineStr">
         <is>
-          <t>enabling → Summative SA Achievement (row above) + tracker Content–Assessment Alignment — the early-warning formative read</t>
+          <t>direct → org KRA 1 — the summative achievement number itself (org scoreboard; the tracker reads it via module-quiz Bands + Alignment)</t>
         </is>
       </c>
       <c r="I25" s="123" t="inlineStr">
@@ -6518,7 +6530,7 @@
       </c>
       <c r="J25" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K25" s="123" t="n"/>
@@ -6529,13 +6541,13 @@
       </c>
       <c r="N25" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 23 · A 33.4 — 75% cap used as the Skill Assessments cut-off.</t>
+          <t>Q1 ref: B 35 (quarterly) · default threshold 70%.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="58" customHeight="1">
       <c r="A26" s="123" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B26" s="123" t="inlineStr">
         <is>
@@ -6549,7 +6561,7 @@
       </c>
       <c r="D26" s="123" t="inlineStr">
         <is>
-          <t>NIAT</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E26" s="123" t="inlineStr">
@@ -6559,17 +6571,17 @@
       </c>
       <c r="F26" s="125" t="inlineStr">
         <is>
-          <t>Graded Assessment Achievement Rate</t>
+          <t>Formative Skill Assessment Achievement Rate</t>
         </is>
       </c>
       <c r="G26" s="124" t="inlineStr">
         <is>
-          <t>Students scoring above the defined passing threshold in university-conducted graded assessments — Mid-1, Mid-2 and End Semester exams — delivered in collaboration with the university.</t>
+          <t>Students scoring above the defined passing threshold in formative skill assessments across owned domains. Passing threshold set by the team per domain context (default reference: 70%).</t>
         </is>
       </c>
       <c r="H26" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Business Impact (§5) — university-conducted exams: NIAT SPI &amp; university trust</t>
+          <t>enabling → Summative SA Achievement (row above) + tracker Content–Assessment Alignment — the early-warning formative read</t>
         </is>
       </c>
       <c r="I26" s="123" t="inlineStr">
@@ -6588,11 +6600,15 @@
         <f>IF(AND(ISNUMBER(K26),ISNUMBER(L26)),K26-L26,"")</f>
         <v/>
       </c>
-      <c r="N26" s="124" t="inlineStr"/>
-    </row>
-    <row r="27" ht="45" customHeight="1">
+      <c r="N26" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 23 · A 33.4 — 75% cap used as the Skill Assessments cut-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
       <c r="A27" s="123" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="123" t="inlineStr">
         <is>
@@ -6606,7 +6622,7 @@
       </c>
       <c r="D27" s="123" t="inlineStr">
         <is>
-          <t>Launchpad</t>
+          <t>NIAT</t>
         </is>
       </c>
       <c r="E27" s="123" t="inlineStr">
@@ -6616,27 +6632,27 @@
       </c>
       <c r="F27" s="125" t="inlineStr">
         <is>
-          <t>Weekly Active Users</t>
+          <t>Graded Assessment Achievement Rate</t>
         </is>
       </c>
       <c r="G27" s="124" t="inlineStr">
         <is>
-          <t>Total prospective learner leads generated in the period through content-driven channels (organic, referral, campaigns, partnerships).</t>
+          <t>Students scoring above the defined passing threshold in university-conducted graded assessments — Mid-1, Mid-2 and End Semester exams — delivered in collaboration with the university.</t>
         </is>
       </c>
       <c r="H27" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Business Impact (§5) — Launchpad top-of-funnel</t>
+          <t>enabling → dept Business Impact (§5) — university-conducted exams: NIAT SPI &amp; university trust</t>
         </is>
       </c>
       <c r="I27" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J27" s="123" t="inlineStr">
         <is>
-          <t>Monthly (wkly avg)</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K27" s="123" t="n"/>
@@ -6647,9 +6663,9 @@
       </c>
       <c r="N27" s="124" t="inlineStr"/>
     </row>
-    <row r="28" ht="58" customHeight="1">
+    <row r="28" ht="45" customHeight="1">
       <c r="A28" s="123" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="123" t="inlineStr">
         <is>
@@ -6658,32 +6674,32 @@
       </c>
       <c r="C28" s="124" t="inlineStr">
         <is>
-          <t>Content Effectiveness</t>
+          <t>Business Impact</t>
         </is>
       </c>
       <c r="D28" s="123" t="inlineStr">
         <is>
+          <t>Launchpad</t>
+        </is>
+      </c>
+      <c r="E28" s="123" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E28" s="123" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
       <c r="F28" s="125" t="inlineStr">
         <is>
-          <t>Pedagogy Initiative Impact</t>
+          <t>Weekly Active Users</t>
         </is>
       </c>
       <c r="G28" s="124" t="inlineStr">
         <is>
-          <t>Implemented pedagogy initiatives with measurable learning-outcome improvement. Outcome baseline must be defined and agreed before the initiative is launched.</t>
+          <t>Total prospective learner leads generated in the period through content-driven channels (organic, referral, campaigns, partnerships).</t>
         </is>
       </c>
       <c r="H28" s="124" t="inlineStr">
         <is>
-          <t>enabling → module-quiz Bands + org KRA 2 Academics CSAT — pedagogy initiatives move the learning numbers</t>
+          <t>enabling → dept Business Impact (§5) — Launchpad top-of-funnel</t>
         </is>
       </c>
       <c r="I28" s="123" t="inlineStr">
@@ -6693,7 +6709,7 @@
       </c>
       <c r="J28" s="123" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Monthly (wkly avg)</t>
         </is>
       </c>
       <c r="K28" s="123" t="n"/>
@@ -6702,15 +6718,11 @@
         <f>IF(AND(ISNUMBER(K28),ISNUMBER(L28)),K28-L28,"")</f>
         <v/>
       </c>
-      <c r="N28" s="124" t="inlineStr">
-        <is>
-          <t>Owned by the domain SME on this team; embedded Pedagogy Experts contribute to the initiatives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="45" customHeight="1">
+      <c r="N28" s="124" t="inlineStr"/>
+    </row>
+    <row r="29" ht="58" customHeight="1">
       <c r="A29" s="123" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29" s="123" t="inlineStr">
         <is>
@@ -6734,27 +6746,27 @@
       </c>
       <c r="F29" s="125" t="inlineStr">
         <is>
-          <t>Learner Accessed Content Completion Rate</t>
+          <t>Pedagogy Initiative Impact</t>
         </is>
       </c>
       <c r="G29" s="124" t="inlineStr">
         <is>
-          <t>Video units: for each learner, % of video units they opened that they also completed; averaged across learners. Excludes units with zero opens.</t>
+          <t>Implemented pedagogy initiatives with measurable learning-outcome improvement. Outcome baseline must be defined and agreed before the initiative is launched.</t>
         </is>
       </c>
       <c r="H29" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Engagement-Matrix Cell Migration — video-stickiness leg of the value axis; access-conditioned, so conduction effects are stripped</t>
+          <t>enabling → module-quiz Bands + org KRA 2 Academics CSAT — pedagogy initiatives move the learning numbers</t>
         </is>
       </c>
       <c r="I29" s="123" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J29" s="123" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="K29" s="123" t="n"/>
@@ -6763,11 +6775,15 @@
         <f>IF(AND(ISNUMBER(K29),ISNUMBER(L29)),K29-L29,"")</f>
         <v/>
       </c>
-      <c r="N29" s="124" t="inlineStr"/>
-    </row>
-    <row r="30" ht="58" customHeight="1">
+      <c r="N29" s="124" t="inlineStr">
+        <is>
+          <t>Owned by the domain SME on this team; embedded Pedagogy Experts contribute to the initiatives. Pre-agreed outcome form: becomes Domain Learning-Value Uplift — ability/band improvement across this domain's courses per cycle (HE×HV machinery) — once per-course ability instruments are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
       <c r="A30" s="123" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" s="123" t="inlineStr">
         <is>
@@ -6791,17 +6807,17 @@
       </c>
       <c r="F30" s="125" t="inlineStr">
         <is>
-          <t>Practice Attempt-to-Completion Rate</t>
+          <t>Learner Accessed Content Completion Rate</t>
         </is>
       </c>
       <c r="G30" s="124" t="inlineStr">
         <is>
-          <t>Practice units: for each learner, % of coding/project exercises attempted that they also completed. Surfaces environment friction (IDE, playground, cloud setup) vs difficulty-related drop-off.</t>
+          <t>Video units: for each learner, % of video units they opened that they also completed; averaged across learners. Excludes units with zero opens.</t>
         </is>
       </c>
       <c r="H30" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Journey Step Health steps 6–7 (practice return &amp; completion) + Learning Environment Satisfaction</t>
+          <t>enabling → tracker Engagement-Matrix Cell Migration — video-stickiness leg of the value axis; access-conditioned, so conduction effects are stripped</t>
         </is>
       </c>
       <c r="I30" s="123" t="inlineStr">
@@ -6820,15 +6836,11 @@
         <f>IF(AND(ISNUMBER(K30),ISNUMBER(L30)),K30-L30,"")</f>
         <v/>
       </c>
-      <c r="N30" s="124" t="inlineStr">
-        <is>
-          <t>Q1 Jul: B 38.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+      <c r="N30" s="124" t="inlineStr"/>
+    </row>
+    <row r="31" ht="58" customHeight="1">
       <c r="A31" s="123" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B31" s="123" t="inlineStr">
         <is>
@@ -6837,7 +6849,7 @@
       </c>
       <c r="C31" s="124" t="inlineStr">
         <is>
-          <t>Content Velocity</t>
+          <t>Content Effectiveness</t>
         </is>
       </c>
       <c r="D31" s="123" t="inlineStr">
@@ -6852,22 +6864,22 @@
       </c>
       <c r="F31" s="125" t="inlineStr">
         <is>
-          <t>Learning Content Hours Delivered</t>
+          <t>Practice Attempt-to-Completion Rate</t>
         </is>
       </c>
       <c r="G31" s="124" t="inlineStr">
         <is>
-          <t>Total learning content hours created per month across all formats (video, text, interactive). Content serving multiple products counted once.</t>
+          <t>Practice units: for each learner, % of coding/project exercises attempted that they also completed. Surfaces environment friction (IDE, playground, cloud setup) vs difficulty-related drop-off.</t>
         </is>
       </c>
       <c r="H31" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — capacity for B4 &amp; new stacks</t>
+          <t>enabling → tracker Journey Step Health steps 6–7 (practice return &amp; completion) + Learning Environment Satisfaction</t>
         </is>
       </c>
       <c r="I31" s="123" t="inlineStr">
         <is>
-          <t>Hours</t>
+          <t>%</t>
         </is>
       </c>
       <c r="J31" s="123" t="inlineStr">
@@ -6883,13 +6895,13 @@
       </c>
       <c r="N31" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 50 · A 46.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="58" customHeight="1">
+          <t>Q1 Jul: B 38.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
       <c r="A32" s="123" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B32" s="123" t="inlineStr">
         <is>
@@ -6913,17 +6925,17 @@
       </c>
       <c r="F32" s="125" t="inlineStr">
         <is>
-          <t>Vernacular Content Hours Delivered</t>
+          <t>Learning Content Hours Delivered</t>
         </is>
       </c>
       <c r="G32" s="124" t="inlineStr">
         <is>
-          <t>Total vernacular-language learning content hours created per month. Tracked separately from English hours — effort per vernacular hour differs significantly.</t>
+          <t>Total learning content hours created per month across all formats (video, text, interactive). Content serving multiple products counted once.</t>
         </is>
       </c>
       <c r="H32" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — vernacular capacity</t>
+          <t>enabling → dept Content Velocity (§5) — capacity for B4 &amp; new stacks</t>
         </is>
       </c>
       <c r="I32" s="123" t="inlineStr">
@@ -6944,13 +6956,13 @@
       </c>
       <c r="N32" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 — no vernacular slate yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="45" customHeight="1">
+          <t>Q1 Jul: B 50 · A 46.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="58" customHeight="1">
       <c r="A33" s="123" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B33" s="123" t="inlineStr">
         <is>
@@ -6974,22 +6986,22 @@
       </c>
       <c r="F33" s="125" t="inlineStr">
         <is>
-          <t>Practice &amp; Assessment Content Pieces Delivered</t>
+          <t>Vernacular Content Hours Delivered</t>
         </is>
       </c>
       <c r="G33" s="124" t="inlineStr">
         <is>
-          <t>Total practice and assessment pieces delivered monthly across owned domains (MCQs, coding questions, projects, case studies).</t>
+          <t>Total vernacular-language learning content hours created per month. Tracked separately from English hours — effort per vernacular hour differs significantly.</t>
         </is>
       </c>
       <c r="H33" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5) — practice depth behind Journey Step Health steps 5–7</t>
+          <t>enabling → dept Content Velocity (§5) — vernacular capacity</t>
         </is>
       </c>
       <c r="I33" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="J33" s="123" t="inlineStr">
@@ -7005,13 +7017,13 @@
       </c>
       <c r="N33" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 1,600 · A 1,499 (Aug B: 1,000).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1">
+          <t>Q1 Jul: B 0 — no vernacular slate yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="45" customHeight="1">
       <c r="A34" s="123" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B34" s="123" t="inlineStr">
         <is>
@@ -7035,17 +7047,17 @@
       </c>
       <c r="F34" s="125" t="inlineStr">
         <is>
-          <t>Branding Content Assets Delivered</t>
+          <t>Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
       </c>
       <c r="G34" s="124" t="inlineStr">
         <is>
-          <t>Total branded content pieces produced monthly (thumbnails, banners, promo assets).</t>
+          <t>Total practice and assessment pieces delivered monthly across owned domains (MCQs, coding questions, projects, case studies).</t>
         </is>
       </c>
       <c r="H34" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Content Velocity (§5)</t>
+          <t>enabling → dept Content Velocity (§5) — practice depth behind Journey Step Health steps 5–7</t>
         </is>
       </c>
       <c r="I34" s="123" t="inlineStr">
@@ -7066,13 +7078,13 @@
       </c>
       <c r="N34" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="58" customHeight="1">
+          <t>Q1 Jul: B 1,600 · A 1,499 (Aug B: 1,000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="123" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B35" s="123" t="inlineStr">
         <is>
@@ -7081,7 +7093,7 @@
       </c>
       <c r="C35" s="124" t="inlineStr">
         <is>
-          <t>Content Efficiency</t>
+          <t>Content Velocity</t>
         </is>
       </c>
       <c r="D35" s="123" t="inlineStr">
@@ -7096,22 +7108,22 @@
       </c>
       <c r="F35" s="125" t="inlineStr">
         <is>
-          <t>Cost per Learning Hour Produced</t>
+          <t>Branding Content Assets Delivered</t>
         </is>
       </c>
       <c r="G35" s="124" t="inlineStr">
         <is>
-          <t>Average cost to produce one hour of learning content. Includes people, tools and infra involved in creation. Tracks creation efficiency — not delivery cost.</t>
+          <t>Total branded content pieces produced monthly (thumbnails, banners, promo assets).</t>
         </is>
       </c>
       <c r="H35" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Learning Hour (§5 Content Efficiency)</t>
+          <t>enabling → dept Content Velocity (§5)</t>
         </is>
       </c>
       <c r="I35" s="123" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="J35" s="123" t="inlineStr">
@@ -7127,13 +7139,13 @@
       </c>
       <c r="N35" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B ₹10,000 · A ₹6,803 — 46 h across 4 products.</t>
+          <t>Q1 Jul: B 0.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="58" customHeight="1">
       <c r="A36" s="123" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" s="123" t="inlineStr">
         <is>
@@ -7157,17 +7169,17 @@
       </c>
       <c r="F36" s="125" t="inlineStr">
         <is>
-          <t>Cost per Vernacular Content Hour</t>
+          <t>Cost per Learning Hour Produced</t>
         </is>
       </c>
       <c r="G36" s="124" t="inlineStr">
         <is>
-          <t>Average cost to produce one hour of vernacular-language content. Includes team bandwidth involved in creation (contract basis, tools &amp; infrastructure).</t>
+          <t>Average cost to produce one hour of learning content. Includes people, tools and infra involved in creation. Tracks creation efficiency — not delivery cost.</t>
         </is>
       </c>
       <c r="H36" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Vernacular Content Hour (§5) — production-side twin of CSI's central track</t>
+          <t>enabling → dept Cost per Learning Hour (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I36" s="123" t="inlineStr">
@@ -7188,13 +7200,13 @@
       </c>
       <c r="N36" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 · A 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="32" customHeight="1">
+          <t>Q1 Jul: B ₹10,000 · A ₹6,803 — 46 h across 4 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="58" customHeight="1">
       <c r="A37" s="123" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B37" s="123" t="inlineStr">
         <is>
@@ -7218,17 +7230,17 @@
       </c>
       <c r="F37" s="125" t="inlineStr">
         <is>
-          <t>Cost per MCQ Generated</t>
+          <t>Cost per Vernacular Content Hour</t>
         </is>
       </c>
       <c r="G37" s="124" t="inlineStr">
         <is>
-          <t>Average cost to develop one objective question, including both manual and AI-assisted production.</t>
+          <t>Average cost to produce one hour of vernacular-language content. Includes team bandwidth involved in creation (contract basis, tools &amp; infrastructure).</t>
         </is>
       </c>
       <c r="H37" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per MCQ (§5 Content Efficiency)</t>
+          <t>enabling → dept Cost per Vernacular Content Hour (§5) — production-side twin of CSI's central track</t>
         </is>
       </c>
       <c r="I37" s="123" t="inlineStr">
@@ -7249,13 +7261,13 @@
       </c>
       <c r="N37" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B ₹40 · A ₹26 — 1,347 MCQs across 2 products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="45" customHeight="1">
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="123" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B38" s="123" t="inlineStr">
         <is>
@@ -7279,17 +7291,17 @@
       </c>
       <c r="F38" s="125" t="inlineStr">
         <is>
-          <t>Cost per Coding Question</t>
+          <t>Cost per MCQ Generated</t>
         </is>
       </c>
       <c r="G38" s="124" t="inlineStr">
         <is>
-          <t>Average cost to develop one coding question, including test-case design and evaluation-engine configuration.</t>
+          <t>Average cost to develop one objective question, including both manual and AI-assisted production.</t>
         </is>
       </c>
       <c r="H38" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Coding Question (§5 Content Efficiency)</t>
+          <t>enabling → dept Cost per MCQ (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I38" s="123" t="inlineStr">
@@ -7310,13 +7322,13 @@
       </c>
       <c r="N38" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B ₹400 · A ₹163 — 131 coding questions across 3 products.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="32" customHeight="1">
+          <t>Q1 Jul: B ₹40 · A ₹26 — 1,347 MCQs across 2 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
       <c r="A39" s="123" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B39" s="123" t="inlineStr">
         <is>
@@ -7340,17 +7352,17 @@
       </c>
       <c r="F39" s="125" t="inlineStr">
         <is>
-          <t>Cost per Branding Content Asset</t>
+          <t>Cost per Coding Question</t>
         </is>
       </c>
       <c r="G39" s="124" t="inlineStr">
         <is>
-          <t>Average cost to create one branded content piece.</t>
+          <t>Average cost to develop one coding question, including test-case design and evaluation-engine configuration.</t>
         </is>
       </c>
       <c r="H39" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Cost per Branding Asset (§5 Content Efficiency)</t>
+          <t>enabling → dept Cost per Coding Question (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I39" s="123" t="inlineStr">
@@ -7371,13 +7383,13 @@
       </c>
       <c r="N39" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: B 0 · A 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="58" customHeight="1">
+          <t>Q1 Jul: B ₹400 · A ₹163 — 131 coding questions across 3 products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="123" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B40" s="123" t="inlineStr">
         <is>
@@ -7401,17 +7413,17 @@
       </c>
       <c r="F40" s="125" t="inlineStr">
         <is>
-          <t>Platform Runtime Cost per Active Learner</t>
+          <t>Cost per Branding Content Asset</t>
         </is>
       </c>
       <c r="G40" s="124" t="inlineStr">
         <is>
-          <t>Total platform delivery costs (cloud compute, code-execution infra, cloud IDE hosting, GenAI API calls) divided by active learners in the period. Tracks delivery-cost efficiency as usage scales.</t>
+          <t>Average cost to create one branded content piece.</t>
         </is>
       </c>
       <c r="H40" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept Platform Runtime Cost per Active Learner (§5) — the team's share of delivery cost</t>
+          <t>enabling → dept Cost per Branding Asset (§5 Content Efficiency)</t>
         </is>
       </c>
       <c r="I40" s="123" t="inlineStr">
@@ -7430,11 +7442,15 @@
         <f>IF(AND(ISNUMBER(K40),ISNUMBER(L40)),K40-L40,"")</f>
         <v/>
       </c>
-      <c r="N40" s="124" t="inlineStr"/>
-    </row>
-    <row r="41" ht="45" customHeight="1">
+      <c r="N40" s="124" t="inlineStr">
+        <is>
+          <t>Q1 Jul: B 0 · A 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="58" customHeight="1">
       <c r="A41" s="123" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B41" s="123" t="inlineStr">
         <is>
@@ -7458,27 +7474,27 @@
       </c>
       <c r="F41" s="125" t="inlineStr">
         <is>
-          <t>R&amp;D Initiative Impact</t>
+          <t>Platform Runtime Cost per Active Learner</t>
         </is>
       </c>
       <c r="G41" s="124" t="inlineStr">
         <is>
-          <t>Implemented R&amp;D initiatives — including adoption of agentic AI solutions and automation pipelines — with measurable content-production improvement.</t>
+          <t>Total platform delivery costs (cloud compute, code-execution infra, cloud IDE hosting, GenAI API calls) divided by active learners in the period. Tracks delivery-cost efficiency as usage scales.</t>
         </is>
       </c>
       <c r="H41" s="124" t="inlineStr">
         <is>
-          <t>enabling → dept R&amp;D Initiative Impact (§5) + tracker row Agentic Production Coverage</t>
+          <t>enabling → dept Platform Runtime Cost per Active Learner (§5) — the team's share of delivery cost</t>
         </is>
       </c>
       <c r="I41" s="123" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="J41" s="123" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K41" s="123" t="n"/>
@@ -7487,15 +7503,11 @@
         <f>IF(AND(ISNUMBER(K41),ISNUMBER(L41)),K41-L41,"")</f>
         <v/>
       </c>
-      <c r="N41" s="124" t="inlineStr">
-        <is>
-          <t>Q1 Jul: B 0 · A 0.</t>
-        </is>
-      </c>
+      <c r="N41" s="124" t="inlineStr"/>
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="123" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" s="123" t="inlineStr">
         <is>
@@ -7556,7 +7568,7 @@
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="123" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B43" s="123" t="inlineStr">
         <is>
@@ -7617,7 +7629,7 @@
     </row>
     <row r="44" ht="58" customHeight="1">
       <c r="A44" s="123" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B44" s="123" t="inlineStr">
         <is>
@@ -7678,7 +7690,7 @@
     </row>
     <row r="45" ht="84" customHeight="1">
       <c r="A45" s="123" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B45" s="123" t="inlineStr">
         <is>
@@ -7733,13 +7745,13 @@
       </c>
       <c r="N45" s="124" t="inlineStr">
         <is>
-          <t>Baseline first: build the item-type × environment registry, then set the budget (APC precedent).</t>
+          <t>Baseline first: build the item-type × environment registry, then set the budget (APC precedent). Pre-agreed evolution: at ~90% coverage or after two cycles, EEC + DCD fold into one funnel KPI — raised → accepted → delivered rate + TAT, with capabilities-raised/quarter as a non-budgeted context line.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="71" customHeight="1">
       <c r="A46" s="123" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B46" s="123" t="inlineStr">
         <is>
@@ -7794,13 +7806,13 @@
       </c>
       <c r="N46" s="124" t="inlineStr">
         <is>
-          <t>Generic/reusable capabilities rest with the Learning Platform lane (product-owned), not here.</t>
+          <t>Generic/reusable capabilities rest with the Learning Platform lane (product-owned), not here. Folds into the raised → accepted → delivered funnel with EEC when the trigger lands (see EEC remark + Legend).</t>
         </is>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1">
       <c r="A47" s="123" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B47" s="123" t="inlineStr">
         <is>
@@ -7861,7 +7873,7 @@
     </row>
     <row r="48" ht="58" customHeight="1">
       <c r="A48" s="123" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B48" s="123" t="inlineStr">
         <is>
@@ -8081,10 +8093,10 @@
     <mergeCell ref="G51:N51"/>
     <mergeCell ref="G52:N52"/>
     <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A24:N24"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="G50:N50"/>
     <mergeCell ref="A49:N49"/>
-    <mergeCell ref="A23:N23"/>
     <mergeCell ref="G53:N53"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Content–Central team view: APC mirror + 5 owned rows + §7 asks
New 6th tab in kra_training_sheet.xlsx (Section-B-first, org tracker
untouched): Section A = live APC mirror with units-at-bar Central read
(new per-view a_notes hook); Section B = Deliverables Landed, Spend vs
Plan, Shared Tool Adoption, Check-ins Run, Actions Closed (baseline
first, budgets blank); Section C = execution-management + creative
delivery-management asks. CRU verified not an org row — Section A is
APC-only. Html/site tab counts synced; both artifacts republished.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSI Team View" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FullStack &amp; CS Core View" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content–Central View" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,7 +99,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill/>
     </fill>
@@ -226,6 +227,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1BAF7A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDA100"/>
       </patternFill>
     </fill>
   </fills>
@@ -962,7 +968,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1300,6 +1306,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8102,4 +8126,624 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFEDA100"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="137" t="inlineStr">
+        <is>
+          <t>Content–Central — Functional Operating View · FY 2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="116" t="inlineStr">
+        <is>
+          <t>Shared/PMO lane — the central two-person team: a Business Ops owner (shared-team delivery + Agentic Content Platform builds; reports to the HOD) with a PMO manager reporting to them — role titles pending. Section A mirrors the department tracker (live formulas — numbers are edited on the KPI Tracker tab only) · Section B is owned here, budgets &amp; actuals live on this tab · Section C = asks of counterparties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="138" t="inlineStr">
+        <is>
+          <t>S. No</t>
+        </is>
+      </c>
+      <c r="B3" s="138" t="inlineStr">
+        <is>
+          <t>Sect</t>
+        </is>
+      </c>
+      <c r="C3" s="138" t="inlineStr">
+        <is>
+          <t>Metric category</t>
+        </is>
+      </c>
+      <c r="D3" s="138" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E3" s="138" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="F3" s="138" t="inlineStr">
+        <is>
+          <t>KPI name</t>
+        </is>
+      </c>
+      <c r="G3" s="138" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H3" s="138" t="inlineStr">
+        <is>
+          <t>Ladders to</t>
+        </is>
+      </c>
+      <c r="I3" s="138" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="J3" s="138" t="inlineStr">
+        <is>
+          <t>Freq</t>
+        </is>
+      </c>
+      <c r="K3" s="138" t="inlineStr">
+        <is>
+          <t>Budgeted</t>
+        </is>
+      </c>
+      <c r="L3" s="138" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="M3" s="138" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="N3" s="138" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="139" t="inlineStr">
+        <is>
+          <t>A — Inherited: org-KRA rows this team is on the hook for (live mirror — numbers live on the KPI Tracker tab; edit there)</t>
+        </is>
+      </c>
+      <c r="B4" s="119" t="n"/>
+      <c r="C4" s="119" t="n"/>
+      <c r="D4" s="119" t="n"/>
+      <c r="E4" s="119" t="n"/>
+      <c r="F4" s="119" t="n"/>
+      <c r="G4" s="119" t="n"/>
+      <c r="H4" s="119" t="n"/>
+      <c r="I4" s="119" t="n"/>
+      <c r="J4" s="119" t="n"/>
+      <c r="K4" s="119" t="n"/>
+      <c r="L4" s="119" t="n"/>
+      <c r="M4" s="119" t="n"/>
+      <c r="N4" s="119" t="n"/>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="140" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B5" s="140" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="141">
+        <f>IF('KPI Tracker FY26-27'!C18="","",'KPI Tracker FY26-27'!C18)</f>
+        <v/>
+      </c>
+      <c r="D5" s="140">
+        <f>IF('KPI Tracker FY26-27'!D18="","",'KPI Tracker FY26-27'!D18)</f>
+        <v/>
+      </c>
+      <c r="E5" s="140">
+        <f>IF('KPI Tracker FY26-27'!E18="","",'KPI Tracker FY26-27'!E18)</f>
+        <v/>
+      </c>
+      <c r="F5" s="142">
+        <f>IF('KPI Tracker FY26-27'!G18="","",'KPI Tracker FY26-27'!G18)</f>
+        <v/>
+      </c>
+      <c r="G5" s="141">
+        <f>IF('KPI Tracker FY26-27'!H18="","",'KPI Tracker FY26-27'!H18)</f>
+        <v/>
+      </c>
+      <c r="H5" s="141" t="inlineStr">
+        <is>
+          <t>inherited — via Functions (col K) · Central read: units-at-bar — how many of the 5 learning-domain units hold ≥ 90 (a count, not a blended average); each domain owns its own slice in its own view (FS &amp; CS Core wired, others as their views land).</t>
+        </is>
+      </c>
+      <c r="I5" s="140">
+        <f>IF('KPI Tracker FY26-27'!M18="","",'KPI Tracker FY26-27'!M18)</f>
+        <v/>
+      </c>
+      <c r="J5" s="140">
+        <f>IF('KPI Tracker FY26-27'!N18="","",'KPI Tracker FY26-27'!N18)</f>
+        <v/>
+      </c>
+      <c r="K5" s="140">
+        <f>IF('KPI Tracker FY26-27'!O18="","",'KPI Tracker FY26-27'!O18)</f>
+        <v/>
+      </c>
+      <c r="L5" s="140">
+        <f>IF('KPI Tracker FY26-27'!P18="","",'KPI Tracker FY26-27'!P18)</f>
+        <v/>
+      </c>
+      <c r="M5" s="140">
+        <f>IF('KPI Tracker FY26-27'!Q18="","",'KPI Tracker FY26-27'!Q18)</f>
+        <v/>
+      </c>
+      <c r="N5" s="141">
+        <f>IF('KPI Tracker FY26-27'!R18="","",'KPI Tracker FY26-27'!R18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="139" t="inlineStr">
+        <is>
+          <t>B — Owned: functional KPIs this team runs (budgets &amp; actuals live here) — Ladders-to key: direct = an org-KRA number · enabling = a dept §5 KPI · hygiene = guardrail by design</t>
+        </is>
+      </c>
+      <c r="B6" s="119" t="n"/>
+      <c r="C6" s="119" t="n"/>
+      <c r="D6" s="119" t="n"/>
+      <c r="E6" s="119" t="n"/>
+      <c r="F6" s="119" t="n"/>
+      <c r="G6" s="119" t="n"/>
+      <c r="H6" s="119" t="n"/>
+      <c r="I6" s="119" t="n"/>
+      <c r="J6" s="119" t="n"/>
+      <c r="K6" s="119" t="n"/>
+      <c r="L6" s="119" t="n"/>
+      <c r="M6" s="119" t="n"/>
+      <c r="N6" s="119" t="n"/>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" s="124" t="inlineStr">
+        <is>
+          <t>Business Ops — Shared Teams</t>
+        </is>
+      </c>
+      <c r="D7" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E7" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F7" s="125" t="inlineStr">
+        <is>
+          <t>Shared-Team Deliverables Landed</t>
+        </is>
+      </c>
+      <c r="G7" s="124" t="inlineStr">
+        <is>
+          <t>Of the deliverables the shared-resource teams (Product, Engineering, DA/DEs, Product Design) committed to content work for the period, the % delivered and accepted. Acceptance sits with the requesting unit — Central verifies the register, not the work.</t>
+        </is>
+      </c>
+      <c r="H7" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Stakeholder Alignment (§5) — the delivery contract with the embedded shared teams</t>
+        </is>
+      </c>
+      <c r="I7" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J7" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K7" s="123" t="n"/>
+      <c r="L7" s="123" t="n"/>
+      <c r="M7" s="126">
+        <f>IF(AND(ISNUMBER(K7),ISNUMBER(L7)),K7-L7,"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="124" t="inlineStr">
+        <is>
+          <t>Baseline first: Q1 builds the committed-deliverables register per shared team; budget set after one full cycle. Owned by the Business Ops lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="71" customHeight="1">
+      <c r="A8" s="123" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" s="124" t="inlineStr">
+        <is>
+          <t>Business Ops — Shared Teams</t>
+        </is>
+      </c>
+      <c r="D8" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E8" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F8" s="125" t="inlineStr">
+        <is>
+          <t>Shared-Team Spend vs Plan</t>
+        </is>
+      </c>
+      <c r="G8" s="124" t="inlineStr">
+        <is>
+          <t>Actual spend on shared-resource team allocations vs planned spend for the period. Reads over- and under-runs early; the value-for-spend judgment stays with the Business Ops owner at the monthly review.</t>
+        </is>
+      </c>
+      <c r="H8" s="124" t="inlineStr">
+        <is>
+          <t>enabling → dept Content Efficiency (§5) — the ₹ side of the shared-team delivery contract</t>
+        </is>
+      </c>
+      <c r="I8" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J8" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K8" s="123" t="n"/>
+      <c r="L8" s="123" t="n"/>
+      <c r="M8" s="126">
+        <f>IF(AND(ISNUMBER(K8),ISNUMBER(L8)),K8-L8,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="124" t="inlineStr">
+        <is>
+          <t>Baseline first: plan numbers come from the allocation agreed with each function head; tolerance band set after one full cycle. Owned by the Business Ops lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="71" customHeight="1">
+      <c r="A9" s="123" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" s="124" t="inlineStr">
+        <is>
+          <t>Agentic Content Platform</t>
+        </is>
+      </c>
+      <c r="D9" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F9" s="125" t="inlineStr">
+        <is>
+          <t>Shared Tool Adoption</t>
+        </is>
+      </c>
+      <c r="G9" s="124" t="inlineStr">
+        <is>
+          <t>% of shipped shared ACP tools (content-generation workflows, MCP servers, production pipelines built for all domains) that every learning-domain unit is publishing through within a month of shipping. Adopted = used in live production, not a trial.</t>
+        </is>
+      </c>
+      <c r="H9" s="124" t="inlineStr">
+        <is>
+          <t>enabling → tracker Agentic Production Coverage — adoption is how all units reach the 90 bar</t>
+        </is>
+      </c>
+      <c r="I9" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J9" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K9" s="123" t="n"/>
+      <c r="L9" s="123" t="n"/>
+      <c r="M9" s="126">
+        <f>IF(AND(ISNUMBER(K9),ISNUMBER(L9)),K9-L9,"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="124" t="inlineStr">
+        <is>
+          <t>Bar: ALL learning domains within a month of shipping — an unadopted shared tool is shelfware. Owned by the Business Ops lead (ACP builder hat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="123" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" s="124" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="D10" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E10" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F10" s="125" t="inlineStr">
+        <is>
+          <t>Check-ins Run</t>
+        </is>
+      </c>
+      <c r="G10" s="124" t="inlineStr">
+        <is>
+          <t>% of scheduled monthly unit check-ins with the HOD held on schedule, with the pre-read circulated a day before. Covers every sub-department and embedded function on the check-in calendar (~10 units).</t>
+        </is>
+      </c>
+      <c r="H10" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I10" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J10" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K10" s="123" t="n"/>
+      <c r="L10" s="123" t="n"/>
+      <c r="M10" s="126">
+        <f>IF(AND(ISNUMBER(K10),ISNUMBER(L10)),K10-L10,"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="124" t="inlineStr">
+        <is>
+          <t>Run by the PMO manager; unit PMs supply the pre-read inputs — orchestration here, the work stays with the units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="123" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" s="124" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="D11" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E11" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F11" s="125" t="inlineStr">
+        <is>
+          <t>Actions Closed</t>
+        </is>
+      </c>
+      <c r="G11" s="124" t="inlineStr">
+        <is>
+          <t>% of actions logged in a monthly check-in that are closed before that unit's next check-in. The follow-through half of the cadence — check-ins that close loops, not meetings that merely happen.</t>
+        </is>
+      </c>
+      <c r="H11" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I11" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J11" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K11" s="123" t="n"/>
+      <c r="L11" s="123" t="n"/>
+      <c r="M11" s="126">
+        <f>IF(AND(ISNUMBER(K11),ISNUMBER(L11)),K11-L11,"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="124" t="inlineStr">
+        <is>
+          <t>Run by the PMO manager. Deferred companions (spend → outcome map · tracker freshness · finance turnaround) join after the start set runs a cycle or two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="139" t="inlineStr">
+        <is>
+          <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
+        </is>
+      </c>
+      <c r="B12" s="119" t="n"/>
+      <c r="C12" s="119" t="n"/>
+      <c r="D12" s="119" t="n"/>
+      <c r="E12" s="119" t="n"/>
+      <c r="F12" s="119" t="n"/>
+      <c r="G12" s="119" t="n"/>
+      <c r="H12" s="119" t="n"/>
+      <c r="I12" s="119" t="n"/>
+      <c r="J12" s="119" t="n"/>
+      <c r="K12" s="119" t="n"/>
+      <c r="L12" s="119" t="n"/>
+      <c r="M12" s="119" t="n"/>
+      <c r="N12" s="119" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="140" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="140" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C13" s="141" t="inlineStr">
+        <is>
+          <t>Product, Engineering, Product Design &amp; Pedagogy function heads</t>
+        </is>
+      </c>
+      <c r="D13" s="140" t="n"/>
+      <c r="E13" s="140" t="n"/>
+      <c r="F13" s="142" t="inlineStr">
+        <is>
+          <t>Execution-management KPI tracking</t>
+        </is>
+      </c>
+      <c r="G13" s="141" t="inlineStr">
+        <is>
+          <t>Own execution KPIs (roadmap predictability, on-time delivery, budget adherence…) for teams embedded with us, tracked in their home functions — Central consumes the read at the monthly check-in; feeds Shared-Team Deliverables Landed (§7 ask).</t>
+        </is>
+      </c>
+      <c r="H13" s="141" t="n"/>
+      <c r="I13" s="140" t="n"/>
+      <c r="J13" s="140" t="n"/>
+      <c r="K13" s="140" t="n"/>
+      <c r="L13" s="140" t="n"/>
+      <c r="M13" s="140" t="n"/>
+      <c r="N13" s="141" t="n"/>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="140" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="140" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C14" s="141" t="inlineStr">
+        <is>
+          <t>Graphic Design &amp; Video Editing team heads</t>
+        </is>
+      </c>
+      <c r="D14" s="140" t="n"/>
+      <c r="E14" s="140" t="n"/>
+      <c r="F14" s="142" t="inlineStr">
+        <is>
+          <t>Creative delivery-management tracking</t>
+        </is>
+      </c>
+      <c r="G14" s="141" t="inlineStr">
+        <is>
+          <t>Delivery-management KPIs for the design &amp; video pipeline (on-time %, asset turnaround TAT, rework rate…) stay with the creative team heads; domain PMs manage day-to-day utilisation (FS view carries Creative Resource Utilisation) — §7 ask, reviewed quarterly.</t>
+        </is>
+      </c>
+      <c r="H14" s="141" t="n"/>
+      <c r="I14" s="140" t="n"/>
+      <c r="J14" s="140" t="n"/>
+      <c r="K14" s="140" t="n"/>
+      <c r="L14" s="140" t="n"/>
+      <c r="M14" s="140" t="n"/>
+      <c r="N14" s="141" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A6:N6"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="G14:N14"/>
+    <mergeCell ref="G13:N13"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Content–Central Section B: two All-Units utilisation rows (5 -> 7)
Creative + Cross-functional Resource Utilisation — All Units join
Business Ops — Shared Teams (%, Monthly, budgets blank, baseline-first
allocation register). Both ladder to their §5 PMO-lane dept KPIs, which
land a team owner for the first time; domain slices stay (FS row kept).
Org tracker and other views untouched; training-sheet html unchanged;
site b64 refreshed and republished.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -8135,7 +8135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8463,7 +8463,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="71" customHeight="1">
+    <row r="9" ht="92" customHeight="1">
       <c r="A9" s="123" t="n">
         <v>3</v>
       </c>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="C9" s="124" t="inlineStr">
         <is>
-          <t>Agentic Content Platform</t>
+          <t>Business Ops — Shared Teams</t>
         </is>
       </c>
       <c r="D9" s="123" t="inlineStr">
@@ -8489,17 +8489,17 @@
       </c>
       <c r="F9" s="125" t="inlineStr">
         <is>
-          <t>Shared Tool Adoption</t>
+          <t>Creative Resource Utilisation — All Units</t>
         </is>
       </c>
       <c r="G9" s="124" t="inlineStr">
         <is>
-          <t>% of shipped shared ACP tools (content-generation workflows, MCP servers, production pipelines built for all domains) that every learning-domain unit is publishing through within a month of shipping. Adopted = used in live production, not a trial.</t>
+          <t>Of the Graphic Designer &amp; Video Editor bandwidth allocated across all sub-departments, the % actually used against planned deliverables in the cycle. Central reads the aggregate and the skew — which units are stretched, which under-use; day-to-day management stays with unit PMs. Low = planning gaps · over = scope creep or under-resourcing.</t>
         </is>
       </c>
       <c r="H9" s="124" t="inlineStr">
         <is>
-          <t>enabling → tracker Agentic Production Coverage — adoption is how all units reach the 90 bar</t>
+          <t>enabling → dept Creative Resource Utilisation (§5, PMO lane) — the dept KPI lands its team owner here; domain views keep their own slice (FS: Creative Resource Utilisation Rate)</t>
         </is>
       </c>
       <c r="I9" s="123" t="inlineStr">
@@ -8520,11 +8520,11 @@
       </c>
       <c r="N9" s="124" t="inlineStr">
         <is>
-          <t>Bar: ALL learning domains within a month of shipping — an unadopted shared tool is shelfware. Owned by the Business Ops lead (ACP builder hat).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
+          <t>Baseline first: Q1 builds the allocation register per unit; unit PMs supply the reads, the PMO manager collects at the check-in, the Business Ops lead owns the judgment. FS Q1 Jul reference: A 100% — fully utilised, at times stretched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
       <c r="A10" s="123" t="n">
         <v>4</v>
       </c>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="C10" s="124" t="inlineStr">
         <is>
-          <t>PMO</t>
+          <t>Business Ops — Shared Teams</t>
         </is>
       </c>
       <c r="D10" s="123" t="inlineStr">
@@ -8550,17 +8550,17 @@
       </c>
       <c r="F10" s="125" t="inlineStr">
         <is>
-          <t>Check-ins Run</t>
+          <t>Cross-functional Resource Utilisation — All Units</t>
         </is>
       </c>
       <c r="G10" s="124" t="inlineStr">
         <is>
-          <t>% of scheduled monthly unit check-ins with the HOD held on schedule, with the pre-read circulated a day before. Covers every sub-department and embedded function on the check-in calendar (~10 units).</t>
+          <t>Of the embedded function bandwidth (Engineering, Product, Pedagogy, DA/DEs, Product Design) allocated into units, the % actually used on committed work in the cycle — across every sub-department and function. Read the same way: low = planning gaps · over = scope creep or under-resourcing.</t>
         </is>
       </c>
       <c r="H10" s="124" t="inlineStr">
         <is>
-          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+          <t>enabling → dept Cross-functional Resource Utilisation (§5, PMO lane) — the dept KPI lands its team owner here</t>
         </is>
       </c>
       <c r="I10" s="123" t="inlineStr">
@@ -8581,11 +8581,11 @@
       </c>
       <c r="N10" s="124" t="inlineStr">
         <is>
-          <t>Run by the PMO manager; unit PMs supply the pre-read inputs — orchestration here, the work stays with the units.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
+          <t>Baseline first: same allocation register; unit PMs supply the reads, the PMO manager collects at the check-in, the Business Ops lead owns the judgment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="71" customHeight="1">
       <c r="A11" s="123" t="n">
         <v>5</v>
       </c>
@@ -8596,7 +8596,7 @@
       </c>
       <c r="C11" s="124" t="inlineStr">
         <is>
-          <t>PMO</t>
+          <t>Agentic Content Platform</t>
         </is>
       </c>
       <c r="D11" s="123" t="inlineStr">
@@ -8611,17 +8611,17 @@
       </c>
       <c r="F11" s="125" t="inlineStr">
         <is>
-          <t>Actions Closed</t>
+          <t>Shared Tool Adoption</t>
         </is>
       </c>
       <c r="G11" s="124" t="inlineStr">
         <is>
-          <t>% of actions logged in a monthly check-in that are closed before that unit's next check-in. The follow-through half of the cadence — check-ins that close loops, not meetings that merely happen.</t>
+          <t>% of shipped shared ACP tools (content-generation workflows, MCP servers, production pipelines built for all domains) that every learning-domain unit is publishing through within a month of shipping. Adopted = used in live production, not a trial.</t>
         </is>
       </c>
       <c r="H11" s="124" t="inlineStr">
         <is>
-          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+          <t>enabling → tracker Agentic Production Coverage — adoption is how all units reach the 90 bar</t>
         </is>
       </c>
       <c r="I11" s="123" t="inlineStr">
@@ -8642,106 +8642,228 @@
       </c>
       <c r="N11" s="124" t="inlineStr">
         <is>
+          <t>Bar: ALL learning domains within a month of shipping — an unadopted shared tool is shelfware. Owned by the Business Ops lead (ACP builder hat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="123" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C12" s="124" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="D12" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E12" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F12" s="125" t="inlineStr">
+        <is>
+          <t>Check-ins Run</t>
+        </is>
+      </c>
+      <c r="G12" s="124" t="inlineStr">
+        <is>
+          <t>% of scheduled monthly unit check-ins with the HOD held on schedule, with the pre-read circulated a day before. Covers every sub-department and embedded function on the check-in calendar (~10 units).</t>
+        </is>
+      </c>
+      <c r="H12" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I12" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J12" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K12" s="123" t="n"/>
+      <c r="L12" s="123" t="n"/>
+      <c r="M12" s="126">
+        <f>IF(AND(ISNUMBER(K12),ISNUMBER(L12)),K12-L12,"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="124" t="inlineStr">
+        <is>
+          <t>Run by the PMO manager; unit PMs supply the pre-read inputs — orchestration here, the work stays with the units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="123" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C13" s="124" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="D13" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E13" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F13" s="125" t="inlineStr">
+        <is>
+          <t>Actions Closed</t>
+        </is>
+      </c>
+      <c r="G13" s="124" t="inlineStr">
+        <is>
+          <t>% of actions logged in a monthly check-in that are closed before that unit's next check-in. The follow-through half of the cadence — check-ins that close loops, not meetings that merely happen.</t>
+        </is>
+      </c>
+      <c r="H13" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I13" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J13" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K13" s="123" t="n"/>
+      <c r="L13" s="123" t="n"/>
+      <c r="M13" s="126">
+        <f>IF(AND(ISNUMBER(K13),ISNUMBER(L13)),K13-L13,"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="124" t="inlineStr">
+        <is>
           <t>Run by the PMO manager. Deferred companions (spend → outcome map · tracker freshness · finance turnaround) join after the start set runs a cycle or two.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="139" t="inlineStr">
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="139" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B12" s="119" t="n"/>
-      <c r="C12" s="119" t="n"/>
-      <c r="D12" s="119" t="n"/>
-      <c r="E12" s="119" t="n"/>
-      <c r="F12" s="119" t="n"/>
-      <c r="G12" s="119" t="n"/>
-      <c r="H12" s="119" t="n"/>
-      <c r="I12" s="119" t="n"/>
-      <c r="J12" s="119" t="n"/>
-      <c r="K12" s="119" t="n"/>
-      <c r="L12" s="119" t="n"/>
-      <c r="M12" s="119" t="n"/>
-      <c r="N12" s="119" t="n"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="140" t="n">
+      <c r="B14" s="119" t="n"/>
+      <c r="C14" s="119" t="n"/>
+      <c r="D14" s="119" t="n"/>
+      <c r="E14" s="119" t="n"/>
+      <c r="F14" s="119" t="n"/>
+      <c r="G14" s="119" t="n"/>
+      <c r="H14" s="119" t="n"/>
+      <c r="I14" s="119" t="n"/>
+      <c r="J14" s="119" t="n"/>
+      <c r="K14" s="119" t="n"/>
+      <c r="L14" s="119" t="n"/>
+      <c r="M14" s="119" t="n"/>
+      <c r="N14" s="119" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="140" t="n">
         <v>1</v>
       </c>
-      <c r="B13" s="140" t="inlineStr">
+      <c r="B15" s="140" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C13" s="141" t="inlineStr">
+      <c r="C15" s="141" t="inlineStr">
         <is>
           <t>Product, Engineering, Product Design &amp; Pedagogy function heads</t>
         </is>
       </c>
-      <c r="D13" s="140" t="n"/>
-      <c r="E13" s="140" t="n"/>
-      <c r="F13" s="142" t="inlineStr">
+      <c r="D15" s="140" t="n"/>
+      <c r="E15" s="140" t="n"/>
+      <c r="F15" s="142" t="inlineStr">
         <is>
           <t>Execution-management KPI tracking</t>
         </is>
       </c>
-      <c r="G13" s="141" t="inlineStr">
+      <c r="G15" s="141" t="inlineStr">
         <is>
           <t>Own execution KPIs (roadmap predictability, on-time delivery, budget adherence…) for teams embedded with us, tracked in their home functions — Central consumes the read at the monthly check-in; feeds Shared-Team Deliverables Landed (§7 ask).</t>
         </is>
       </c>
-      <c r="H13" s="141" t="n"/>
-      <c r="I13" s="140" t="n"/>
-      <c r="J13" s="140" t="n"/>
-      <c r="K13" s="140" t="n"/>
-      <c r="L13" s="140" t="n"/>
-      <c r="M13" s="140" t="n"/>
-      <c r="N13" s="141" t="n"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="140" t="n">
+      <c r="H15" s="141" t="n"/>
+      <c r="I15" s="140" t="n"/>
+      <c r="J15" s="140" t="n"/>
+      <c r="K15" s="140" t="n"/>
+      <c r="L15" s="140" t="n"/>
+      <c r="M15" s="140" t="n"/>
+      <c r="N15" s="141" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="140" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="140" t="inlineStr">
+      <c r="B16" s="140" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C14" s="141" t="inlineStr">
+      <c r="C16" s="141" t="inlineStr">
         <is>
           <t>Graphic Design &amp; Video Editing team heads</t>
         </is>
       </c>
-      <c r="D14" s="140" t="n"/>
-      <c r="E14" s="140" t="n"/>
-      <c r="F14" s="142" t="inlineStr">
+      <c r="D16" s="140" t="n"/>
+      <c r="E16" s="140" t="n"/>
+      <c r="F16" s="142" t="inlineStr">
         <is>
           <t>Creative delivery-management tracking</t>
         </is>
       </c>
-      <c r="G14" s="141" t="inlineStr">
+      <c r="G16" s="141" t="inlineStr">
         <is>
           <t>Delivery-management KPIs for the design &amp; video pipeline (on-time %, asset turnaround TAT, rework rate…) stay with the creative team heads; domain PMs manage day-to-day utilisation (FS view carries Creative Resource Utilisation) — §7 ask, reviewed quarterly.</t>
         </is>
       </c>
-      <c r="H14" s="141" t="n"/>
-      <c r="I14" s="140" t="n"/>
-      <c r="J14" s="140" t="n"/>
-      <c r="K14" s="140" t="n"/>
-      <c r="L14" s="140" t="n"/>
-      <c r="M14" s="140" t="n"/>
-      <c r="N14" s="141" t="n"/>
+      <c r="H16" s="141" t="n"/>
+      <c r="I16" s="140" t="n"/>
+      <c r="J16" s="140" t="n"/>
+      <c r="K16" s="140" t="n"/>
+      <c r="L16" s="140" t="n"/>
+      <c r="M16" s="140" t="n"/>
+      <c r="N16" s="141" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A6:N6"/>
-    <mergeCell ref="A12:N12"/>
     <mergeCell ref="A4:N4"/>
+    <mergeCell ref="G15:N15"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="G14:N14"/>
-    <mergeCell ref="G13:N13"/>
+    <mergeCell ref="G16:N16"/>
+    <mergeCell ref="A14:N14"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Team Ops & People category: PM-layer metric set in FS & CSI; Central worklog hygiene row
Executive Ops renamed and rebuilt in both domain views — six rows replace
Operations & Growth Cost (Cost of Operations, Roadmap Items Completion,
Hires Made, Cost per Hire, Team Retention Rate, Power Performers Created),
KPIs cascade Lead → PM. Content–Central PMO gains Worklog & Status Hygiene
— All Units (fed → held → closed pipeline). Site asserts/ranges updated
(FS B 29); 🗺️ republished same URL.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -4252,7 +4252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="N15" s="124" t="inlineStr"/>
     </row>
-    <row r="16" ht="45" customHeight="1">
+    <row r="16" ht="92" customHeight="1">
       <c r="A16" s="123" t="n">
         <v>3</v>
       </c>
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C16" s="124" t="inlineStr">
         <is>
-          <t>Executive Ops</t>
+          <t>Team Ops &amp; People</t>
         </is>
       </c>
       <c r="D16" s="123" t="inlineStr">
@@ -5029,12 +5029,12 @@
       </c>
       <c r="F16" s="125" t="inlineStr">
         <is>
-          <t>Operations &amp; Growth Cost</t>
+          <t>Cost of Operations</t>
         </is>
       </c>
       <c r="G16" s="124" t="inlineStr">
         <is>
-          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+          <t>Monthly cost of running the team's operating rhythm: manager–reportee one-on-ones, roadmap reviews (Head-approved), standups &amp; learning hours, monthly check-in scheduling &amp; documentation, team assets (laptops, systems), ClickUp adoption &amp; status freshness, worklog capture, newsletters, team outings and cycle-wise appraisals — plus operational-efficiency and market-analysis work. Worklog capture is the load-bearing activity: it is what makes deliverable costing computable.</t>
         </is>
       </c>
       <c r="H16" s="124" t="inlineStr">
@@ -5058,139 +5058,448 @@
         <f>IF(AND(ISNUMBER(K16),ISNUMBER(L16)),K16-L16,"")</f>
         <v/>
       </c>
-      <c r="N16" s="124" t="inlineStr"/>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="118" t="inlineStr">
+      <c r="N16" s="124" t="inlineStr">
+        <is>
+          <t>Replaces Operations &amp; Growth Cost (no baseline yet) — worklog capture builds the first read. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="123" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C17" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D17" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E17" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F17" s="125" t="inlineStr">
+        <is>
+          <t>Roadmap Items Completion</t>
+        </is>
+      </c>
+      <c r="G17" s="124" t="inlineStr">
+        <is>
+          <t>Of the roadmap items committed for the cycle — reviewed in the roadmap meetings the PM schedules and approved by the Head — the % completed. The execution-predictability read for the team's own plan.</t>
+        </is>
+      </c>
+      <c r="H17" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — execution-predictability guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I17" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J17" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K17" s="123" t="n"/>
+      <c r="L17" s="123" t="n"/>
+      <c r="M17" s="126">
+        <f>IF(AND(ISNUMBER(K17),ISNUMBER(L17)),K17-L17,"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="124" t="inlineStr">
+        <is>
+          <t>Cycle-anchored: the commitment is the Head-approved cycle roadmap; the % is read monthly as items land. Run by the team's PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="123" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C18" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D18" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E18" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F18" s="125" t="inlineStr">
+        <is>
+          <t>Hires Made</t>
+        </is>
+      </c>
+      <c r="G18" s="124" t="inlineStr">
+        <is>
+          <t>Offers joined against the team's approved hiring plan for the period. Reads whether the team is growing at the planned pace.</t>
+        </is>
+      </c>
+      <c r="H18" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — hiring-plan guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I18" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="J18" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K18" s="123" t="n"/>
+      <c r="L18" s="123" t="n"/>
+      <c r="M18" s="126">
+        <f>IF(AND(ISNUMBER(K18),ISNUMBER(L18)),K18-L18,"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="124" t="inlineStr">
+        <is>
+          <t>Budget = the approved hiring plan. Run by the team's PM; hiring decisions stay with the Lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="123" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C19" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D19" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E19" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F19" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Hire</t>
+        </is>
+      </c>
+      <c r="G19" s="124" t="inlineStr">
+        <is>
+          <t>Average cost per closed hire — sourcing, interview bandwidth and onboarding effort attributed to hiring for this team.</t>
+        </is>
+      </c>
+      <c r="H19" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — hiring-efficiency guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I19" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="J19" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K19" s="123" t="n"/>
+      <c r="L19" s="123" t="n"/>
+      <c r="M19" s="126">
+        <f>IF(AND(ISNUMBER(K19),ISNUMBER(L19)),K19-L19,"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="124" t="inlineStr">
+        <is>
+          <t>Hiring cost split out of the old Operations &amp; Growth Cost row — worklogs attribute the interview bandwidth. Run by the team's PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="71" customHeight="1">
+      <c r="A20" s="123" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C20" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D20" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E20" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F20" s="125" t="inlineStr">
+        <is>
+          <t>Team Retention Rate</t>
+        </is>
+      </c>
+      <c r="G20" s="124" t="inlineStr">
+        <is>
+          <t>% of cycle-start team members still on the team at the appraisal cycle's end, on a trailing 12-month window. Internal transfers don't count against the team; regrettable exits are flagged by the Lead in the remark.</t>
+        </is>
+      </c>
+      <c r="H20" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — team-health guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I20" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J20" s="123" t="inlineStr">
+        <is>
+          <t>Per appraisal cycle</t>
+        </is>
+      </c>
+      <c r="K20" s="123" t="n"/>
+      <c r="L20" s="123" t="n"/>
+      <c r="M20" s="126">
+        <f>IF(AND(ISNUMBER(K20),ISNUMBER(L20)),K20-L20,"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="124" t="inlineStr">
+        <is>
+          <t>Trailing 12 months smooths small-team noise (one exit is a big % swing). Lead-driven outcome; the PM carries the machinery and the number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="123" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C21" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D21" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E21" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F21" s="125" t="inlineStr">
+        <is>
+          <t>Power Performers Created</t>
+        </is>
+      </c>
+      <c r="G21" s="124" t="inlineStr">
+        <is>
+          <t>Team members newly reaching the top appraisal band in the cycle-wise appraisal. The direct metric for 'developing the best (mentoring subordinates)'.</t>
+        </is>
+      </c>
+      <c r="H21" s="124" t="inlineStr">
+        <is>
+          <t>enabling → the §5 'developing the best (mentoring subordinates)' intent — its first direct metric</t>
+        </is>
+      </c>
+      <c r="I21" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="J21" s="123" t="inlineStr">
+        <is>
+          <t>Per appraisal cycle</t>
+        </is>
+      </c>
+      <c r="K21" s="123" t="n"/>
+      <c r="L21" s="123" t="n"/>
+      <c r="M21" s="126">
+        <f>IF(AND(ISNUMBER(K21),ISNUMBER(L21)),K21-L21,"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="124" t="inlineStr">
+        <is>
+          <t>Top band per the cycle-wise appraisal; mentoring by managers and the Lead is the driver. Lead-driven outcome; the PM runs the appraisal machinery and carries the number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="118" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B17" s="119" t="n"/>
-      <c r="C17" s="119" t="n"/>
-      <c r="D17" s="119" t="n"/>
-      <c r="E17" s="119" t="n"/>
-      <c r="F17" s="119" t="n"/>
-      <c r="G17" s="119" t="n"/>
-      <c r="H17" s="119" t="n"/>
-      <c r="I17" s="119" t="n"/>
-      <c r="J17" s="119" t="n"/>
-      <c r="K17" s="119" t="n"/>
-      <c r="L17" s="119" t="n"/>
-      <c r="M17" s="119" t="n"/>
-      <c r="N17" s="119" t="n"/>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="120" t="n">
+      <c r="B22" s="119" t="n"/>
+      <c r="C22" s="119" t="n"/>
+      <c r="D22" s="119" t="n"/>
+      <c r="E22" s="119" t="n"/>
+      <c r="F22" s="119" t="n"/>
+      <c r="G22" s="119" t="n"/>
+      <c r="H22" s="119" t="n"/>
+      <c r="I22" s="119" t="n"/>
+      <c r="J22" s="119" t="n"/>
+      <c r="K22" s="119" t="n"/>
+      <c r="L22" s="119" t="n"/>
+      <c r="M22" s="119" t="n"/>
+      <c r="N22" s="119" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="120" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="120" t="inlineStr">
+      <c r="B23" s="120" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C18" s="121" t="inlineStr">
+      <c r="C23" s="121" t="inlineStr">
         <is>
           <t>Program Ops</t>
         </is>
       </c>
-      <c r="D18" s="120" t="n"/>
-      <c r="E18" s="120" t="n"/>
-      <c r="F18" s="122" t="inlineStr">
+      <c r="D23" s="120" t="n"/>
+      <c r="E23" s="120" t="n"/>
+      <c r="F23" s="122" t="inlineStr">
         <is>
           <t>Conduction adherence</t>
         </is>
       </c>
-      <c r="G18" s="121" t="inlineStr">
+      <c r="G23" s="121" t="inlineStr">
         <is>
           <t>Zero schedule deviation on lectures / quizzes / assessments + attendance drive — feeds Program Delivery Gap &amp; Journey Step Health (§7 ask; exact thresholds pending).</t>
         </is>
       </c>
-      <c r="H18" s="121" t="n"/>
-      <c r="I18" s="120" t="n"/>
-      <c r="J18" s="120" t="n"/>
-      <c r="K18" s="120" t="n"/>
-      <c r="L18" s="120" t="n"/>
-      <c r="M18" s="120" t="n"/>
-      <c r="N18" s="121" t="n"/>
-    </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="120" t="n">
+      <c r="H23" s="121" t="n"/>
+      <c r="I23" s="120" t="n"/>
+      <c r="J23" s="120" t="n"/>
+      <c r="K23" s="120" t="n"/>
+      <c r="L23" s="120" t="n"/>
+      <c r="M23" s="120" t="n"/>
+      <c r="N23" s="121" t="n"/>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="120" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="120" t="inlineStr">
+      <c r="B24" s="120" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C19" s="121" t="inlineStr">
+      <c r="C24" s="121" t="inlineStr">
         <is>
           <t>Instructors dept</t>
         </is>
       </c>
-      <c r="D19" s="120" t="n"/>
-      <c r="E19" s="120" t="n"/>
-      <c r="F19" s="122" t="inlineStr">
+      <c r="D24" s="120" t="n"/>
+      <c r="E24" s="120" t="n"/>
+      <c r="F24" s="122" t="inlineStr">
         <is>
           <t>Learning-assets SLA</t>
         </is>
       </c>
-      <c r="G19" s="121" t="inlineStr">
+      <c r="G24" s="121" t="inlineStr">
         <is>
           <t>PPT + recorded video ready &amp; loaded ≥1 month ahead of delivery — feeds the assets leg of Program Delivery Gap.</t>
         </is>
       </c>
-      <c r="H19" s="121" t="n"/>
-      <c r="I19" s="120" t="n"/>
-      <c r="J19" s="120" t="n"/>
-      <c r="K19" s="120" t="n"/>
-      <c r="L19" s="120" t="n"/>
-      <c r="M19" s="120" t="n"/>
-      <c r="N19" s="121" t="n"/>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="120" t="n">
+      <c r="H24" s="121" t="n"/>
+      <c r="I24" s="120" t="n"/>
+      <c r="J24" s="120" t="n"/>
+      <c r="K24" s="120" t="n"/>
+      <c r="L24" s="120" t="n"/>
+      <c r="M24" s="120" t="n"/>
+      <c r="N24" s="121" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="120" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="120" t="inlineStr">
+      <c r="B25" s="120" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C20" s="121" t="inlineStr">
+      <c r="C25" s="121" t="inlineStr">
         <is>
           <t>Univ Relations</t>
         </is>
       </c>
-      <c r="D20" s="120" t="n"/>
-      <c r="E20" s="120" t="n"/>
-      <c r="F20" s="122" t="inlineStr">
+      <c r="D25" s="120" t="n"/>
+      <c r="E25" s="120" t="n"/>
+      <c r="F25" s="122" t="inlineStr">
         <is>
           <t>University response windows</t>
         </is>
       </c>
-      <c r="G20" s="121" t="inlineStr">
+      <c r="G25" s="121" t="inlineStr">
         <is>
           <t>BOS meeting windows + response SLAs on university communications — feeds BOS Credit Acceptance &amp; University Communication TAT.</t>
         </is>
       </c>
-      <c r="H20" s="121" t="n"/>
-      <c r="I20" s="120" t="n"/>
-      <c r="J20" s="120" t="n"/>
-      <c r="K20" s="120" t="n"/>
-      <c r="L20" s="120" t="n"/>
-      <c r="M20" s="120" t="n"/>
-      <c r="N20" s="121" t="n"/>
+      <c r="H25" s="121" t="n"/>
+      <c r="I25" s="120" t="n"/>
+      <c r="J25" s="120" t="n"/>
+      <c r="K25" s="120" t="n"/>
+      <c r="L25" s="120" t="n"/>
+      <c r="M25" s="120" t="n"/>
+      <c r="N25" s="121" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="G18:N18"/>
-    <mergeCell ref="G20:N20"/>
+    <mergeCell ref="A22:N22"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="G19:N19"/>
+    <mergeCell ref="G25:N25"/>
+    <mergeCell ref="G24:N24"/>
     <mergeCell ref="A13:N13"/>
+    <mergeCell ref="G23:N23"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5204,7 +5513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7834,7 +8143,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="45" customHeight="1">
+    <row r="47" ht="92" customHeight="1">
       <c r="A47" s="123" t="n">
         <v>23</v>
       </c>
@@ -7845,7 +8154,7 @@
       </c>
       <c r="C47" s="124" t="inlineStr">
         <is>
-          <t>Executive Ops</t>
+          <t>Team Ops &amp; People</t>
         </is>
       </c>
       <c r="D47" s="123" t="inlineStr">
@@ -7860,12 +8169,12 @@
       </c>
       <c r="F47" s="125" t="inlineStr">
         <is>
-          <t>Operations &amp; Growth Cost</t>
+          <t>Cost of Operations</t>
         </is>
       </c>
       <c r="G47" s="124" t="inlineStr">
         <is>
-          <t>Average cost across executive ops, operational efficiency, market analysis and hiring activities. Tracked at team scope, not per product.</t>
+          <t>Monthly cost of running the team's operating rhythm: manager–reportee one-on-ones, roadmap reviews (Head-approved), standups &amp; learning hours, monthly check-in scheduling &amp; documentation, team assets (laptops, systems), ClickUp adoption &amp; status freshness, worklog capture, newsletters, team outings and cycle-wise appraisals — plus operational-efficiency and market-analysis work. Worklog capture is the load-bearing activity: it is what makes deliverable costing computable.</t>
         </is>
       </c>
       <c r="H47" s="124" t="inlineStr">
@@ -7891,7 +8200,7 @@
       </c>
       <c r="N47" s="124" t="inlineStr">
         <is>
-          <t>Q1 Jul: A ₹300,863.</t>
+          <t>Replaces Operations &amp; Growth Cost — Jul A ₹300,863 spans ops + hiring; worklog capture splits it from next month. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
         </is>
       </c>
     </row>
@@ -7906,7 +8215,7 @@
       </c>
       <c r="C48" s="124" t="inlineStr">
         <is>
-          <t>Executive Ops</t>
+          <t>Team Ops &amp; People</t>
         </is>
       </c>
       <c r="D48" s="123" t="inlineStr">
@@ -7921,17 +8230,17 @@
       </c>
       <c r="F48" s="125" t="inlineStr">
         <is>
-          <t>Creative Resource Utilisation Rate</t>
+          <t>Roadmap Items Completion</t>
         </is>
       </c>
       <c r="G48" s="124" t="inlineStr">
         <is>
-          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
+          <t>Of the roadmap items committed for the cycle — reviewed in the roadmap meetings the PM schedules and approved by the Head — the % completed. The execution-predictability read for the team's own plan.</t>
         </is>
       </c>
       <c r="H48" s="124" t="inlineStr">
         <is>
-          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
+          <t>hygiene — execution-predictability guardrail; no org ladder by design</t>
         </is>
       </c>
       <c r="I48" s="123" t="inlineStr">
@@ -7952,176 +8261,481 @@
       </c>
       <c r="N48" s="124" t="inlineStr">
         <is>
+          <t>Cycle-anchored: the commitment is the Head-approved cycle roadmap; the % is read monthly as items land. Run by the team's PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="123" t="n">
+        <v>25</v>
+      </c>
+      <c r="B49" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C49" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D49" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E49" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F49" s="125" t="inlineStr">
+        <is>
+          <t>Hires Made</t>
+        </is>
+      </c>
+      <c r="G49" s="124" t="inlineStr">
+        <is>
+          <t>Offers joined against the team's approved hiring plan for the period. Reads whether the team is growing at the planned pace.</t>
+        </is>
+      </c>
+      <c r="H49" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — hiring-plan guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I49" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="J49" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K49" s="123" t="n"/>
+      <c r="L49" s="123" t="n"/>
+      <c r="M49" s="126">
+        <f>IF(AND(ISNUMBER(K49),ISNUMBER(L49)),K49-L49,"")</f>
+        <v/>
+      </c>
+      <c r="N49" s="124" t="inlineStr">
+        <is>
+          <t>Budget = the approved hiring plan. Run by the team's PM; hiring decisions stay with the Lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="A50" s="123" t="n">
+        <v>26</v>
+      </c>
+      <c r="B50" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C50" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D50" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E50" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F50" s="125" t="inlineStr">
+        <is>
+          <t>Cost per Hire</t>
+        </is>
+      </c>
+      <c r="G50" s="124" t="inlineStr">
+        <is>
+          <t>Average cost per closed hire — sourcing, interview bandwidth and onboarding effort attributed to hiring for this team.</t>
+        </is>
+      </c>
+      <c r="H50" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — hiring-efficiency guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I50" s="123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="J50" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K50" s="123" t="n"/>
+      <c r="L50" s="123" t="n"/>
+      <c r="M50" s="126">
+        <f>IF(AND(ISNUMBER(K50),ISNUMBER(L50)),K50-L50,"")</f>
+        <v/>
+      </c>
+      <c r="N50" s="124" t="inlineStr">
+        <is>
+          <t>Hiring cost split out of the old Operations &amp; Growth Cost row — worklogs attribute the interview bandwidth. Run by the team's PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="71" customHeight="1">
+      <c r="A51" s="123" t="n">
+        <v>27</v>
+      </c>
+      <c r="B51" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C51" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D51" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E51" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F51" s="125" t="inlineStr">
+        <is>
+          <t>Team Retention Rate</t>
+        </is>
+      </c>
+      <c r="G51" s="124" t="inlineStr">
+        <is>
+          <t>% of cycle-start team members still on the team at the appraisal cycle's end, on a trailing 12-month window. Internal transfers don't count against the team; regrettable exits are flagged by the Lead in the remark.</t>
+        </is>
+      </c>
+      <c r="H51" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — team-health guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I51" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J51" s="123" t="inlineStr">
+        <is>
+          <t>Per appraisal cycle</t>
+        </is>
+      </c>
+      <c r="K51" s="123" t="n"/>
+      <c r="L51" s="123" t="n"/>
+      <c r="M51" s="126">
+        <f>IF(AND(ISNUMBER(K51),ISNUMBER(L51)),K51-L51,"")</f>
+        <v/>
+      </c>
+      <c r="N51" s="124" t="inlineStr">
+        <is>
+          <t>Trailing 12 months smooths small-team noise (one exit is a big % swing). Lead-driven outcome; the PM carries the machinery and the number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="A52" s="123" t="n">
+        <v>28</v>
+      </c>
+      <c r="B52" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C52" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D52" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E52" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F52" s="125" t="inlineStr">
+        <is>
+          <t>Power Performers Created</t>
+        </is>
+      </c>
+      <c r="G52" s="124" t="inlineStr">
+        <is>
+          <t>Team members newly reaching the top appraisal band in the cycle-wise appraisal. The direct metric for 'developing the best (mentoring subordinates)'.</t>
+        </is>
+      </c>
+      <c r="H52" s="124" t="inlineStr">
+        <is>
+          <t>enabling → the §5 'developing the best (mentoring subordinates)' intent — its first direct metric</t>
+        </is>
+      </c>
+      <c r="I52" s="123" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="J52" s="123" t="inlineStr">
+        <is>
+          <t>Per appraisal cycle</t>
+        </is>
+      </c>
+      <c r="K52" s="123" t="n"/>
+      <c r="L52" s="123" t="n"/>
+      <c r="M52" s="126">
+        <f>IF(AND(ISNUMBER(K52),ISNUMBER(L52)),K52-L52,"")</f>
+        <v/>
+      </c>
+      <c r="N52" s="124" t="inlineStr">
+        <is>
+          <t>Top band per the cycle-wise appraisal; mentoring by managers and the Lead is the driver. Lead-driven outcome; the PM runs the appraisal machinery and carries the number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="58" customHeight="1">
+      <c r="A53" s="123" t="n">
+        <v>29</v>
+      </c>
+      <c r="B53" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C53" s="124" t="inlineStr">
+        <is>
+          <t>Team Ops &amp; People</t>
+        </is>
+      </c>
+      <c r="D53" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E53" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F53" s="125" t="inlineStr">
+        <is>
+          <t>Creative Resource Utilisation Rate</t>
+        </is>
+      </c>
+      <c r="G53" s="124" t="inlineStr">
+        <is>
+          <t>% of allocated Graphic Designer and Video Editor bandwidth utilised against planned branding and content-asset deliverables within a cycle. Primarily tracked and managed by Project Managers.</t>
+        </is>
+      </c>
+      <c r="H53" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — creative bandwidth guardrail (PM-managed); no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I53" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J53" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K53" s="123" t="n"/>
+      <c r="L53" s="123" t="n"/>
+      <c r="M53" s="126">
+        <f>IF(AND(ISNUMBER(K53),ISNUMBER(L53)),K53-L53,"")</f>
+        <v/>
+      </c>
+      <c r="N53" s="124" t="inlineStr">
+        <is>
           <t>Q1 Jul: A 100% — fully utilised, at times stretched.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="129" t="inlineStr">
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="129" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B49" s="119" t="n"/>
-      <c r="C49" s="119" t="n"/>
-      <c r="D49" s="119" t="n"/>
-      <c r="E49" s="119" t="n"/>
-      <c r="F49" s="119" t="n"/>
-      <c r="G49" s="119" t="n"/>
-      <c r="H49" s="119" t="n"/>
-      <c r="I49" s="119" t="n"/>
-      <c r="J49" s="119" t="n"/>
-      <c r="K49" s="119" t="n"/>
-      <c r="L49" s="119" t="n"/>
-      <c r="M49" s="119" t="n"/>
-      <c r="N49" s="119" t="n"/>
-    </row>
-    <row r="50" ht="40" customHeight="1">
-      <c r="A50" s="130" t="n">
+      <c r="B54" s="119" t="n"/>
+      <c r="C54" s="119" t="n"/>
+      <c r="D54" s="119" t="n"/>
+      <c r="E54" s="119" t="n"/>
+      <c r="F54" s="119" t="n"/>
+      <c r="G54" s="119" t="n"/>
+      <c r="H54" s="119" t="n"/>
+      <c r="I54" s="119" t="n"/>
+      <c r="J54" s="119" t="n"/>
+      <c r="K54" s="119" t="n"/>
+      <c r="L54" s="119" t="n"/>
+      <c r="M54" s="119" t="n"/>
+      <c r="N54" s="119" t="n"/>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="130" t="n">
         <v>1</v>
       </c>
-      <c r="B50" s="130" t="inlineStr">
+      <c r="B55" s="130" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C50" s="131" t="inlineStr">
+      <c r="C55" s="131" t="inlineStr">
         <is>
           <t>Assessments team</t>
         </is>
       </c>
-      <c r="D50" s="130" t="n"/>
-      <c r="E50" s="130" t="n"/>
-      <c r="F50" s="132" t="inlineStr">
+      <c r="D55" s="130" t="n"/>
+      <c r="E55" s="130" t="n"/>
+      <c r="F55" s="132" t="inlineStr">
         <is>
           <t>Assessment blueprints per cycle</t>
         </is>
       </c>
-      <c r="G50" s="131" t="inlineStr">
+      <c r="G55" s="131" t="inlineStr">
         <is>
           <t>Skill-assessment blueprints + knowledge points shared before authoring each cycle; changes communicated — feeds Content–Assessment Alignment (§7 ask).</t>
         </is>
       </c>
-      <c r="H50" s="131" t="n"/>
-      <c r="I50" s="130" t="n"/>
-      <c r="J50" s="130" t="n"/>
-      <c r="K50" s="130" t="n"/>
-      <c r="L50" s="130" t="n"/>
-      <c r="M50" s="130" t="n"/>
-      <c r="N50" s="131" t="n"/>
-    </row>
-    <row r="51" ht="40" customHeight="1">
-      <c r="A51" s="130" t="n">
+      <c r="H55" s="131" t="n"/>
+      <c r="I55" s="130" t="n"/>
+      <c r="J55" s="130" t="n"/>
+      <c r="K55" s="130" t="n"/>
+      <c r="L55" s="130" t="n"/>
+      <c r="M55" s="130" t="n"/>
+      <c r="N55" s="131" t="n"/>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="130" t="n">
         <v>2</v>
       </c>
-      <c r="B51" s="130" t="inlineStr">
+      <c r="B56" s="130" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C51" s="131" t="inlineStr">
+      <c r="C56" s="131" t="inlineStr">
         <is>
           <t>Learning Platform / DA-DEs</t>
         </is>
       </c>
-      <c r="D51" s="130" t="n"/>
-      <c r="E51" s="130" t="n"/>
-      <c r="F51" s="132" t="inlineStr">
+      <c r="D56" s="130" t="n"/>
+      <c r="E56" s="130" t="n"/>
+      <c r="F56" s="132" t="inlineStr">
         <is>
           <t>Engagement &amp; LE dashboards</t>
         </is>
       </c>
-      <c r="G51" s="131" t="inlineStr">
+      <c r="G56" s="131" t="inlineStr">
         <is>
           <t>Monthly LE + engagement-matrix cuts per domain — budgets for Cell Migration and module-quiz Bands come from here. Course-completion cuts included as a read-only view: completion is conduction-driven (Program Ops); the team's owned stickiness KPIs are Learner-Accessed Completion + Practice Attempt-to-Completion.</t>
         </is>
       </c>
-      <c r="H51" s="131" t="n"/>
-      <c r="I51" s="130" t="n"/>
-      <c r="J51" s="130" t="n"/>
-      <c r="K51" s="130" t="n"/>
-      <c r="L51" s="130" t="n"/>
-      <c r="M51" s="130" t="n"/>
-      <c r="N51" s="131" t="n"/>
-    </row>
-    <row r="52" ht="40" customHeight="1">
-      <c r="A52" s="130" t="n">
+      <c r="H56" s="131" t="n"/>
+      <c r="I56" s="130" t="n"/>
+      <c r="J56" s="130" t="n"/>
+      <c r="K56" s="130" t="n"/>
+      <c r="L56" s="130" t="n"/>
+      <c r="M56" s="130" t="n"/>
+      <c r="N56" s="131" t="n"/>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="130" t="n">
         <v>3</v>
       </c>
-      <c r="B52" s="130" t="inlineStr">
+      <c r="B57" s="130" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C52" s="131" t="inlineStr">
+      <c r="C57" s="131" t="inlineStr">
         <is>
           <t>Learning Platform (PMs + Engineering)</t>
         </is>
       </c>
-      <c r="D52" s="130" t="n"/>
-      <c r="E52" s="130" t="n"/>
-      <c r="F52" s="132" t="inlineStr">
+      <c r="D57" s="130" t="n"/>
+      <c r="E57" s="130" t="n"/>
+      <c r="F57" s="132" t="inlineStr">
         <is>
           <t>Domain-specific capability build</t>
         </is>
       </c>
-      <c r="G52" s="131" t="inlineStr">
+      <c r="G57" s="131" t="inlineStr">
         <is>
           <t>Build slots for domain-raised capabilities and evaluation environments — SMEs here raise and accept; PMs + Engineering build. Boundary: generic/reusable capability = Learning Platform lane (product-owned) · domain-specific instance = KPI here, in Learning Domains · ACP = content-facing production pipelines, domain product work = learner-facing systems.</t>
         </is>
       </c>
-      <c r="H52" s="131" t="n"/>
-      <c r="I52" s="130" t="n"/>
-      <c r="J52" s="130" t="n"/>
-      <c r="K52" s="130" t="n"/>
-      <c r="L52" s="130" t="n"/>
-      <c r="M52" s="130" t="n"/>
-      <c r="N52" s="131" t="n"/>
-    </row>
-    <row r="53" ht="40" customHeight="1">
-      <c r="A53" s="130" t="n">
+      <c r="H57" s="131" t="n"/>
+      <c r="I57" s="130" t="n"/>
+      <c r="J57" s="130" t="n"/>
+      <c r="K57" s="130" t="n"/>
+      <c r="L57" s="130" t="n"/>
+      <c r="M57" s="130" t="n"/>
+      <c r="N57" s="131" t="n"/>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="130" t="n">
         <v>4</v>
       </c>
-      <c r="B53" s="130" t="inlineStr">
+      <c r="B58" s="130" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C53" s="131" t="inlineStr">
+      <c r="C58" s="131" t="inlineStr">
         <is>
           <t>Instructors dept + Program Ops</t>
         </is>
       </c>
-      <c r="D53" s="130" t="n"/>
-      <c r="E53" s="130" t="n"/>
-      <c r="F53" s="132" t="inlineStr">
+      <c r="D58" s="130" t="n"/>
+      <c r="E58" s="130" t="n"/>
+      <c r="F58" s="132" t="inlineStr">
         <is>
           <t>Classroom signal loop</t>
         </is>
       </c>
-      <c r="G53" s="131" t="inlineStr">
+      <c r="G58" s="131" t="inlineStr">
         <is>
           <t>Structured instructor feedback + conduction context per module — feeds content iteration and Content Issue routing.</t>
         </is>
       </c>
-      <c r="H53" s="131" t="n"/>
-      <c r="I53" s="130" t="n"/>
-      <c r="J53" s="130" t="n"/>
-      <c r="K53" s="130" t="n"/>
-      <c r="L53" s="130" t="n"/>
-      <c r="M53" s="130" t="n"/>
-      <c r="N53" s="131" t="n"/>
+      <c r="H58" s="131" t="n"/>
+      <c r="I58" s="130" t="n"/>
+      <c r="J58" s="130" t="n"/>
+      <c r="K58" s="130" t="n"/>
+      <c r="L58" s="130" t="n"/>
+      <c r="M58" s="130" t="n"/>
+      <c r="N58" s="131" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="G51:N51"/>
-    <mergeCell ref="G52:N52"/>
+    <mergeCell ref="G55:N55"/>
+    <mergeCell ref="G56:N56"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A54:N54"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="G50:N50"/>
-    <mergeCell ref="A49:N49"/>
-    <mergeCell ref="G53:N53"/>
+    <mergeCell ref="G57:N57"/>
+    <mergeCell ref="G58:N58"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8135,7 +8749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8646,7 +9260,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="84" customHeight="1">
       <c r="A12" s="123" t="n">
         <v>6</v>
       </c>
@@ -8672,17 +9286,17 @@
       </c>
       <c r="F12" s="125" t="inlineStr">
         <is>
-          <t>Check-ins Run</t>
+          <t>Worklog &amp; Status Hygiene — All Units</t>
         </is>
       </c>
       <c r="G12" s="124" t="inlineStr">
         <is>
-          <t>% of scheduled monthly unit check-ins with the HOD held on schedule, with the pre-read circulated a day before. Covers every sub-department and embedded function on the check-in calendar (~10 units).</t>
+          <t>Of the ~10 units on the check-in calendar, the % entering the monthly check-in with complete worklogs and current deliverable statuses (ClickUp). Check-ins Run says the meeting happened; this says it was fed — and complete worklogs are what make deliverable costing computable in every unit.</t>
         </is>
       </c>
       <c r="H12" s="124" t="inlineStr">
         <is>
-          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+          <t>hygiene — operating-rhythm guardrail (input side); no org ladder by design</t>
         </is>
       </c>
       <c r="I12" s="123" t="inlineStr">
@@ -8703,7 +9317,7 @@
       </c>
       <c r="N12" s="124" t="inlineStr">
         <is>
-          <t>Run by the PMO manager; unit PMs supply the pre-read inputs — orchestration here, the work stays with the units.</t>
+          <t>Unit PMs capture worklogs &amp; statuses in their own Team Ops &amp; People category; the PMO manager checks completeness at collection. Baseline first: needs the unit-PM layer live.</t>
         </is>
       </c>
     </row>
@@ -8733,12 +9347,12 @@
       </c>
       <c r="F13" s="125" t="inlineStr">
         <is>
-          <t>Actions Closed</t>
+          <t>Check-ins Run</t>
         </is>
       </c>
       <c r="G13" s="124" t="inlineStr">
         <is>
-          <t>% of actions logged in a monthly check-in that are closed before that unit's next check-in. The follow-through half of the cadence — check-ins that close loops, not meetings that merely happen.</t>
+          <t>% of scheduled monthly unit check-ins with the HOD held on schedule, with the pre-read circulated a day before. Covers every sub-department and embedded function on the check-in calendar (~10 units).</t>
         </is>
       </c>
       <c r="H13" s="124" t="inlineStr">
@@ -8764,67 +9378,94 @@
       </c>
       <c r="N13" s="124" t="inlineStr">
         <is>
+          <t>Run by the PMO manager; unit PMs supply the pre-read inputs — orchestration here, the work stays with the units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="123" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C14" s="124" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="D14" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E14" s="123" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F14" s="125" t="inlineStr">
+        <is>
+          <t>Actions Closed</t>
+        </is>
+      </c>
+      <c r="G14" s="124" t="inlineStr">
+        <is>
+          <t>% of actions logged in a monthly check-in that are closed before that unit's next check-in. The follow-through half of the cadence — check-ins that close loops, not meetings that merely happen.</t>
+        </is>
+      </c>
+      <c r="H14" s="124" t="inlineStr">
+        <is>
+          <t>hygiene — operating-rhythm guardrail; no org ladder by design</t>
+        </is>
+      </c>
+      <c r="I14" s="123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J14" s="123" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K14" s="123" t="n"/>
+      <c r="L14" s="123" t="n"/>
+      <c r="M14" s="126">
+        <f>IF(AND(ISNUMBER(K14),ISNUMBER(L14)),K14-L14,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="124" t="inlineStr">
+        <is>
           <t>Run by the PMO manager. Deferred companions (spend → outcome map · tracker freshness · finance turnaround) join after the start set runs a cycle or two.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="139" t="inlineStr">
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="139" t="inlineStr">
         <is>
           <t>C — Asks: what this team needs from counterparties (thin interface contracts — reviewed monthly)</t>
         </is>
       </c>
-      <c r="B14" s="119" t="n"/>
-      <c r="C14" s="119" t="n"/>
-      <c r="D14" s="119" t="n"/>
-      <c r="E14" s="119" t="n"/>
-      <c r="F14" s="119" t="n"/>
-      <c r="G14" s="119" t="n"/>
-      <c r="H14" s="119" t="n"/>
-      <c r="I14" s="119" t="n"/>
-      <c r="J14" s="119" t="n"/>
-      <c r="K14" s="119" t="n"/>
-      <c r="L14" s="119" t="n"/>
-      <c r="M14" s="119" t="n"/>
-      <c r="N14" s="119" t="n"/>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="140" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="140" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C15" s="141" t="inlineStr">
-        <is>
-          <t>Product, Engineering, Product Design &amp; Pedagogy function heads</t>
-        </is>
-      </c>
-      <c r="D15" s="140" t="n"/>
-      <c r="E15" s="140" t="n"/>
-      <c r="F15" s="142" t="inlineStr">
-        <is>
-          <t>Execution-management KPI tracking</t>
-        </is>
-      </c>
-      <c r="G15" s="141" t="inlineStr">
-        <is>
-          <t>Own execution KPIs (roadmap predictability, on-time delivery, budget adherence…) for teams embedded with us, tracked in their home functions — Central consumes the read at the monthly check-in; feeds Shared-Team Deliverables Landed (§7 ask).</t>
-        </is>
-      </c>
-      <c r="H15" s="141" t="n"/>
-      <c r="I15" s="140" t="n"/>
-      <c r="J15" s="140" t="n"/>
-      <c r="K15" s="140" t="n"/>
-      <c r="L15" s="140" t="n"/>
-      <c r="M15" s="140" t="n"/>
-      <c r="N15" s="141" t="n"/>
+      <c r="B15" s="119" t="n"/>
+      <c r="C15" s="119" t="n"/>
+      <c r="D15" s="119" t="n"/>
+      <c r="E15" s="119" t="n"/>
+      <c r="F15" s="119" t="n"/>
+      <c r="G15" s="119" t="n"/>
+      <c r="H15" s="119" t="n"/>
+      <c r="I15" s="119" t="n"/>
+      <c r="J15" s="119" t="n"/>
+      <c r="K15" s="119" t="n"/>
+      <c r="L15" s="119" t="n"/>
+      <c r="M15" s="119" t="n"/>
+      <c r="N15" s="119" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="140" t="inlineStr">
         <is>
@@ -8833,19 +9474,19 @@
       </c>
       <c r="C16" s="141" t="inlineStr">
         <is>
-          <t>Graphic Design &amp; Video Editing team heads</t>
+          <t>Product, Engineering, Product Design &amp; Pedagogy function heads</t>
         </is>
       </c>
       <c r="D16" s="140" t="n"/>
       <c r="E16" s="140" t="n"/>
       <c r="F16" s="142" t="inlineStr">
         <is>
-          <t>Creative delivery-management tracking</t>
+          <t>Execution-management KPI tracking</t>
         </is>
       </c>
       <c r="G16" s="141" t="inlineStr">
         <is>
-          <t>Delivery-management KPIs for the design &amp; video pipeline (on-time %, asset turnaround TAT, rework rate…) stay with the creative team heads; domain PMs manage day-to-day utilisation (FS view carries Creative Resource Utilisation) — §7 ask, reviewed quarterly.</t>
+          <t>Own execution KPIs (roadmap predictability, on-time delivery, budget adherence…) for teams embedded with us, tracked in their home functions — Central consumes the read at the monthly check-in; feeds Shared-Team Deliverables Landed (§7 ask).</t>
         </is>
       </c>
       <c r="H16" s="141" t="n"/>
@@ -8856,14 +9497,48 @@
       <c r="M16" s="140" t="n"/>
       <c r="N16" s="141" t="n"/>
     </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="140" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="140" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C17" s="141" t="inlineStr">
+        <is>
+          <t>Graphic Design &amp; Video Editing team heads</t>
+        </is>
+      </c>
+      <c r="D17" s="140" t="n"/>
+      <c r="E17" s="140" t="n"/>
+      <c r="F17" s="142" t="inlineStr">
+        <is>
+          <t>Creative delivery-management tracking</t>
+        </is>
+      </c>
+      <c r="G17" s="141" t="inlineStr">
+        <is>
+          <t>Delivery-management KPIs for the design &amp; video pipeline (on-time %, asset turnaround TAT, rework rate…) stay with the creative team heads; domain PMs manage day-to-day utilisation (FS view carries Creative Resource Utilisation) — §7 ask, reviewed quarterly.</t>
+        </is>
+      </c>
+      <c r="H17" s="141" t="n"/>
+      <c r="I17" s="140" t="n"/>
+      <c r="J17" s="140" t="n"/>
+      <c r="K17" s="140" t="n"/>
+      <c r="L17" s="140" t="n"/>
+      <c r="M17" s="140" t="n"/>
+      <c r="N17" s="141" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="G17:N17"/>
     <mergeCell ref="A6:N6"/>
     <mergeCell ref="A4:N4"/>
-    <mergeCell ref="G15:N15"/>
     <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A15:N15"/>
     <mergeCell ref="G16:N16"/>
-    <mergeCell ref="A14:N14"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
PM role card (tab 6 + ladder section); Cost of Operations ops register; wiring audit fixes
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/kra_training_sheet.xlsx
+++ b/docs/handoff/artifacts/kra_training_sheet.xlsx
@@ -5060,7 +5060,7 @@
       </c>
       <c r="N16" s="124" t="inlineStr">
         <is>
-          <t>Replaces Operations &amp; Growth Cost (no baseline yet) — worklog capture builds the first read. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
+          <t>Full ops register (so nothing is forgotten): monthly manager–reportee one-on-ones · scheduling roadmap review meetings + Head approval · day-to-day ops (standups, learning hours) · scheduling monthly check-in meets &amp; documenting them in the right place · maintaining team assets (laptops, systems) · ensuring ClickUp adoption · keeping deliverable statuses up to date · monthly worklog capture → deliverable costs computed for the check-in · generating newsletters monthly · conducting team outings · conducting cycle-wise appraisal meetings. Replaces Operations &amp; Growth Cost (no baseline yet) — worklog capture builds the first read. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
         </is>
       </c>
     </row>
@@ -8200,7 +8200,7 @@
       </c>
       <c r="N47" s="124" t="inlineStr">
         <is>
-          <t>Replaces Operations &amp; Growth Cost — Jul A ₹300,863 spans ops + hiring; worklog capture splits it from next month. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
+          <t>Full ops register (so nothing is forgotten): monthly manager–reportee one-on-ones · scheduling roadmap review meetings + Head approval · day-to-day ops (standups, learning hours) · scheduling monthly check-in meets &amp; documenting them in the right place · maintaining team assets (laptops, systems) · ensuring ClickUp adoption · keeping deliverable statuses up to date · monthly worklog capture → deliverable costs computed for the check-in · generating newsletters monthly · conducting team outings · conducting cycle-wise appraisal meetings. Replaces Operations &amp; Growth Cost — Jul A ₹300,863 spans ops + hiring; worklog capture splits it from next month. Sub-metrics per activity (one-on-one coverage, status freshness…) get added as reads emerge. Run by the team's PM (reports to the Lead; KPI cascades Lead → PM).</t>
         </is>
       </c>
     </row>

</xml_diff>